<commit_message>
Update Egyptian Speech Therapy Centers with comprehensive Cairo district data
- Added comprehensive search results for all Cairo districts and neighborhoods
- Included 24 speech therapy centers across Cairo with contact information
- Maintained all 314 cities from original dataset with merged cells
- Updated file structure with proper Arabic formatting and RTL layout
</commit_message>
<xml_diff>
--- a/Egyptian_Speech_Therapy_Centers.xlsx
+++ b/Egyptian_Speech_Therapy_Centers.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G351"/>
+  <dimension ref="A1:G360"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1070,7 +1070,7 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
-      <c r="B37" s="5" t="n"/>
+      <c r="B37" s="6" t="n"/>
       <c r="C37" s="4" t="inlineStr">
         <is>
           <t>أكاديمية زويل</t>
@@ -1087,26 +1087,22 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n"/>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>جمعية إشراق الشمس</t>
-        </is>
-      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>برج العرب</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr"/>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr"/>
       <c r="F38" s="4" t="inlineStr"/>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>الإسكندرية</t>
-        </is>
-      </c>
+      <c r="G38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>برج العرب</t>
+          <t>مونتازا</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr"/>
@@ -1119,25 +1115,29 @@
       <c r="A40" s="5" t="n"/>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>مونتازا</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr"/>
+          <t>سيدي بشر</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>مركز كلام عيال للتخاطب وتنمية مهارات</t>
+        </is>
+      </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr"/>
-      <c r="G40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>144 شارع جمال عبد الناصر سيدي بشر</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>سيدي بشر</t>
-        </is>
-      </c>
+      <c r="B41" s="5" t="n"/>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>مركز كلام عيال للتخاطب وتنمية مهارات</t>
+          <t>عيادة تخاطب شارع الطفولة السعيدة</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr"/>
@@ -1145,16 +1145,16 @@
       <c r="F41" s="4" t="inlineStr"/>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>144 شارع جمال عبد الناصر سيدي بشر</t>
+          <t>شارع الطفولة السعيدة، سيدي بشر</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
-      <c r="B42" s="5" t="n"/>
+      <c r="B42" s="6" t="n"/>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>عيادة تخاطب شارع الطفولة السعيدة</t>
+          <t>مركز تومورو للتخاطب</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
@@ -1162,32 +1162,28 @@
       <c r="F42" s="4" t="inlineStr"/>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>شارع الطفولة السعيدة، سيدي بشر</t>
+          <t>البيطاش وسيدي بشر والجيزة</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>مركز تومورو للتخاطب</t>
-        </is>
-      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>أبي قير</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr"/>
       <c r="D43" s="4" t="inlineStr"/>
       <c r="E43" s="4" t="inlineStr"/>
       <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>البيطاش وسيدي بشر والجيزة</t>
-        </is>
-      </c>
+      <c r="G43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n"/>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>أبي قير</t>
+          <t>الدخيلة</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr"/>
@@ -1200,7 +1196,7 @@
       <c r="A45" s="5" t="n"/>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>الدخيلة</t>
+          <t>كوم الدكة</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr"/>
@@ -1213,7 +1209,7 @@
       <c r="A46" s="5" t="n"/>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>كوم الدكة</t>
+          <t>ستانلي</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr"/>
@@ -1226,7 +1222,7 @@
       <c r="A47" s="5" t="n"/>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>ستانلي</t>
+          <t>الشاطبي</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr"/>
@@ -1239,7 +1235,7 @@
       <c r="A48" s="5" t="n"/>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>الشاطبي</t>
+          <t>رشدي</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr"/>
@@ -1252,7 +1248,7 @@
       <c r="A49" s="5" t="n"/>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>رشدي</t>
+          <t>الرملة</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr"/>
@@ -1265,7 +1261,7 @@
       <c r="A50" s="5" t="n"/>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>الرملة</t>
+          <t>الإبراهيمية</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr"/>
@@ -1278,7 +1274,7 @@
       <c r="A51" s="5" t="n"/>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>الإبراهيمية</t>
+          <t>القنطرة</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr"/>
@@ -1291,7 +1287,7 @@
       <c r="A52" s="5" t="n"/>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>القنطرة</t>
+          <t>كفر عبده</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr"/>
@@ -1304,7 +1300,7 @@
       <c r="A53" s="5" t="n"/>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>كفر عبده</t>
+          <t>الحمام</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr"/>
@@ -1317,7 +1313,7 @@
       <c r="A54" s="5" t="n"/>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>الحمام</t>
+          <t>مارينا</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr"/>
@@ -1330,7 +1326,7 @@
       <c r="A55" s="5" t="n"/>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>مارينا</t>
+          <t>عمومية</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr"/>
@@ -1340,10 +1336,10 @@
       <c r="G55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="n"/>
+      <c r="A56" s="6" t="n"/>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>عمومية</t>
+          <t>ضواحي</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr"/>
@@ -1353,10 +1349,14 @@
       <c r="G56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="n"/>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>الإسماعيلية</t>
+        </is>
+      </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>ضواحي</t>
+          <t>الإسماعيلية</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr"/>
@@ -1366,14 +1366,10 @@
       <c r="G57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>الإسماعيلية</t>
-        </is>
-      </c>
+      <c r="A58" s="5" t="n"/>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>الإسماعيلية</t>
+          <t>بورسعيد</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr"/>
@@ -1386,7 +1382,7 @@
       <c r="A59" s="5" t="n"/>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>بورسعيد</t>
+          <t>السويس</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr"/>
@@ -1399,7 +1395,7 @@
       <c r="A60" s="5" t="n"/>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>السويس</t>
+          <t>القنطرة غرب</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr"/>
@@ -1412,7 +1408,7 @@
       <c r="A61" s="5" t="n"/>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>القنطرة غرب</t>
+          <t>القنطرة شرق</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr"/>
@@ -1425,7 +1421,7 @@
       <c r="A62" s="5" t="n"/>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>القنطرة شرق</t>
+          <t>فايد</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr"/>
@@ -1438,7 +1434,7 @@
       <c r="A63" s="5" t="n"/>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>فايد</t>
+          <t>تل الكبير</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr"/>
@@ -1451,7 +1447,7 @@
       <c r="A64" s="5" t="n"/>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>تل الكبير</t>
+          <t>الشلوفة</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr"/>
@@ -1461,10 +1457,10 @@
       <c r="G64" s="4" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="n"/>
+      <c r="A65" s="6" t="n"/>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>الشلوفة</t>
+          <t>الدفرسوار</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr"/>
@@ -1474,32 +1470,36 @@
       <c r="G65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="n"/>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>البحر الأحمر</t>
+        </is>
+      </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>الدفرسوار</t>
-        </is>
-      </c>
-      <c r="C66" s="4" t="inlineStr"/>
+          <t>الغردقة</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب الغردقة بمركز شباب الغردقة</t>
+        </is>
+      </c>
       <c r="D66" s="4" t="inlineStr"/>
       <c r="E66" s="4" t="inlineStr"/>
       <c r="F66" s="4" t="inlineStr"/>
-      <c r="G66" s="4" t="inlineStr"/>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب الغردقة</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>البحر الأحمر</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>الغردقة</t>
-        </is>
-      </c>
+      <c r="A67" s="5" t="n"/>
+      <c r="B67" s="6" t="n"/>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>مركز تخاطب الغردقة بمركز شباب الغردقة</t>
+          <t>مركز تخاطب سفاجة</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr"/>
@@ -1507,32 +1507,28 @@
       <c r="F67" s="4" t="inlineStr"/>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>مركز شباب الغردقة</t>
+          <t>سفاجة</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n"/>
-      <c r="B68" s="6" t="n"/>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب سفاجة</t>
-        </is>
-      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>سفاجة</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr"/>
       <c r="D68" s="4" t="inlineStr"/>
       <c r="E68" s="4" t="inlineStr"/>
       <c r="F68" s="4" t="inlineStr"/>
-      <c r="G68" s="4" t="inlineStr">
-        <is>
-          <t>سفاجة</t>
-        </is>
-      </c>
+      <c r="G68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n"/>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>سفاجة</t>
+          <t>القصير</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr"/>
@@ -1545,7 +1541,7 @@
       <c r="A70" s="5" t="n"/>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>القصير</t>
+          <t>مرسى علم</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr"/>
@@ -1558,7 +1554,7 @@
       <c r="A71" s="5" t="n"/>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>مرسى علم</t>
+          <t>شلاتين</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr"/>
@@ -1571,7 +1567,7 @@
       <c r="A72" s="5" t="n"/>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>شلاتين</t>
+          <t>حلايب</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr"/>
@@ -1584,7 +1580,7 @@
       <c r="A73" s="5" t="n"/>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>حلايب</t>
+          <t>أبو رماد</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr"/>
@@ -1597,7 +1593,7 @@
       <c r="A74" s="5" t="n"/>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>أبو رماد</t>
+          <t>قصير الجديدة</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr"/>
@@ -1610,7 +1606,7 @@
       <c r="A75" s="5" t="n"/>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>قصير الجديدة</t>
+          <t>رأس غارب</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr"/>
@@ -1620,10 +1616,10 @@
       <c r="G75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="5" t="n"/>
+      <c r="A76" s="6" t="n"/>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>رأس غارب</t>
+          <t>دهب</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr"/>
@@ -1633,82 +1629,82 @@
       <c r="G76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="n"/>
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>البحيرة</t>
+        </is>
+      </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>دهب</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr"/>
+          <t>دمنهور</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>مركز لايف للتخاطب</t>
+        </is>
+      </c>
       <c r="D77" s="4" t="inlineStr"/>
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr"/>
-      <c r="G77" s="4" t="inlineStr"/>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>21 شارع إبراهيم مظهر، ميدان الساعة</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>البحيرة</t>
-        </is>
-      </c>
+      <c r="A78" s="5" t="n"/>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>دمنهور</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>مركز لايف للتخاطب</t>
-        </is>
-      </c>
+          <t>كفر الدوار</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr"/>
       <c r="D78" s="4" t="inlineStr"/>
       <c r="E78" s="4" t="inlineStr"/>
       <c r="F78" s="4" t="inlineStr"/>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>21 شارع إبراهيم مظهر، ميدان الساعة</t>
-        </is>
-      </c>
+      <c r="G78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n"/>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>كفر الدوار</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr"/>
+          <t>رشيد</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>مركز الإيمان للتخاطب</t>
+        </is>
+      </c>
       <c r="D79" s="4" t="inlineStr"/>
       <c r="E79" s="4" t="inlineStr"/>
       <c r="F79" s="4" t="inlineStr"/>
-      <c r="G79" s="4" t="inlineStr"/>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>شارع عبد السلام عارف</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n"/>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>رشيد</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>مركز الإيمان للتخاطب</t>
-        </is>
-      </c>
+          <t>إدكو</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr"/>
       <c r="D80" s="4" t="inlineStr"/>
       <c r="E80" s="4" t="inlineStr"/>
       <c r="F80" s="4" t="inlineStr"/>
-      <c r="G80" s="4" t="inlineStr">
-        <is>
-          <t>شارع عبد السلام عارف</t>
-        </is>
-      </c>
+      <c r="G80" s="4" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n"/>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>إدكو</t>
+          <t>أبو حمص</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr"/>
@@ -1721,7 +1717,7 @@
       <c r="A82" s="5" t="n"/>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>أبو حمص</t>
+          <t>كوم حمادة</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr"/>
@@ -1734,7 +1730,7 @@
       <c r="A83" s="5" t="n"/>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>كوم حمادة</t>
+          <t>شبراخيت</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr"/>
@@ -1747,7 +1743,7 @@
       <c r="A84" s="5" t="n"/>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>شبراخيت</t>
+          <t>كفر الشيخ</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr"/>
@@ -1760,7 +1756,7 @@
       <c r="A85" s="5" t="n"/>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>كفر الشيخ</t>
+          <t>نوقة</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr"/>
@@ -1773,7 +1769,7 @@
       <c r="A86" s="5" t="n"/>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>نوقة</t>
+          <t>الحامول</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr"/>
@@ -1786,7 +1782,7 @@
       <c r="A87" s="5" t="n"/>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>الحامول</t>
+          <t>شرقية</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr"/>
@@ -1799,7 +1795,7 @@
       <c r="A88" s="5" t="n"/>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>شرقية</t>
+          <t>الدلنجات</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr"/>
@@ -1812,7 +1808,7 @@
       <c r="A89" s="5" t="n"/>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>الدلنجات</t>
+          <t>إيتاي البارود</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr"/>
@@ -1825,7 +1821,7 @@
       <c r="A90" s="5" t="n"/>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>إيتاي البارود</t>
+          <t>بسيون</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr"/>
@@ -1835,10 +1831,10 @@
       <c r="G90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="n"/>
+      <c r="A91" s="6" t="n"/>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>بسيون</t>
+          <t>سنجور</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr"/>
@@ -1848,32 +1844,36 @@
       <c r="G91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="6" t="n"/>
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>سنجور</t>
-        </is>
-      </c>
-      <c r="C92" s="4" t="inlineStr"/>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>مركز التخاطب النموذجي</t>
+        </is>
+      </c>
       <c r="D92" s="4" t="inlineStr"/>
       <c r="E92" s="4" t="inlineStr"/>
       <c r="F92" s="4" t="inlineStr"/>
-      <c r="G92" s="4" t="inlineStr"/>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>شارع النيل، العجوزة</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>الجيزة</t>
-        </is>
-      </c>
-      <c r="B93" s="3" t="inlineStr">
-        <is>
-          <t>الجيزة</t>
-        </is>
-      </c>
+      <c r="A93" s="5" t="n"/>
+      <c r="B93" s="5" t="n"/>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>مركز التخاطب النموذجي</t>
+          <t>مركز تخاطب وسمع واتزان</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr"/>
@@ -1881,7 +1881,7 @@
       <c r="F93" s="4" t="inlineStr"/>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>شارع النيل، العجوزة</t>
+          <t>شارع نادي إمبابة الرياضي، إمبابة</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       <c r="B94" s="5" t="n"/>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>مركز تخاطب وسمع واتزان</t>
+          <t>مركز قدرات للتخاطب</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr"/>
@@ -1898,7 +1898,7 @@
       <c r="F94" s="4" t="inlineStr"/>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>شارع نادي إمبابة الرياضي، إمبابة</t>
+          <t>119 شارع الهرم، الهرم</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1907,7 @@
       <c r="B95" s="5" t="n"/>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>مركز قدرات للتخاطب</t>
+          <t>مركز مكة للتخاطب وتنمية مهارات</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr"/>
@@ -1915,16 +1915,16 @@
       <c r="F95" s="4" t="inlineStr"/>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>119 شارع الهرم، الهرم</t>
+          <t>الهرم، الجيزة</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n"/>
-      <c r="B96" s="5" t="n"/>
+      <c r="B96" s="6" t="n"/>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>مركز مكة للتخاطب وتنمية مهارات</t>
+          <t>مركز القادة للتخاطب وتنمية المهارات</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr"/>
@@ -1938,26 +1938,22 @@
     </row>
     <row r="97">
       <c r="A97" s="5" t="n"/>
-      <c r="B97" s="6" t="n"/>
-      <c r="C97" s="4" t="inlineStr">
-        <is>
-          <t>مركز القادة للتخاطب وتنمية المهارات</t>
-        </is>
-      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>مدينة 6 أكتوبر</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr"/>
       <c r="D97" s="4" t="inlineStr"/>
       <c r="E97" s="4" t="inlineStr"/>
       <c r="F97" s="4" t="inlineStr"/>
-      <c r="G97" s="4" t="inlineStr">
-        <is>
-          <t>الهرم، الجيزة</t>
-        </is>
-      </c>
+      <c r="G97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n"/>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>مدينة 6 أكتوبر</t>
+          <t>حلوان</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr"/>
@@ -1970,7 +1966,7 @@
       <c r="A99" s="5" t="n"/>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>حلوان</t>
+          <t>البدرشين</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr"/>
@@ -1983,7 +1979,7 @@
       <c r="A100" s="5" t="n"/>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>البدرشين</t>
+          <t>دهشور</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr"/>
@@ -1996,7 +1992,7 @@
       <c r="A101" s="5" t="n"/>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>دهشور</t>
+          <t>أبو رواش</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr"/>
@@ -2009,7 +2005,7 @@
       <c r="A102" s="5" t="n"/>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>أبو رواش</t>
+          <t>الوراق</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr"/>
@@ -2022,7 +2018,7 @@
       <c r="A103" s="5" t="n"/>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>الوراق</t>
+          <t>الساحل</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr"/>
@@ -2035,7 +2031,7 @@
       <c r="A104" s="5" t="n"/>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>الساحل</t>
+          <t>الكيت كات</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr"/>
@@ -2048,25 +2044,29 @@
       <c r="A105" s="5" t="n"/>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>الكيت كات</t>
-        </is>
-      </c>
-      <c r="C105" s="4" t="inlineStr"/>
+          <t>الهرم</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>مركز هووب للتخاطب</t>
+        </is>
+      </c>
       <c r="D105" s="4" t="inlineStr"/>
       <c r="E105" s="4" t="inlineStr"/>
       <c r="F105" s="4" t="inlineStr"/>
-      <c r="G105" s="4" t="inlineStr"/>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>الهرم وفيصل</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="n"/>
-      <c r="B106" s="3" t="inlineStr">
-        <is>
-          <t>الهرم</t>
-        </is>
-      </c>
+      <c r="B106" s="5" t="n"/>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>مركز هووب للتخاطب</t>
+          <t>مركز طريقنا للتخاطب</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr"/>
@@ -2074,16 +2074,16 @@
       <c r="F106" s="4" t="inlineStr"/>
       <c r="G106" s="4" t="inlineStr">
         <is>
-          <t>الهرم وفيصل</t>
+          <t>10 شارع أحمد عبد المحسن، التعاون</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n"/>
-      <c r="B107" s="5" t="n"/>
+      <c r="B107" s="6" t="n"/>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>مركز طريقنا للتخاطب</t>
+          <t>مركز الأهرام للتخاطب</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr"/>
@@ -2091,16 +2091,20 @@
       <c r="F107" s="4" t="inlineStr"/>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>10 شارع أحمد عبد المحسن، التعاون</t>
+          <t>شارع اللبيني، المريوطية</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="n"/>
-      <c r="B108" s="6" t="n"/>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>إمبابة</t>
+        </is>
+      </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>مركز الأهرام للتخاطب</t>
+          <t>معهد السمع والكلام بإمبابة</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr"/>
@@ -2108,22 +2112,26 @@
       <c r="F108" s="4" t="inlineStr"/>
       <c r="G108" s="4" t="inlineStr">
         <is>
-          <t>شارع اللبيني، المريوطية</t>
+          <t>1 شارع الطيار فكري، بجوار مستشفى الحميات</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="n"/>
-      <c r="B109" s="3" t="inlineStr">
-        <is>
-          <t>إمبابة</t>
-        </is>
-      </c>
-      <c r="C109" s="4" t="inlineStr"/>
+      <c r="B109" s="6" t="n"/>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب شارع عزبة الصعايدة</t>
+        </is>
+      </c>
       <c r="D109" s="4" t="inlineStr"/>
       <c r="E109" s="4" t="inlineStr"/>
       <c r="F109" s="4" t="inlineStr"/>
-      <c r="G109" s="4" t="inlineStr"/>
+      <c r="G109" s="4" t="inlineStr">
+        <is>
+          <t>عزبة الصعايدة أعلى مسجد أولاد عمرو، متفرع من شارع ترعة السواحل</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n"/>
@@ -3186,7 +3194,11 @@
           <t>د. وفاء وافي</t>
         </is>
       </c>
-      <c r="E178" s="4" t="inlineStr"/>
+      <c r="E178" s="4" t="inlineStr">
+        <is>
+          <t>0222406301</t>
+        </is>
+      </c>
       <c r="F178" s="4" t="inlineStr"/>
       <c r="G178" s="4" t="inlineStr">
         <is>
@@ -3216,15 +3228,19 @@
       <c r="B180" s="5" t="n"/>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>مركز هليوبوليس للتخاطب وتنمية المهارات</t>
-        </is>
-      </c>
-      <c r="D180" s="4" t="inlineStr"/>
+          <t>مركز تخاطب أخصائية التخاطب هبة المصري</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>د. هبة المصري</t>
+        </is>
+      </c>
       <c r="E180" s="4" t="inlineStr"/>
       <c r="F180" s="4" t="inlineStr"/>
       <c r="G180" s="4" t="inlineStr">
         <is>
-          <t>28 شارع محمد عبيد من شارع النزهة، مصر الجديدة</t>
+          <t>ترعة القبة، مساكن الأميرية الجنوبية، حدائق القبة</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3249,7 @@
       <c r="B181" s="5" t="n"/>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>مركز Speak للتخاطب</t>
+          <t>مركز نور الحياة للتخاطب</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr"/>
@@ -3241,16 +3257,16 @@
       <c r="F181" s="4" t="inlineStr"/>
       <c r="G181" s="4" t="inlineStr">
         <is>
-          <t>زهراء مدينة نصر - المرحلة الأولى</t>
+          <t>شارع شبرا الخلفاوي، قسم الساحل</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="5" t="n"/>
-      <c r="B182" s="6" t="n"/>
+      <c r="B182" s="5" t="n"/>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>مركز Almony للتخاطب وصعوبات التعلم</t>
+          <t>مركز الرضا للتخاطب وتنمية المهارات</t>
         </is>
       </c>
       <c r="D182" s="4" t="inlineStr"/>
@@ -3258,20 +3274,16 @@
       <c r="F182" s="4" t="inlineStr"/>
       <c r="G182" s="4" t="inlineStr">
         <is>
-          <t>8 عمارات منتصر، بجانب مسجد عبد الرحمن، حدائق حلوان</t>
+          <t>شارع ترعة جزيرة بدران، قسم روض الفرج</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="5" t="n"/>
-      <c r="B183" s="3" t="inlineStr">
-        <is>
-          <t>مدينة نصر</t>
-        </is>
-      </c>
+      <c r="B183" s="5" t="n"/>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>المركز الذهبي التخصصي (GSC)</t>
+          <t>معهد السمع والكلام بإمبابة</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr"/>
@@ -3279,32 +3291,24 @@
       <c r="F183" s="4" t="inlineStr"/>
       <c r="G183" s="4" t="inlineStr">
         <is>
-          <t>مدينة نصر، القاهرة</t>
+          <t>1 شارع الطيار فكري، بجوار مستشفى الحميات، إمبابة</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="5" t="n"/>
-      <c r="B184" s="3" t="inlineStr">
-        <is>
-          <t>مصر الجديدة</t>
-        </is>
-      </c>
+      <c r="B184" s="6" t="n"/>
       <c r="C184" s="4" t="inlineStr">
         <is>
-          <t>مركز التخاطب الشامل و صعوبات التعلم</t>
-        </is>
-      </c>
-      <c r="D184" s="4" t="inlineStr">
-        <is>
-          <t>د. وفاء وافي</t>
-        </is>
-      </c>
+          <t>مركز Speak للتخاطب</t>
+        </is>
+      </c>
+      <c r="D184" s="4" t="inlineStr"/>
       <c r="E184" s="4" t="inlineStr"/>
       <c r="F184" s="4" t="inlineStr"/>
       <c r="G184" s="4" t="inlineStr">
         <is>
-          <t>مصر الجديدة</t>
+          <t>زهراء مدينة نصر - المرحلة الأولى</t>
         </is>
       </c>
     </row>
@@ -3312,85 +3316,117 @@
       <c r="A185" s="5" t="n"/>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>الزمالك</t>
-        </is>
-      </c>
-      <c r="C185" s="4" t="inlineStr"/>
+          <t>مدينة نصر</t>
+        </is>
+      </c>
+      <c r="C185" s="4" t="inlineStr">
+        <is>
+          <t>المركز الذهبي التخصصي (GSC)</t>
+        </is>
+      </c>
       <c r="D185" s="4" t="inlineStr"/>
       <c r="E185" s="4" t="inlineStr"/>
       <c r="F185" s="4" t="inlineStr"/>
-      <c r="G185" s="4" t="inlineStr"/>
+      <c r="G185" s="4" t="inlineStr">
+        <is>
+          <t>مدينة نصر، القاهرة</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="5" t="n"/>
-      <c r="B186" s="3" t="inlineStr">
-        <is>
-          <t>الجيزة</t>
-        </is>
-      </c>
-      <c r="C186" s="4" t="inlineStr"/>
+      <c r="B186" s="5" t="n"/>
+      <c r="C186" s="4" t="inlineStr">
+        <is>
+          <t>مركز الزهراء للتخاطب</t>
+        </is>
+      </c>
       <c r="D186" s="4" t="inlineStr"/>
       <c r="E186" s="4" t="inlineStr"/>
       <c r="F186" s="4" t="inlineStr"/>
-      <c r="G186" s="4" t="inlineStr"/>
+      <c r="G186" s="4" t="inlineStr">
+        <is>
+          <t>5 شارع الصواف، المنطقة العاشرة، مدينة نصر</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="5" t="n"/>
-      <c r="B187" s="3" t="inlineStr">
-        <is>
-          <t>العبّاسية</t>
-        </is>
-      </c>
-      <c r="C187" s="4" t="inlineStr"/>
+      <c r="B187" s="5" t="n"/>
+      <c r="C187" s="4" t="inlineStr">
+        <is>
+          <t>مركز الحمد للعلاج الطبيعي والتخاطب</t>
+        </is>
+      </c>
       <c r="D187" s="4" t="inlineStr"/>
       <c r="E187" s="4" t="inlineStr"/>
       <c r="F187" s="4" t="inlineStr"/>
-      <c r="G187" s="4" t="inlineStr"/>
+      <c r="G187" s="4" t="inlineStr">
+        <is>
+          <t>شارع مصطفى النحاس فوق التوحيد والنور بعد مدرسة المنهل</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="5" t="n"/>
-      <c r="B188" s="3" t="inlineStr">
-        <is>
-          <t>مدينة 6 أكتوبر</t>
-        </is>
-      </c>
-      <c r="C188" s="4" t="inlineStr"/>
+      <c r="B188" s="6" t="n"/>
+      <c r="C188" s="4" t="inlineStr">
+        <is>
+          <t>مركز الشمس للتخاطب</t>
+        </is>
+      </c>
       <c r="D188" s="4" t="inlineStr"/>
       <c r="E188" s="4" t="inlineStr"/>
       <c r="F188" s="4" t="inlineStr"/>
-      <c r="G188" s="4" t="inlineStr"/>
+      <c r="G188" s="4" t="inlineStr">
+        <is>
+          <t>مدينة نصر</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="5" t="n"/>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>مدينة الشروق</t>
-        </is>
-      </c>
-      <c r="C189" s="4" t="inlineStr"/>
-      <c r="D189" s="4" t="inlineStr"/>
+          <t>مصر الجديدة</t>
+        </is>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>مركز التخاطب الشامل و صعوبات التعلم</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>د. وفاء وافي</t>
+        </is>
+      </c>
       <c r="E189" s="4" t="inlineStr"/>
       <c r="F189" s="4" t="inlineStr"/>
-      <c r="G189" s="4" t="inlineStr"/>
+      <c r="G189" s="4" t="inlineStr">
+        <is>
+          <t>1 شارع المنتزه خلف مستشفى هليوبوليس</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n"/>
-      <c r="B190" s="3" t="inlineStr">
-        <is>
-          <t>مدينة بدر</t>
-        </is>
-      </c>
+      <c r="B190" s="6" t="n"/>
       <c r="C190" s="4" t="inlineStr">
         <is>
-          <t>مركز متخصص للتخاطب</t>
+          <t>مركز هليوبوليس للتخاطب وتنمية المهارات</t>
         </is>
       </c>
       <c r="D190" s="4" t="inlineStr"/>
-      <c r="E190" s="4" t="inlineStr"/>
+      <c r="E190" s="4" t="inlineStr">
+        <is>
+          <t>01151194780</t>
+        </is>
+      </c>
       <c r="F190" s="4" t="inlineStr"/>
       <c r="G190" s="4" t="inlineStr">
         <is>
-          <t>مدينة بدر، القاهرة</t>
+          <t>28 شارع محمد عبيد من شارع النزهة، ميدان السبع عمارات</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3434,7 @@
       <c r="A191" s="5" t="n"/>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>مدينة 15 مايو</t>
+          <t>الزمالك</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr"/>
@@ -3411,49 +3447,33 @@
       <c r="A192" s="5" t="n"/>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>المعادي</t>
-        </is>
-      </c>
-      <c r="C192" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب بزهراء المعادي</t>
-        </is>
-      </c>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="C192" s="4" t="inlineStr"/>
       <c r="D192" s="4" t="inlineStr"/>
       <c r="E192" s="4" t="inlineStr"/>
       <c r="F192" s="4" t="inlineStr"/>
-      <c r="G192" s="4" t="inlineStr">
-        <is>
-          <t>شارع الأرقم بن الأرقم، الدائري، بستان</t>
-        </is>
-      </c>
+      <c r="G192" s="4" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n"/>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>حلوان</t>
-        </is>
-      </c>
-      <c r="C193" s="4" t="inlineStr">
-        <is>
-          <t>مركز Almony للتخاطب</t>
-        </is>
-      </c>
+          <t>العبّاسية</t>
+        </is>
+      </c>
+      <c r="C193" s="4" t="inlineStr"/>
       <c r="D193" s="4" t="inlineStr"/>
       <c r="E193" s="4" t="inlineStr"/>
       <c r="F193" s="4" t="inlineStr"/>
-      <c r="G193" s="4" t="inlineStr">
-        <is>
-          <t>حدائق حلوان</t>
-        </is>
-      </c>
+      <c r="G193" s="4" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="5" t="n"/>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>المقطم</t>
+          <t>مدينة 6 أكتوبر</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr"/>
@@ -3466,7 +3486,7 @@
       <c r="A195" s="5" t="n"/>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>القاهرة الجديدة</t>
+          <t>مدينة الشروق</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr"/>
@@ -3479,20 +3499,28 @@
       <c r="A196" s="5" t="n"/>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>الشيخ زايد</t>
-        </is>
-      </c>
-      <c r="C196" s="4" t="inlineStr"/>
+          <t>مدينة بدر</t>
+        </is>
+      </c>
+      <c r="C196" s="4" t="inlineStr">
+        <is>
+          <t>مركز متخصص للتخاطب</t>
+        </is>
+      </c>
       <c r="D196" s="4" t="inlineStr"/>
       <c r="E196" s="4" t="inlineStr"/>
       <c r="F196" s="4" t="inlineStr"/>
-      <c r="G196" s="4" t="inlineStr"/>
+      <c r="G196" s="4" t="inlineStr">
+        <is>
+          <t>مدينة بدر، القاهرة</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="5" t="n"/>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>الرحاب</t>
+          <t>مدينة 15 مايو</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr"/>
@@ -3505,59 +3533,83 @@
       <c r="A198" s="5" t="n"/>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>الحي العاشر</t>
-        </is>
-      </c>
-      <c r="C198" s="4" t="inlineStr"/>
+          <t>المعادي</t>
+        </is>
+      </c>
+      <c r="C198" s="4" t="inlineStr">
+        <is>
+          <t>المركز المصري الكندي</t>
+        </is>
+      </c>
       <c r="D198" s="4" t="inlineStr"/>
       <c r="E198" s="4" t="inlineStr"/>
       <c r="F198" s="4" t="inlineStr"/>
-      <c r="G198" s="4" t="inlineStr"/>
+      <c r="G198" s="4" t="inlineStr">
+        <is>
+          <t>5/3 شارع اللاسلكي بجوار شركة غاز مصر</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="5" t="n"/>
-      <c r="B199" s="3" t="inlineStr">
-        <is>
-          <t>المنيل</t>
-        </is>
-      </c>
-      <c r="C199" s="4" t="inlineStr"/>
+      <c r="B199" s="5" t="n"/>
+      <c r="C199" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب البر والتقوى</t>
+        </is>
+      </c>
       <c r="D199" s="4" t="inlineStr"/>
       <c r="E199" s="4" t="inlineStr"/>
       <c r="F199" s="4" t="inlineStr"/>
-      <c r="G199" s="4" t="inlineStr"/>
+      <c r="G199" s="4" t="inlineStr">
+        <is>
+          <t>104 برج الأوقاف، شارع ابن سندر</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="5" t="n"/>
-      <c r="B200" s="3" t="inlineStr">
-        <is>
-          <t>الدقي</t>
-        </is>
-      </c>
-      <c r="C200" s="4" t="inlineStr"/>
+      <c r="B200" s="6" t="n"/>
+      <c r="C200" s="4" t="inlineStr">
+        <is>
+          <t>مركز كيور لجراحات الأذن والقوقعة والتخاطب</t>
+        </is>
+      </c>
       <c r="D200" s="4" t="inlineStr"/>
       <c r="E200" s="4" t="inlineStr"/>
       <c r="F200" s="4" t="inlineStr"/>
-      <c r="G200" s="4" t="inlineStr"/>
+      <c r="G200" s="4" t="inlineStr">
+        <is>
+          <t>شارع النصر، تقاطع اللاسلكي</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="5" t="n"/>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>الجيزة</t>
-        </is>
-      </c>
-      <c r="C201" s="4" t="inlineStr"/>
+          <t>حلوان</t>
+        </is>
+      </c>
+      <c r="C201" s="4" t="inlineStr">
+        <is>
+          <t>مركز Almony للتخاطب وصعوبات التعلم</t>
+        </is>
+      </c>
       <c r="D201" s="4" t="inlineStr"/>
       <c r="E201" s="4" t="inlineStr"/>
       <c r="F201" s="4" t="inlineStr"/>
-      <c r="G201" s="4" t="inlineStr"/>
+      <c r="G201" s="4" t="inlineStr">
+        <is>
+          <t>8 عمارات منتصر، بجانب مسجد عبد الرحمن، حدائق حلوان</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="5" t="n"/>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>الموسكي</t>
+          <t>المقطم</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr"/>
@@ -3570,7 +3622,7 @@
       <c r="A203" s="5" t="n"/>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>الفجالة</t>
+          <t>القاهرة الجديدة</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr"/>
@@ -3583,7 +3635,7 @@
       <c r="A204" s="5" t="n"/>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>باب الشعرية</t>
+          <t>الشيخ زايد</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr"/>
@@ -3596,7 +3648,7 @@
       <c r="A205" s="5" t="n"/>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>الساحل</t>
+          <t>الرحاب</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr"/>
@@ -3609,7 +3661,7 @@
       <c r="A206" s="5" t="n"/>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>المطرية</t>
+          <t>الحي العاشر</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr"/>
@@ -3622,7 +3674,7 @@
       <c r="A207" s="5" t="n"/>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>عين شمس</t>
+          <t>المنيل</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr"/>
@@ -3635,33 +3687,45 @@
       <c r="A208" s="5" t="n"/>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>الزيتون</t>
-        </is>
-      </c>
-      <c r="C208" s="4" t="inlineStr"/>
+          <t>الدقي</t>
+        </is>
+      </c>
+      <c r="C208" s="4" t="inlineStr">
+        <is>
+          <t>فرع الدقي من مركز الحمد</t>
+        </is>
+      </c>
       <c r="D208" s="4" t="inlineStr"/>
       <c r="E208" s="4" t="inlineStr"/>
       <c r="F208" s="4" t="inlineStr"/>
-      <c r="G208" s="4" t="inlineStr"/>
+      <c r="G208" s="4" t="inlineStr">
+        <is>
+          <t>4 شارع حسين واصف، بجوار مدرسة العروبة</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="5" t="n"/>
-      <c r="B209" s="3" t="inlineStr">
-        <is>
-          <t>وسيط</t>
-        </is>
-      </c>
-      <c r="C209" s="4" t="inlineStr"/>
+      <c r="B209" s="6" t="n"/>
+      <c r="C209" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب شارع التحرير</t>
+        </is>
+      </c>
       <c r="D209" s="4" t="inlineStr"/>
       <c r="E209" s="4" t="inlineStr"/>
       <c r="F209" s="4" t="inlineStr"/>
-      <c r="G209" s="4" t="inlineStr"/>
+      <c r="G209" s="4" t="inlineStr">
+        <is>
+          <t>شارع التحرير، أمام محطة مترو الدقي</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="5" t="n"/>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>المنصورية</t>
+          <t>الجيزة</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr"/>
@@ -3674,7 +3738,7 @@
       <c r="A211" s="5" t="n"/>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>الدراسة</t>
+          <t>الموسكي</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr"/>
@@ -3687,7 +3751,7 @@
       <c r="A212" s="5" t="n"/>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>درب الجنينة</t>
+          <t>الفجالة</t>
         </is>
       </c>
       <c r="C212" s="4" t="inlineStr"/>
@@ -3700,7 +3764,7 @@
       <c r="A213" s="5" t="n"/>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>الشرابية</t>
+          <t>باب الشعرية</t>
         </is>
       </c>
       <c r="C213" s="4" t="inlineStr"/>
@@ -3713,7 +3777,7 @@
       <c r="A214" s="5" t="n"/>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>النزهة</t>
+          <t>الساحل</t>
         </is>
       </c>
       <c r="C214" s="4" t="inlineStr"/>
@@ -3726,46 +3790,74 @@
       <c r="A215" s="5" t="n"/>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>الرويسي</t>
-        </is>
-      </c>
-      <c r="C215" s="4" t="inlineStr"/>
+          <t>المطرية</t>
+        </is>
+      </c>
+      <c r="C215" s="4" t="inlineStr">
+        <is>
+          <t>مركز التخاطب الشامل بالمطرية</t>
+        </is>
+      </c>
       <c r="D215" s="4" t="inlineStr"/>
-      <c r="E215" s="4" t="inlineStr"/>
+      <c r="E215" s="4" t="inlineStr">
+        <is>
+          <t>01270756267, 01092975341</t>
+        </is>
+      </c>
       <c r="F215" s="4" t="inlineStr"/>
-      <c r="G215" s="4" t="inlineStr"/>
+      <c r="G215" s="4" t="inlineStr">
+        <is>
+          <t>شارع منية مطر المطرية، بجوار محطة مترو المطرية</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="5" t="n"/>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>قصر النيل</t>
-        </is>
-      </c>
-      <c r="C216" s="4" t="inlineStr"/>
+          <t>عين شمس</t>
+        </is>
+      </c>
+      <c r="C216" s="4" t="inlineStr">
+        <is>
+          <t>مركز الشمس للتخاطب</t>
+        </is>
+      </c>
       <c r="D216" s="4" t="inlineStr"/>
       <c r="E216" s="4" t="inlineStr"/>
       <c r="F216" s="4" t="inlineStr"/>
-      <c r="G216" s="4" t="inlineStr"/>
+      <c r="G216" s="4" t="inlineStr">
+        <is>
+          <t>عين شمس</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="5" t="n"/>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>الفسطاط</t>
-        </is>
-      </c>
-      <c r="C217" s="4" t="inlineStr"/>
+          <t>الزيتون</t>
+        </is>
+      </c>
+      <c r="C217" s="4" t="inlineStr">
+        <is>
+          <t>حورس للسمعيات والتخاطب</t>
+        </is>
+      </c>
       <c r="D217" s="4" t="inlineStr"/>
       <c r="E217" s="4" t="inlineStr"/>
       <c r="F217" s="4" t="inlineStr"/>
-      <c r="G217" s="4" t="inlineStr"/>
+      <c r="G217" s="4" t="inlineStr">
+        <is>
+          <t>1 ميدان المطرية، الزيتون</t>
+        </is>
+      </c>
     </row>
     <row r="218">
-      <c r="A218" s="6" t="n"/>
+      <c r="A218" s="5" t="n"/>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>الرحاب</t>
+          <t>وسيط</t>
         </is>
       </c>
       <c r="C218" s="4" t="inlineStr"/>
@@ -3775,69 +3867,49 @@
       <c r="G218" s="4" t="inlineStr"/>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="inlineStr">
-        <is>
-          <t>القليوبية</t>
-        </is>
-      </c>
+      <c r="A219" s="5" t="n"/>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>بنها</t>
-        </is>
-      </c>
-      <c r="C219" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب برج مكة</t>
-        </is>
-      </c>
+          <t>المنصورية</t>
+        </is>
+      </c>
+      <c r="C219" s="4" t="inlineStr"/>
       <c r="D219" s="4" t="inlineStr"/>
       <c r="E219" s="4" t="inlineStr"/>
       <c r="F219" s="4" t="inlineStr"/>
-      <c r="G219" s="4" t="inlineStr">
-        <is>
-          <t>شارع جميل أمام بنك القاهرة</t>
-        </is>
-      </c>
+      <c r="G219" s="4" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="5" t="n"/>
-      <c r="B220" s="5" t="n"/>
-      <c r="C220" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب كفر الجزار</t>
-        </is>
-      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>الدراسة</t>
+        </is>
+      </c>
+      <c r="C220" s="4" t="inlineStr"/>
       <c r="D220" s="4" t="inlineStr"/>
       <c r="E220" s="4" t="inlineStr"/>
       <c r="F220" s="4" t="inlineStr"/>
-      <c r="G220" s="4" t="inlineStr">
-        <is>
-          <t>بنها</t>
-        </is>
-      </c>
+      <c r="G220" s="4" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="5" t="n"/>
-      <c r="B221" s="6" t="n"/>
-      <c r="C221" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب العمار</t>
-        </is>
-      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>درب الجنينة</t>
+        </is>
+      </c>
+      <c r="C221" s="4" t="inlineStr"/>
       <c r="D221" s="4" t="inlineStr"/>
       <c r="E221" s="4" t="inlineStr"/>
       <c r="F221" s="4" t="inlineStr"/>
-      <c r="G221" s="4" t="inlineStr">
-        <is>
-          <t>بنها</t>
-        </is>
-      </c>
+      <c r="G221" s="4" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="5" t="n"/>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>قليوب</t>
+          <t>الشرابية</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr"/>
@@ -3850,12 +3922,12 @@
       <c r="A223" s="5" t="n"/>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>شبرا الخيمة</t>
+          <t>النزهة</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>مركز الغد للتخاطب وصعوبات التعلم</t>
+          <t>المركز المصري الكندي (فرع النزهة)</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr"/>
@@ -3863,49 +3935,41 @@
       <c r="F223" s="4" t="inlineStr"/>
       <c r="G223" s="4" t="inlineStr">
         <is>
-          <t>75 شارع حنفي الشيخوني</t>
+          <t>14 شارع جمال الدين علي بجوار ملاهي السندباد</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="5" t="n"/>
-      <c r="B224" s="5" t="n"/>
-      <c r="C224" s="4" t="inlineStr">
-        <is>
-          <t>مركز النور الهدى الطبي</t>
-        </is>
-      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>الرويسي</t>
+        </is>
+      </c>
+      <c r="C224" s="4" t="inlineStr"/>
       <c r="D224" s="4" t="inlineStr"/>
       <c r="E224" s="4" t="inlineStr"/>
       <c r="F224" s="4" t="inlineStr"/>
-      <c r="G224" s="4" t="inlineStr">
-        <is>
-          <t>شارع محمد القطان</t>
-        </is>
-      </c>
+      <c r="G224" s="4" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="5" t="n"/>
-      <c r="B225" s="6" t="n"/>
-      <c r="C225" s="4" t="inlineStr">
-        <is>
-          <t>مركز تواصل للتخاطب</t>
-        </is>
-      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>قصر النيل</t>
+        </is>
+      </c>
+      <c r="C225" s="4" t="inlineStr"/>
       <c r="D225" s="4" t="inlineStr"/>
       <c r="E225" s="4" t="inlineStr"/>
       <c r="F225" s="4" t="inlineStr"/>
-      <c r="G225" s="4" t="inlineStr">
-        <is>
-          <t>2 شارع أحمد عبد ربه</t>
-        </is>
-      </c>
+      <c r="G225" s="4" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="5" t="n"/>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>الخانكة</t>
+          <t>الفسطاط</t>
         </is>
       </c>
       <c r="C226" s="4" t="inlineStr"/>
@@ -3915,10 +3979,10 @@
       <c r="G226" s="4" t="inlineStr"/>
     </row>
     <row r="227">
-      <c r="A227" s="5" t="n"/>
+      <c r="A227" s="6" t="n"/>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>رمسيس</t>
+          <t>الرحاب</t>
         </is>
       </c>
       <c r="C227" s="4" t="inlineStr"/>
@@ -3928,49 +3992,69 @@
       <c r="G227" s="4" t="inlineStr"/>
     </row>
     <row r="228">
-      <c r="A228" s="5" t="n"/>
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>القليوبية</t>
+        </is>
+      </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>مدينة 10 رمضان</t>
-        </is>
-      </c>
-      <c r="C228" s="4" t="inlineStr"/>
+          <t>بنها</t>
+        </is>
+      </c>
+      <c r="C228" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب برج مكة</t>
+        </is>
+      </c>
       <c r="D228" s="4" t="inlineStr"/>
       <c r="E228" s="4" t="inlineStr"/>
       <c r="F228" s="4" t="inlineStr"/>
-      <c r="G228" s="4" t="inlineStr"/>
+      <c r="G228" s="4" t="inlineStr">
+        <is>
+          <t>شارع جميل أمام بنك القاهرة</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="5" t="n"/>
-      <c r="B229" s="3" t="inlineStr">
-        <is>
-          <t>الشيخ زايد</t>
-        </is>
-      </c>
-      <c r="C229" s="4" t="inlineStr"/>
+      <c r="B229" s="5" t="n"/>
+      <c r="C229" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب كفر الجزار</t>
+        </is>
+      </c>
       <c r="D229" s="4" t="inlineStr"/>
       <c r="E229" s="4" t="inlineStr"/>
       <c r="F229" s="4" t="inlineStr"/>
-      <c r="G229" s="4" t="inlineStr"/>
+      <c r="G229" s="4" t="inlineStr">
+        <is>
+          <t>بنها</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="5" t="n"/>
-      <c r="B230" s="3" t="inlineStr">
-        <is>
-          <t>القناطر الخيرية</t>
-        </is>
-      </c>
-      <c r="C230" s="4" t="inlineStr"/>
+      <c r="B230" s="6" t="n"/>
+      <c r="C230" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب العمار</t>
+        </is>
+      </c>
       <c r="D230" s="4" t="inlineStr"/>
       <c r="E230" s="4" t="inlineStr"/>
       <c r="F230" s="4" t="inlineStr"/>
-      <c r="G230" s="4" t="inlineStr"/>
+      <c r="G230" s="4" t="inlineStr">
+        <is>
+          <t>بنها</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="5" t="n"/>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>قها</t>
+          <t>قليوب</t>
         </is>
       </c>
       <c r="C231" s="4" t="inlineStr"/>
@@ -3983,46 +4067,62 @@
       <c r="A232" s="5" t="n"/>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>الدقهلية</t>
-        </is>
-      </c>
-      <c r="C232" s="4" t="inlineStr"/>
+          <t>شبرا الخيمة</t>
+        </is>
+      </c>
+      <c r="C232" s="4" t="inlineStr">
+        <is>
+          <t>مركز الغد للتخاطب وصعوبات التعلم</t>
+        </is>
+      </c>
       <c r="D232" s="4" t="inlineStr"/>
       <c r="E232" s="4" t="inlineStr"/>
       <c r="F232" s="4" t="inlineStr"/>
-      <c r="G232" s="4" t="inlineStr"/>
+      <c r="G232" s="4" t="inlineStr">
+        <is>
+          <t>75 شارع حنفي الشيخوني</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="5" t="n"/>
-      <c r="B233" s="3" t="inlineStr">
-        <is>
-          <t>الجيزة</t>
-        </is>
-      </c>
-      <c r="C233" s="4" t="inlineStr"/>
+      <c r="B233" s="5" t="n"/>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>مركز النور الهدى الطبي</t>
+        </is>
+      </c>
       <c r="D233" s="4" t="inlineStr"/>
       <c r="E233" s="4" t="inlineStr"/>
       <c r="F233" s="4" t="inlineStr"/>
-      <c r="G233" s="4" t="inlineStr"/>
+      <c r="G233" s="4" t="inlineStr">
+        <is>
+          <t>شارع محمد القطان</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="5" t="n"/>
-      <c r="B234" s="3" t="inlineStr">
-        <is>
-          <t>أوسيم</t>
-        </is>
-      </c>
-      <c r="C234" s="4" t="inlineStr"/>
+      <c r="B234" s="6" t="n"/>
+      <c r="C234" s="4" t="inlineStr">
+        <is>
+          <t>مركز تواصل للتخاطب</t>
+        </is>
+      </c>
       <c r="D234" s="4" t="inlineStr"/>
       <c r="E234" s="4" t="inlineStr"/>
       <c r="F234" s="4" t="inlineStr"/>
-      <c r="G234" s="4" t="inlineStr"/>
+      <c r="G234" s="4" t="inlineStr">
+        <is>
+          <t>2 شارع أحمد عبد ربه</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="5" t="n"/>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>طره</t>
+          <t>الخانكة</t>
         </is>
       </c>
       <c r="C235" s="4" t="inlineStr"/>
@@ -4035,7 +4135,7 @@
       <c r="A236" s="5" t="n"/>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>الخصوص</t>
+          <t>رمسيس</t>
         </is>
       </c>
       <c r="C236" s="4" t="inlineStr"/>
@@ -4045,10 +4145,10 @@
       <c r="G236" s="4" t="inlineStr"/>
     </row>
     <row r="237">
-      <c r="A237" s="6" t="n"/>
+      <c r="A237" s="5" t="n"/>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>القنطرة</t>
+          <t>مدينة 10 رمضان</t>
         </is>
       </c>
       <c r="C237" s="4" t="inlineStr"/>
@@ -4058,14 +4158,10 @@
       <c r="G237" s="4" t="inlineStr"/>
     </row>
     <row r="238">
-      <c r="A238" s="2" t="inlineStr">
-        <is>
-          <t>المنوفية</t>
-        </is>
-      </c>
+      <c r="A238" s="5" t="n"/>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>شبين الكوم</t>
+          <t>الشيخ زايد</t>
         </is>
       </c>
       <c r="C238" s="4" t="inlineStr"/>
@@ -4078,7 +4174,7 @@
       <c r="A239" s="5" t="n"/>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>منوف</t>
+          <t>القناطر الخيرية</t>
         </is>
       </c>
       <c r="C239" s="4" t="inlineStr"/>
@@ -4091,7 +4187,7 @@
       <c r="A240" s="5" t="n"/>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>شبين القناطر</t>
+          <t>قها</t>
         </is>
       </c>
       <c r="C240" s="4" t="inlineStr"/>
@@ -4104,7 +4200,7 @@
       <c r="A241" s="5" t="n"/>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>مدينة السادات</t>
+          <t>الدقهلية</t>
         </is>
       </c>
       <c r="C241" s="4" t="inlineStr"/>
@@ -4117,7 +4213,7 @@
       <c r="A242" s="5" t="n"/>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>باقور</t>
+          <t>الجيزة</t>
         </is>
       </c>
       <c r="C242" s="4" t="inlineStr"/>
@@ -4130,7 +4226,7 @@
       <c r="A243" s="5" t="n"/>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>تلا</t>
+          <t>أوسيم</t>
         </is>
       </c>
       <c r="C243" s="4" t="inlineStr"/>
@@ -4143,7 +4239,7 @@
       <c r="A244" s="5" t="n"/>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>قويسنا</t>
+          <t>طره</t>
         </is>
       </c>
       <c r="C244" s="4" t="inlineStr"/>
@@ -4156,28 +4252,20 @@
       <c r="A245" s="5" t="n"/>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>أشمون</t>
-        </is>
-      </c>
-      <c r="C245" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب أشمون للتخاطب</t>
-        </is>
-      </c>
+          <t>الخصوص</t>
+        </is>
+      </c>
+      <c r="C245" s="4" t="inlineStr"/>
       <c r="D245" s="4" t="inlineStr"/>
       <c r="E245" s="4" t="inlineStr"/>
       <c r="F245" s="4" t="inlineStr"/>
-      <c r="G245" s="4" t="inlineStr">
-        <is>
-          <t>أشمون</t>
-        </is>
-      </c>
+      <c r="G245" s="4" t="inlineStr"/>
     </row>
     <row r="246">
-      <c r="A246" s="5" t="n"/>
+      <c r="A246" s="6" t="n"/>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>البرجايه</t>
+          <t>القنطرة</t>
         </is>
       </c>
       <c r="C246" s="4" t="inlineStr"/>
@@ -4187,31 +4275,27 @@
       <c r="G246" s="4" t="inlineStr"/>
     </row>
     <row r="247">
-      <c r="A247" s="5" t="n"/>
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>المنوفية</t>
+        </is>
+      </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>بركة السبع</t>
-        </is>
-      </c>
-      <c r="C247" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب وصعوبات تعلم</t>
-        </is>
-      </c>
+          <t>شبين الكوم</t>
+        </is>
+      </c>
+      <c r="C247" s="4" t="inlineStr"/>
       <c r="D247" s="4" t="inlineStr"/>
       <c r="E247" s="4" t="inlineStr"/>
       <c r="F247" s="4" t="inlineStr"/>
-      <c r="G247" s="4" t="inlineStr">
-        <is>
-          <t>بركة السبع</t>
-        </is>
-      </c>
+      <c r="G247" s="4" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="5" t="n"/>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>منوف الجديدة</t>
+          <t>منوف</t>
         </is>
       </c>
       <c r="C248" s="4" t="inlineStr"/>
@@ -4221,10 +4305,10 @@
       <c r="G248" s="4" t="inlineStr"/>
     </row>
     <row r="249">
-      <c r="A249" s="6" t="n"/>
+      <c r="A249" s="5" t="n"/>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>كفر عبده</t>
+          <t>شبين القناطر</t>
         </is>
       </c>
       <c r="C249" s="4" t="inlineStr"/>
@@ -4234,52 +4318,36 @@
       <c r="G249" s="4" t="inlineStr"/>
     </row>
     <row r="250">
-      <c r="A250" s="2" t="inlineStr">
-        <is>
-          <t>المنيا</t>
-        </is>
-      </c>
+      <c r="A250" s="5" t="n"/>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>المنيا</t>
-        </is>
-      </c>
-      <c r="C250" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب بني أحمد للتخاطب</t>
-        </is>
-      </c>
+          <t>مدينة السادات</t>
+        </is>
+      </c>
+      <c r="C250" s="4" t="inlineStr"/>
       <c r="D250" s="4" t="inlineStr"/>
       <c r="E250" s="4" t="inlineStr"/>
       <c r="F250" s="4" t="inlineStr"/>
-      <c r="G250" s="4" t="inlineStr">
-        <is>
-          <t>المنيا</t>
-        </is>
-      </c>
+      <c r="G250" s="4" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="5" t="n"/>
-      <c r="B251" s="6" t="n"/>
-      <c r="C251" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب مقوسة للتخاطب</t>
-        </is>
-      </c>
+      <c r="B251" s="3" t="inlineStr">
+        <is>
+          <t>باقور</t>
+        </is>
+      </c>
+      <c r="C251" s="4" t="inlineStr"/>
       <c r="D251" s="4" t="inlineStr"/>
       <c r="E251" s="4" t="inlineStr"/>
       <c r="F251" s="4" t="inlineStr"/>
-      <c r="G251" s="4" t="inlineStr">
-        <is>
-          <t>المنيا</t>
-        </is>
-      </c>
+      <c r="G251" s="4" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="5" t="n"/>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>سمالوط</t>
+          <t>تلا</t>
         </is>
       </c>
       <c r="C252" s="4" t="inlineStr"/>
@@ -4292,7 +4360,7 @@
       <c r="A253" s="5" t="n"/>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>بني حسن</t>
+          <t>قويسنا</t>
         </is>
       </c>
       <c r="C253" s="4" t="inlineStr"/>
@@ -4305,20 +4373,28 @@
       <c r="A254" s="5" t="n"/>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>هرموبوليس</t>
-        </is>
-      </c>
-      <c r="C254" s="4" t="inlineStr"/>
+          <t>أشمون</t>
+        </is>
+      </c>
+      <c r="C254" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب أشمون للتخاطب</t>
+        </is>
+      </c>
       <c r="D254" s="4" t="inlineStr"/>
       <c r="E254" s="4" t="inlineStr"/>
       <c r="F254" s="4" t="inlineStr"/>
-      <c r="G254" s="4" t="inlineStr"/>
+      <c r="G254" s="4" t="inlineStr">
+        <is>
+          <t>أشمون</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="5" t="n"/>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>ملوي</t>
+          <t>البرجايه</t>
         </is>
       </c>
       <c r="C255" s="4" t="inlineStr"/>
@@ -4331,20 +4407,28 @@
       <c r="A256" s="5" t="n"/>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>العدوة</t>
-        </is>
-      </c>
-      <c r="C256" s="4" t="inlineStr"/>
+          <t>بركة السبع</t>
+        </is>
+      </c>
+      <c r="C256" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب وصعوبات تعلم</t>
+        </is>
+      </c>
       <c r="D256" s="4" t="inlineStr"/>
       <c r="E256" s="4" t="inlineStr"/>
       <c r="F256" s="4" t="inlineStr"/>
-      <c r="G256" s="4" t="inlineStr"/>
+      <c r="G256" s="4" t="inlineStr">
+        <is>
+          <t>بركة السبع</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="5" t="n"/>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>ديروط الشريف</t>
+          <t>منوف الجديدة</t>
         </is>
       </c>
       <c r="C257" s="4" t="inlineStr"/>
@@ -4354,10 +4438,10 @@
       <c r="G257" s="4" t="inlineStr"/>
     </row>
     <row r="258">
-      <c r="A258" s="5" t="n"/>
+      <c r="A258" s="6" t="n"/>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>أبوقرقاص</t>
+          <t>كفر عبده</t>
         </is>
       </c>
       <c r="C258" s="4" t="inlineStr"/>
@@ -4367,36 +4451,52 @@
       <c r="G258" s="4" t="inlineStr"/>
     </row>
     <row r="259">
-      <c r="A259" s="5" t="n"/>
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>المنيا</t>
+        </is>
+      </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>الفشن</t>
-        </is>
-      </c>
-      <c r="C259" s="4" t="inlineStr"/>
+          <t>المنيا</t>
+        </is>
+      </c>
+      <c r="C259" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب بني أحمد للتخاطب</t>
+        </is>
+      </c>
       <c r="D259" s="4" t="inlineStr"/>
       <c r="E259" s="4" t="inlineStr"/>
       <c r="F259" s="4" t="inlineStr"/>
-      <c r="G259" s="4" t="inlineStr"/>
+      <c r="G259" s="4" t="inlineStr">
+        <is>
+          <t>المنيا</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="5" t="n"/>
-      <c r="B260" s="3" t="inlineStr">
-        <is>
-          <t>بني مازن</t>
-        </is>
-      </c>
-      <c r="C260" s="4" t="inlineStr"/>
+      <c r="B260" s="6" t="n"/>
+      <c r="C260" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب مقوسة للتخاطب</t>
+        </is>
+      </c>
       <c r="D260" s="4" t="inlineStr"/>
       <c r="E260" s="4" t="inlineStr"/>
       <c r="F260" s="4" t="inlineStr"/>
-      <c r="G260" s="4" t="inlineStr"/>
+      <c r="G260" s="4" t="inlineStr">
+        <is>
+          <t>المنيا</t>
+        </is>
+      </c>
     </row>
     <row r="261">
-      <c r="A261" s="6" t="n"/>
+      <c r="A261" s="5" t="n"/>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>العدوة</t>
+          <t>سمالوط</t>
         </is>
       </c>
       <c r="C261" s="4" t="inlineStr"/>
@@ -4406,56 +4506,36 @@
       <c r="G261" s="4" t="inlineStr"/>
     </row>
     <row r="262">
-      <c r="A262" s="2" t="inlineStr">
-        <is>
-          <t>الوادي الجديد</t>
-        </is>
-      </c>
+      <c r="A262" s="5" t="n"/>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>الخارجة</t>
-        </is>
-      </c>
-      <c r="C262" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب الخارجة للتخاطب</t>
-        </is>
-      </c>
+          <t>بني حسن</t>
+        </is>
+      </c>
+      <c r="C262" s="4" t="inlineStr"/>
       <c r="D262" s="4" t="inlineStr"/>
       <c r="E262" s="4" t="inlineStr"/>
       <c r="F262" s="4" t="inlineStr"/>
-      <c r="G262" s="4" t="inlineStr">
-        <is>
-          <t>الخارجة</t>
-        </is>
-      </c>
+      <c r="G262" s="4" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="5" t="n"/>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>الداخلة</t>
-        </is>
-      </c>
-      <c r="C263" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب باريس للتخاطب</t>
-        </is>
-      </c>
+          <t>هرموبوليس</t>
+        </is>
+      </c>
+      <c r="C263" s="4" t="inlineStr"/>
       <c r="D263" s="4" t="inlineStr"/>
       <c r="E263" s="4" t="inlineStr"/>
       <c r="F263" s="4" t="inlineStr"/>
-      <c r="G263" s="4" t="inlineStr">
-        <is>
-          <t>باريس</t>
-        </is>
-      </c>
+      <c r="G263" s="4" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="5" t="n"/>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>موط</t>
+          <t>ملوي</t>
         </is>
       </c>
       <c r="C264" s="4" t="inlineStr"/>
@@ -4468,7 +4548,7 @@
       <c r="A265" s="5" t="n"/>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>بلاط</t>
+          <t>العدوة</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr"/>
@@ -4481,7 +4561,7 @@
       <c r="A266" s="5" t="n"/>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>فرافرة</t>
+          <t>ديروط الشريف</t>
         </is>
       </c>
       <c r="C266" s="4" t="inlineStr"/>
@@ -4494,7 +4574,7 @@
       <c r="A267" s="5" t="n"/>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>باريس</t>
+          <t>أبوقرقاص</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr"/>
@@ -4507,7 +4587,7 @@
       <c r="A268" s="5" t="n"/>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>القصر</t>
+          <t>الفشن</t>
         </is>
       </c>
       <c r="C268" s="4" t="inlineStr"/>
@@ -4520,7 +4600,7 @@
       <c r="A269" s="5" t="n"/>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>تينيدة</t>
+          <t>بني مازن</t>
         </is>
       </c>
       <c r="C269" s="4" t="inlineStr"/>
@@ -4533,7 +4613,7 @@
       <c r="A270" s="6" t="n"/>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>دوش</t>
+          <t>العدوة</t>
         </is>
       </c>
       <c r="C270" s="4" t="inlineStr"/>
@@ -4545,17 +4625,17 @@
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>بني سويف</t>
+          <t>الوادي الجديد</t>
         </is>
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>بني سويف</t>
+          <t>الخارجة</t>
         </is>
       </c>
       <c r="C271" s="4" t="inlineStr">
         <is>
-          <t>مركز شباب العبور للتخاطب</t>
+          <t>مركز شباب الخارجة للتخاطب</t>
         </is>
       </c>
       <c r="D271" s="4" t="inlineStr"/>
@@ -4563,7 +4643,7 @@
       <c r="F271" s="4" t="inlineStr"/>
       <c r="G271" s="4" t="inlineStr">
         <is>
-          <t>بني سويف</t>
+          <t>الخارجة</t>
         </is>
       </c>
     </row>
@@ -4571,20 +4651,28 @@
       <c r="A272" s="5" t="n"/>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>الفشن</t>
-        </is>
-      </c>
-      <c r="C272" s="4" t="inlineStr"/>
+          <t>الداخلة</t>
+        </is>
+      </c>
+      <c r="C272" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب باريس للتخاطب</t>
+        </is>
+      </c>
       <c r="D272" s="4" t="inlineStr"/>
       <c r="E272" s="4" t="inlineStr"/>
       <c r="F272" s="4" t="inlineStr"/>
-      <c r="G272" s="4" t="inlineStr"/>
+      <c r="G272" s="4" t="inlineStr">
+        <is>
+          <t>باريس</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="5" t="n"/>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>ساماستا</t>
+          <t>موط</t>
         </is>
       </c>
       <c r="C273" s="4" t="inlineStr"/>
@@ -4597,7 +4685,7 @@
       <c r="A274" s="5" t="n"/>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>إبشواي</t>
+          <t>بلاط</t>
         </is>
       </c>
       <c r="C274" s="4" t="inlineStr"/>
@@ -4610,7 +4698,7 @@
       <c r="A275" s="5" t="n"/>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>الجندية</t>
+          <t>فرافرة</t>
         </is>
       </c>
       <c r="C275" s="4" t="inlineStr"/>
@@ -4623,7 +4711,7 @@
       <c r="A276" s="5" t="n"/>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>ناصر</t>
+          <t>باريس</t>
         </is>
       </c>
       <c r="C276" s="4" t="inlineStr"/>
@@ -4636,7 +4724,7 @@
       <c r="A277" s="5" t="n"/>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>هواره</t>
+          <t>القصر</t>
         </is>
       </c>
       <c r="C277" s="4" t="inlineStr"/>
@@ -4649,7 +4737,7 @@
       <c r="A278" s="5" t="n"/>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>موشية</t>
+          <t>تينيدة</t>
         </is>
       </c>
       <c r="C278" s="4" t="inlineStr"/>
@@ -4659,10 +4747,10 @@
       <c r="G278" s="4" t="inlineStr"/>
     </row>
     <row r="279">
-      <c r="A279" s="5" t="n"/>
+      <c r="A279" s="6" t="n"/>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>نصار البحرية</t>
+          <t>دوش</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr"/>
@@ -4672,27 +4760,35 @@
       <c r="G279" s="4" t="inlineStr"/>
     </row>
     <row r="280">
-      <c r="A280" s="6" t="n"/>
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>بني سويف</t>
+        </is>
+      </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>أحمد حمزة</t>
-        </is>
-      </c>
-      <c r="C280" s="4" t="inlineStr"/>
+          <t>بني سويف</t>
+        </is>
+      </c>
+      <c r="C280" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب العبور للتخاطب</t>
+        </is>
+      </c>
       <c r="D280" s="4" t="inlineStr"/>
       <c r="E280" s="4" t="inlineStr"/>
       <c r="F280" s="4" t="inlineStr"/>
-      <c r="G280" s="4" t="inlineStr"/>
+      <c r="G280" s="4" t="inlineStr">
+        <is>
+          <t>بني سويف</t>
+        </is>
+      </c>
     </row>
     <row r="281">
-      <c r="A281" s="2" t="inlineStr">
-        <is>
-          <t>بورسعيد</t>
-        </is>
-      </c>
+      <c r="A281" s="5" t="n"/>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>بورسعيد</t>
+          <t>الفشن</t>
         </is>
       </c>
       <c r="C281" s="4" t="inlineStr"/>
@@ -4705,7 +4801,7 @@
       <c r="A282" s="5" t="n"/>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>بورفؤاد</t>
+          <t>ساماستا</t>
         </is>
       </c>
       <c r="C282" s="4" t="inlineStr"/>
@@ -4718,7 +4814,7 @@
       <c r="A283" s="5" t="n"/>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>الجميل</t>
+          <t>إبشواي</t>
         </is>
       </c>
       <c r="C283" s="4" t="inlineStr"/>
@@ -4731,7 +4827,7 @@
       <c r="A284" s="5" t="n"/>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>الزهور</t>
+          <t>الجندية</t>
         </is>
       </c>
       <c r="C284" s="4" t="inlineStr"/>
@@ -4744,7 +4840,7 @@
       <c r="A285" s="5" t="n"/>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>بورسعيد</t>
+          <t>ناصر</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr"/>
@@ -4757,7 +4853,7 @@
       <c r="A286" s="5" t="n"/>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>الكنتاوي</t>
+          <t>هواره</t>
         </is>
       </c>
       <c r="C286" s="4" t="inlineStr"/>
@@ -4767,10 +4863,10 @@
       <c r="G286" s="4" t="inlineStr"/>
     </row>
     <row r="287">
-      <c r="A287" s="6" t="n"/>
+      <c r="A287" s="5" t="n"/>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>الضواحي</t>
+          <t>موشية</t>
         </is>
       </c>
       <c r="C287" s="4" t="inlineStr"/>
@@ -4780,14 +4876,10 @@
       <c r="G287" s="4" t="inlineStr"/>
     </row>
     <row r="288">
-      <c r="A288" s="2" t="inlineStr">
-        <is>
-          <t>جنوب سيناء</t>
-        </is>
-      </c>
+      <c r="A288" s="5" t="n"/>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>شرم الشيخ</t>
+          <t>نصار البحرية</t>
         </is>
       </c>
       <c r="C288" s="4" t="inlineStr"/>
@@ -4797,10 +4889,10 @@
       <c r="G288" s="4" t="inlineStr"/>
     </row>
     <row r="289">
-      <c r="A289" s="5" t="n"/>
+      <c r="A289" s="6" t="n"/>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>داهب</t>
+          <t>أحمد حمزة</t>
         </is>
       </c>
       <c r="C289" s="4" t="inlineStr"/>
@@ -4810,10 +4902,14 @@
       <c r="G289" s="4" t="inlineStr"/>
     </row>
     <row r="290">
-      <c r="A290" s="5" t="n"/>
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>بورسعيد</t>
+        </is>
+      </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>نويبع</t>
+          <t>بورسعيد</t>
         </is>
       </c>
       <c r="C290" s="4" t="inlineStr"/>
@@ -4826,7 +4922,7 @@
       <c r="A291" s="5" t="n"/>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>سانت كاترين</t>
+          <t>بورفؤاد</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr"/>
@@ -4839,7 +4935,7 @@
       <c r="A292" s="5" t="n"/>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>طابا</t>
+          <t>الجميل</t>
         </is>
       </c>
       <c r="C292" s="4" t="inlineStr"/>
@@ -4852,7 +4948,7 @@
       <c r="A293" s="5" t="n"/>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>رأس محمد</t>
+          <t>الزهور</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr"/>
@@ -4865,7 +4961,7 @@
       <c r="A294" s="5" t="n"/>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>أم سيد</t>
+          <t>بورسعيد</t>
         </is>
       </c>
       <c r="C294" s="4" t="inlineStr"/>
@@ -4875,10 +4971,10 @@
       <c r="G294" s="4" t="inlineStr"/>
     </row>
     <row r="295">
-      <c r="A295" s="6" t="n"/>
+      <c r="A295" s="5" t="n"/>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>مدينة شرم الشيخ</t>
+          <t>الكنتاوي</t>
         </is>
       </c>
       <c r="C295" s="4" t="inlineStr"/>
@@ -4888,14 +4984,10 @@
       <c r="G295" s="4" t="inlineStr"/>
     </row>
     <row r="296">
-      <c r="A296" s="2" t="inlineStr">
-        <is>
-          <t>حلوان</t>
-        </is>
-      </c>
+      <c r="A296" s="6" t="n"/>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>حلوان</t>
+          <t>الضواحي</t>
         </is>
       </c>
       <c r="C296" s="4" t="inlineStr"/>
@@ -4905,10 +4997,14 @@
       <c r="G296" s="4" t="inlineStr"/>
     </row>
     <row r="297">
-      <c r="A297" s="5" t="n"/>
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>جنوب سيناء</t>
+        </is>
+      </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>المعادي</t>
+          <t>شرم الشيخ</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr"/>
@@ -4921,7 +5017,7 @@
       <c r="A298" s="5" t="n"/>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>واحة الفيوم</t>
+          <t>داهب</t>
         </is>
       </c>
       <c r="C298" s="4" t="inlineStr"/>
@@ -4934,7 +5030,7 @@
       <c r="A299" s="5" t="n"/>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>وادي حوف</t>
+          <t>نويبع</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr"/>
@@ -4947,7 +5043,7 @@
       <c r="A300" s="5" t="n"/>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>عين سخنة</t>
+          <t>سانت كاترين</t>
         </is>
       </c>
       <c r="C300" s="4" t="inlineStr"/>
@@ -4960,7 +5056,7 @@
       <c r="A301" s="5" t="n"/>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>الطور</t>
+          <t>طابا</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr"/>
@@ -4973,7 +5069,7 @@
       <c r="A302" s="5" t="n"/>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>الزيتون</t>
+          <t>رأس محمد</t>
         </is>
       </c>
       <c r="C302" s="4" t="inlineStr"/>
@@ -4983,10 +5079,10 @@
       <c r="G302" s="4" t="inlineStr"/>
     </row>
     <row r="303">
-      <c r="A303" s="6" t="n"/>
+      <c r="A303" s="5" t="n"/>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>المقطم</t>
+          <t>أم سيد</t>
         </is>
       </c>
       <c r="C303" s="4" t="inlineStr"/>
@@ -4996,35 +5092,27 @@
       <c r="G303" s="4" t="inlineStr"/>
     </row>
     <row r="304">
-      <c r="A304" s="2" t="inlineStr">
-        <is>
-          <t>دمياط</t>
-        </is>
-      </c>
+      <c r="A304" s="6" t="n"/>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>دمياط</t>
-        </is>
-      </c>
-      <c r="C304" s="4" t="inlineStr">
-        <is>
-          <t>مركز حلم ابني للتخاطب</t>
-        </is>
-      </c>
+          <t>مدينة شرم الشيخ</t>
+        </is>
+      </c>
+      <c r="C304" s="4" t="inlineStr"/>
       <c r="D304" s="4" t="inlineStr"/>
       <c r="E304" s="4" t="inlineStr"/>
       <c r="F304" s="4" t="inlineStr"/>
-      <c r="G304" s="4" t="inlineStr">
-        <is>
-          <t>دمياط ودمياط الجديدة</t>
-        </is>
-      </c>
+      <c r="G304" s="4" t="inlineStr"/>
     </row>
     <row r="305">
-      <c r="A305" s="5" t="n"/>
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>حلوان</t>
+        </is>
+      </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>دمياط الجديدة</t>
+          <t>حلوان</t>
         </is>
       </c>
       <c r="C305" s="4" t="inlineStr"/>
@@ -5037,7 +5125,7 @@
       <c r="A306" s="5" t="n"/>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>بورت فؤاد</t>
+          <t>المعادي</t>
         </is>
       </c>
       <c r="C306" s="4" t="inlineStr"/>
@@ -5050,7 +5138,7 @@
       <c r="A307" s="5" t="n"/>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>كفر البطة</t>
+          <t>واحة الفيوم</t>
         </is>
       </c>
       <c r="C307" s="4" t="inlineStr"/>
@@ -5063,7 +5151,7 @@
       <c r="A308" s="5" t="n"/>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>كفر سعيد</t>
+          <t>وادي حوف</t>
         </is>
       </c>
       <c r="C308" s="4" t="inlineStr"/>
@@ -5076,7 +5164,7 @@
       <c r="A309" s="5" t="n"/>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>الروضة</t>
+          <t>عين سخنة</t>
         </is>
       </c>
       <c r="C309" s="4" t="inlineStr"/>
@@ -5089,7 +5177,7 @@
       <c r="A310" s="5" t="n"/>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>الزرقا</t>
+          <t>الطور</t>
         </is>
       </c>
       <c r="C310" s="4" t="inlineStr"/>
@@ -5102,7 +5190,7 @@
       <c r="A311" s="5" t="n"/>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>فارسكور</t>
+          <t>الزيتون</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr"/>
@@ -5115,7 +5203,7 @@
       <c r="A312" s="6" t="n"/>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>رومانية</t>
+          <t>المقطم</t>
         </is>
       </c>
       <c r="C312" s="4" t="inlineStr"/>
@@ -5127,17 +5215,17 @@
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>شمال سيناء</t>
+          <t>دمياط</t>
         </is>
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>العريش</t>
+          <t>دمياط</t>
         </is>
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>مركز شباب العريش للتخاطب</t>
+          <t>مركز حلم ابني للتخاطب</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr"/>
@@ -5145,7 +5233,7 @@
       <c r="F313" s="4" t="inlineStr"/>
       <c r="G313" s="4" t="inlineStr">
         <is>
-          <t>مركز شباب العريش</t>
+          <t>دمياط ودمياط الجديدة</t>
         </is>
       </c>
     </row>
@@ -5153,49 +5241,33 @@
       <c r="A314" s="5" t="n"/>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>رفح</t>
-        </is>
-      </c>
-      <c r="C314" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب رفح</t>
-        </is>
-      </c>
+          <t>دمياط الجديدة</t>
+        </is>
+      </c>
+      <c r="C314" s="4" t="inlineStr"/>
       <c r="D314" s="4" t="inlineStr"/>
       <c r="E314" s="4" t="inlineStr"/>
       <c r="F314" s="4" t="inlineStr"/>
-      <c r="G314" s="4" t="inlineStr">
-        <is>
-          <t>رفح</t>
-        </is>
-      </c>
+      <c r="G314" s="4" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" s="5" t="n"/>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>الشيخ زويد</t>
-        </is>
-      </c>
-      <c r="C315" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب الشيخ زويد (قيد الإنشاء)</t>
-        </is>
-      </c>
+          <t>بورت فؤاد</t>
+        </is>
+      </c>
+      <c r="C315" s="4" t="inlineStr"/>
       <c r="D315" s="4" t="inlineStr"/>
       <c r="E315" s="4" t="inlineStr"/>
       <c r="F315" s="4" t="inlineStr"/>
-      <c r="G315" s="4" t="inlineStr">
-        <is>
-          <t>الشيخ زويد</t>
-        </is>
-      </c>
+      <c r="G315" s="4" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" s="5" t="n"/>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>بئر العبد</t>
+          <t>كفر البطة</t>
         </is>
       </c>
       <c r="C316" s="4" t="inlineStr"/>
@@ -5208,7 +5280,7 @@
       <c r="A317" s="5" t="n"/>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>القنطرة، سيناء</t>
+          <t>كفر سعيد</t>
         </is>
       </c>
       <c r="C317" s="4" t="inlineStr"/>
@@ -5221,7 +5293,7 @@
       <c r="A318" s="5" t="n"/>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>نخل</t>
+          <t>الروضة</t>
         </is>
       </c>
       <c r="C318" s="4" t="inlineStr"/>
@@ -5234,7 +5306,7 @@
       <c r="A319" s="5" t="n"/>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>جديدة، حسنة</t>
+          <t>الزرقا</t>
         </is>
       </c>
       <c r="C319" s="4" t="inlineStr"/>
@@ -5247,7 +5319,7 @@
       <c r="A320" s="5" t="n"/>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>دهب الشرقية</t>
+          <t>فارسكور</t>
         </is>
       </c>
       <c r="C320" s="4" t="inlineStr"/>
@@ -5260,7 +5332,7 @@
       <c r="A321" s="6" t="n"/>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>طابا</t>
+          <t>رومانية</t>
         </is>
       </c>
       <c r="C321" s="4" t="inlineStr"/>
@@ -5272,17 +5344,17 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>قنا</t>
+          <t>شمال سيناء</t>
         </is>
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>قنا</t>
+          <t>العريش</t>
         </is>
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>مركز التخاطب بمدينة العمال</t>
+          <t>مركز شباب العريش للتخاطب</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr"/>
@@ -5290,16 +5362,20 @@
       <c r="F322" s="4" t="inlineStr"/>
       <c r="G322" s="4" t="inlineStr">
         <is>
-          <t>مدينة العمال، قنا</t>
+          <t>مركز شباب العريش</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="5" t="n"/>
-      <c r="B323" s="6" t="n"/>
+      <c r="B323" s="3" t="inlineStr">
+        <is>
+          <t>رفح</t>
+        </is>
+      </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>مركز شباب حجير خزام</t>
+          <t>مركز تخاطب رفح</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr"/>
@@ -5307,7 +5383,7 @@
       <c r="F323" s="4" t="inlineStr"/>
       <c r="G323" s="4" t="inlineStr">
         <is>
-          <t>قنا</t>
+          <t>رفح</t>
         </is>
       </c>
     </row>
@@ -5315,20 +5391,28 @@
       <c r="A324" s="5" t="n"/>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>نجع حمادي</t>
-        </is>
-      </c>
-      <c r="C324" s="4" t="inlineStr"/>
+          <t>الشيخ زويد</t>
+        </is>
+      </c>
+      <c r="C324" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب الشيخ زويد (قيد الإنشاء)</t>
+        </is>
+      </c>
       <c r="D324" s="4" t="inlineStr"/>
       <c r="E324" s="4" t="inlineStr"/>
       <c r="F324" s="4" t="inlineStr"/>
-      <c r="G324" s="4" t="inlineStr"/>
+      <c r="G324" s="4" t="inlineStr">
+        <is>
+          <t>الشيخ زويد</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="5" t="n"/>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>دندرة</t>
+          <t>بئر العبد</t>
         </is>
       </c>
       <c r="C325" s="4" t="inlineStr"/>
@@ -5341,7 +5425,7 @@
       <c r="A326" s="5" t="n"/>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>أبيدوس</t>
+          <t>القنطرة، سيناء</t>
         </is>
       </c>
       <c r="C326" s="4" t="inlineStr"/>
@@ -5354,7 +5438,7 @@
       <c r="A327" s="5" t="n"/>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>قفطي</t>
+          <t>نخل</t>
         </is>
       </c>
       <c r="C327" s="4" t="inlineStr"/>
@@ -5367,7 +5451,7 @@
       <c r="A328" s="5" t="n"/>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>أخميم</t>
+          <t>جديدة، حسنة</t>
         </is>
       </c>
       <c r="C328" s="4" t="inlineStr"/>
@@ -5380,7 +5464,7 @@
       <c r="A329" s="5" t="n"/>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>سوهاج القديمة</t>
+          <t>دهب الشرقية</t>
         </is>
       </c>
       <c r="C329" s="4" t="inlineStr"/>
@@ -5390,10 +5474,10 @@
       <c r="G329" s="4" t="inlineStr"/>
     </row>
     <row r="330">
-      <c r="A330" s="5" t="n"/>
+      <c r="A330" s="6" t="n"/>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>النجع البحري</t>
+          <t>طابا</t>
         </is>
       </c>
       <c r="C330" s="4" t="inlineStr"/>
@@ -5403,32 +5487,36 @@
       <c r="G330" s="4" t="inlineStr"/>
     </row>
     <row r="331">
-      <c r="A331" s="6" t="n"/>
+      <c r="A331" s="2" t="inlineStr">
+        <is>
+          <t>قنا</t>
+        </is>
+      </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>الشنقي</t>
-        </is>
-      </c>
-      <c r="C331" s="4" t="inlineStr"/>
+          <t>قنا</t>
+        </is>
+      </c>
+      <c r="C331" s="4" t="inlineStr">
+        <is>
+          <t>مركز التخاطب بمدينة العمال</t>
+        </is>
+      </c>
       <c r="D331" s="4" t="inlineStr"/>
       <c r="E331" s="4" t="inlineStr"/>
       <c r="F331" s="4" t="inlineStr"/>
-      <c r="G331" s="4" t="inlineStr"/>
+      <c r="G331" s="4" t="inlineStr">
+        <is>
+          <t>مدينة العمال، قنا</t>
+        </is>
+      </c>
     </row>
     <row r="332">
-      <c r="A332" s="2" t="inlineStr">
-        <is>
-          <t>كفر الشيخ</t>
-        </is>
-      </c>
-      <c r="B332" s="3" t="inlineStr">
-        <is>
-          <t>كفر الشيخ</t>
-        </is>
-      </c>
+      <c r="A332" s="5" t="n"/>
+      <c r="B332" s="6" t="n"/>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>مركز شباب كفر الشيخ للتخاطب</t>
+          <t>مركز شباب حجير خزام</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr"/>
@@ -5436,7 +5524,7 @@
       <c r="F332" s="4" t="inlineStr"/>
       <c r="G332" s="4" t="inlineStr">
         <is>
-          <t>كفر الشيخ</t>
+          <t>قنا</t>
         </is>
       </c>
     </row>
@@ -5444,28 +5532,20 @@
       <c r="A333" s="5" t="n"/>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>دسوق</t>
-        </is>
-      </c>
-      <c r="C333" s="4" t="inlineStr">
-        <is>
-          <t>مركز رعايه للتخاطب والتدخل المبكر</t>
-        </is>
-      </c>
+          <t>نجع حمادي</t>
+        </is>
+      </c>
+      <c r="C333" s="4" t="inlineStr"/>
       <c r="D333" s="4" t="inlineStr"/>
       <c r="E333" s="4" t="inlineStr"/>
       <c r="F333" s="4" t="inlineStr"/>
-      <c r="G333" s="4" t="inlineStr">
-        <is>
-          <t>شارع شهداء المغربي، خلف جمعية الشروق</t>
-        </is>
-      </c>
+      <c r="G333" s="4" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" s="5" t="n"/>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>بلامون</t>
+          <t>دندرة</t>
         </is>
       </c>
       <c r="C334" s="4" t="inlineStr"/>
@@ -5478,7 +5558,7 @@
       <c r="A335" s="5" t="n"/>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>الرياض</t>
+          <t>أبيدوس</t>
         </is>
       </c>
       <c r="C335" s="4" t="inlineStr"/>
@@ -5491,7 +5571,7 @@
       <c r="A336" s="5" t="n"/>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>سيدي سالم</t>
+          <t>قفطي</t>
         </is>
       </c>
       <c r="C336" s="4" t="inlineStr"/>
@@ -5504,7 +5584,7 @@
       <c r="A337" s="5" t="n"/>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>الحامول</t>
+          <t>أخميم</t>
         </is>
       </c>
       <c r="C337" s="4" t="inlineStr"/>
@@ -5517,7 +5597,7 @@
       <c r="A338" s="5" t="n"/>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>برج البرلس</t>
+          <t>سوهاج القديمة</t>
         </is>
       </c>
       <c r="C338" s="4" t="inlineStr"/>
@@ -5530,7 +5610,7 @@
       <c r="A339" s="5" t="n"/>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>مطوبس</t>
+          <t>النجع البحري</t>
         </is>
       </c>
       <c r="C339" s="4" t="inlineStr"/>
@@ -5540,10 +5620,10 @@
       <c r="G339" s="4" t="inlineStr"/>
     </row>
     <row r="340">
-      <c r="A340" s="5" t="n"/>
+      <c r="A340" s="6" t="n"/>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>المحمودية</t>
+          <t>الشنقي</t>
         </is>
       </c>
       <c r="C340" s="4" t="inlineStr"/>
@@ -5553,44 +5633,56 @@
       <c r="G340" s="4" t="inlineStr"/>
     </row>
     <row r="341">
-      <c r="A341" s="6" t="n"/>
+      <c r="A341" s="2" t="inlineStr">
+        <is>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>بيلا</t>
-        </is>
-      </c>
-      <c r="C341" s="4" t="inlineStr"/>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
+      <c r="C341" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب كفر الشيخ للتخاطب</t>
+        </is>
+      </c>
       <c r="D341" s="4" t="inlineStr"/>
       <c r="E341" s="4" t="inlineStr"/>
       <c r="F341" s="4" t="inlineStr"/>
-      <c r="G341" s="4" t="inlineStr"/>
+      <c r="G341" s="4" t="inlineStr">
+        <is>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
     </row>
     <row r="342">
-      <c r="A342" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A342" s="5" t="n"/>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="C342" s="4" t="inlineStr"/>
+          <t>دسوق</t>
+        </is>
+      </c>
+      <c r="C342" s="4" t="inlineStr">
+        <is>
+          <t>مركز رعايه للتخاطب والتدخل المبكر</t>
+        </is>
+      </c>
       <c r="D342" s="4" t="inlineStr"/>
       <c r="E342" s="4" t="inlineStr"/>
       <c r="F342" s="4" t="inlineStr"/>
-      <c r="G342" s="4" t="inlineStr"/>
+      <c r="G342" s="4" t="inlineStr">
+        <is>
+          <t>شارع شهداء المغربي، خلف جمعية الشروق</t>
+        </is>
+      </c>
     </row>
     <row r="343">
-      <c r="A343" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A343" s="5" t="n"/>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>سيوه</t>
+          <t>بلامون</t>
         </is>
       </c>
       <c r="C343" s="4" t="inlineStr"/>
@@ -5600,14 +5692,10 @@
       <c r="G343" s="4" t="inlineStr"/>
     </row>
     <row r="344">
-      <c r="A344" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A344" s="5" t="n"/>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>السلوم</t>
+          <t>الرياض</t>
         </is>
       </c>
       <c r="C344" s="4" t="inlineStr"/>
@@ -5617,14 +5705,10 @@
       <c r="G344" s="4" t="inlineStr"/>
     </row>
     <row r="345">
-      <c r="A345" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A345" s="5" t="n"/>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>سيدي براني</t>
+          <t>سيدي سالم</t>
         </is>
       </c>
       <c r="C345" s="4" t="inlineStr"/>
@@ -5634,14 +5718,10 @@
       <c r="G345" s="4" t="inlineStr"/>
     </row>
     <row r="346">
-      <c r="A346" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A346" s="5" t="n"/>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>العلمين</t>
+          <t>الحامول</t>
         </is>
       </c>
       <c r="C346" s="4" t="inlineStr"/>
@@ -5651,14 +5731,10 @@
       <c r="G346" s="4" t="inlineStr"/>
     </row>
     <row r="347">
-      <c r="A347" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A347" s="5" t="n"/>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>مارينا</t>
+          <t>برج البرلس</t>
         </is>
       </c>
       <c r="C347" s="4" t="inlineStr"/>
@@ -5668,14 +5744,10 @@
       <c r="G347" s="4" t="inlineStr"/>
     </row>
     <row r="348">
-      <c r="A348" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A348" s="5" t="n"/>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>توريدو</t>
+          <t>مطوبس</t>
         </is>
       </c>
       <c r="C348" s="4" t="inlineStr"/>
@@ -5685,14 +5757,10 @@
       <c r="G348" s="4" t="inlineStr"/>
     </row>
     <row r="349">
-      <c r="A349" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A349" s="5" t="n"/>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>جنوب سيوه</t>
+          <t>المحمودية</t>
         </is>
       </c>
       <c r="C349" s="4" t="inlineStr"/>
@@ -5702,14 +5770,10 @@
       <c r="G349" s="4" t="inlineStr"/>
     </row>
     <row r="350">
-      <c r="A350" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A350" s="6" t="n"/>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>شمال سيوه</t>
+          <t>بيلا</t>
         </is>
       </c>
       <c r="C350" s="4" t="inlineStr"/>
@@ -5726,7 +5790,7 @@
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>كشته</t>
+          <t>مطروح</t>
         </is>
       </c>
       <c r="C351" s="4" t="inlineStr"/>
@@ -5735,90 +5799,240 @@
       <c r="F351" s="4" t="inlineStr"/>
       <c r="G351" s="4" t="inlineStr"/>
     </row>
+    <row r="352">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B352" s="3" t="inlineStr">
+        <is>
+          <t>سيوه</t>
+        </is>
+      </c>
+      <c r="C352" s="4" t="inlineStr"/>
+      <c r="D352" s="4" t="inlineStr"/>
+      <c r="E352" s="4" t="inlineStr"/>
+      <c r="F352" s="4" t="inlineStr"/>
+      <c r="G352" s="4" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B353" s="3" t="inlineStr">
+        <is>
+          <t>السلوم</t>
+        </is>
+      </c>
+      <c r="C353" s="4" t="inlineStr"/>
+      <c r="D353" s="4" t="inlineStr"/>
+      <c r="E353" s="4" t="inlineStr"/>
+      <c r="F353" s="4" t="inlineStr"/>
+      <c r="G353" s="4" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B354" s="3" t="inlineStr">
+        <is>
+          <t>سيدي براني</t>
+        </is>
+      </c>
+      <c r="C354" s="4" t="inlineStr"/>
+      <c r="D354" s="4" t="inlineStr"/>
+      <c r="E354" s="4" t="inlineStr"/>
+      <c r="F354" s="4" t="inlineStr"/>
+      <c r="G354" s="4" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B355" s="3" t="inlineStr">
+        <is>
+          <t>العلمين</t>
+        </is>
+      </c>
+      <c r="C355" s="4" t="inlineStr"/>
+      <c r="D355" s="4" t="inlineStr"/>
+      <c r="E355" s="4" t="inlineStr"/>
+      <c r="F355" s="4" t="inlineStr"/>
+      <c r="G355" s="4" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B356" s="3" t="inlineStr">
+        <is>
+          <t>مارينا</t>
+        </is>
+      </c>
+      <c r="C356" s="4" t="inlineStr"/>
+      <c r="D356" s="4" t="inlineStr"/>
+      <c r="E356" s="4" t="inlineStr"/>
+      <c r="F356" s="4" t="inlineStr"/>
+      <c r="G356" s="4" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B357" s="3" t="inlineStr">
+        <is>
+          <t>توريدو</t>
+        </is>
+      </c>
+      <c r="C357" s="4" t="inlineStr"/>
+      <c r="D357" s="4" t="inlineStr"/>
+      <c r="E357" s="4" t="inlineStr"/>
+      <c r="F357" s="4" t="inlineStr"/>
+      <c r="G357" s="4" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B358" s="3" t="inlineStr">
+        <is>
+          <t>جنوب سيوه</t>
+        </is>
+      </c>
+      <c r="C358" s="4" t="inlineStr"/>
+      <c r="D358" s="4" t="inlineStr"/>
+      <c r="E358" s="4" t="inlineStr"/>
+      <c r="F358" s="4" t="inlineStr"/>
+      <c r="G358" s="4" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B359" s="3" t="inlineStr">
+        <is>
+          <t>شمال سيوه</t>
+        </is>
+      </c>
+      <c r="C359" s="4" t="inlineStr"/>
+      <c r="D359" s="4" t="inlineStr"/>
+      <c r="E359" s="4" t="inlineStr"/>
+      <c r="F359" s="4" t="inlineStr"/>
+      <c r="G359" s="4" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B360" s="3" t="inlineStr">
+        <is>
+          <t>كشته</t>
+        </is>
+      </c>
+      <c r="C360" s="4" t="inlineStr"/>
+      <c r="D360" s="4" t="inlineStr"/>
+      <c r="E360" s="4" t="inlineStr"/>
+      <c r="F360" s="4" t="inlineStr"/>
+      <c r="G360" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="313">
     <mergeCell ref="B6"/>
     <mergeCell ref="B133"/>
     <mergeCell ref="B204"/>
-    <mergeCell ref="B198"/>
-    <mergeCell ref="B296"/>
+    <mergeCell ref="B356"/>
     <mergeCell ref="B4"/>
     <mergeCell ref="B75"/>
     <mergeCell ref="B135"/>
     <mergeCell ref="B306"/>
     <mergeCell ref="B62"/>
-    <mergeCell ref="B233"/>
-    <mergeCell ref="B227"/>
     <mergeCell ref="B72"/>
-    <mergeCell ref="B199"/>
+    <mergeCell ref="A290:A296"/>
     <mergeCell ref="B291"/>
     <mergeCell ref="B70"/>
-    <mergeCell ref="B228"/>
     <mergeCell ref="B293"/>
     <mergeCell ref="A12:A23"/>
-    <mergeCell ref="A219:A237"/>
+    <mergeCell ref="B322"/>
     <mergeCell ref="B17"/>
     <mergeCell ref="B88"/>
     <mergeCell ref="B82"/>
     <mergeCell ref="B152:B156"/>
+    <mergeCell ref="B185:B188"/>
     <mergeCell ref="B19"/>
     <mergeCell ref="B146"/>
     <mergeCell ref="B317"/>
     <mergeCell ref="B217"/>
-    <mergeCell ref="B65"/>
+    <mergeCell ref="A259:A270"/>
     <mergeCell ref="B83"/>
     <mergeCell ref="B344"/>
     <mergeCell ref="B319"/>
+    <mergeCell ref="A178:A227"/>
     <mergeCell ref="B123"/>
+    <mergeCell ref="B221"/>
     <mergeCell ref="B110"/>
-    <mergeCell ref="A262:A270"/>
     <mergeCell ref="B141"/>
     <mergeCell ref="B248"/>
     <mergeCell ref="B297"/>
+    <mergeCell ref="B108:B109"/>
     <mergeCell ref="B235"/>
     <mergeCell ref="B14"/>
+    <mergeCell ref="B331:B332"/>
     <mergeCell ref="B299"/>
     <mergeCell ref="B78"/>
+    <mergeCell ref="B249"/>
     <mergeCell ref="B243"/>
+    <mergeCell ref="A331:A340"/>
     <mergeCell ref="B314"/>
-    <mergeCell ref="A332:A341"/>
+    <mergeCell ref="A247:A258"/>
     <mergeCell ref="B167:B168"/>
     <mergeCell ref="B325"/>
-    <mergeCell ref="B250:B251"/>
-    <mergeCell ref="B91"/>
+    <mergeCell ref="B259:B260"/>
     <mergeCell ref="B25"/>
     <mergeCell ref="B327"/>
-    <mergeCell ref="A178:A218"/>
     <mergeCell ref="B149"/>
+    <mergeCell ref="B220"/>
     <mergeCell ref="B247"/>
-    <mergeCell ref="B223:B225"/>
     <mergeCell ref="B262"/>
+    <mergeCell ref="B38"/>
+    <mergeCell ref="A271:A279"/>
     <mergeCell ref="B84"/>
-    <mergeCell ref="B246"/>
-    <mergeCell ref="B40"/>
     <mergeCell ref="B338"/>
     <mergeCell ref="B15"/>
     <mergeCell ref="B313"/>
     <mergeCell ref="B104"/>
-    <mergeCell ref="B340"/>
     <mergeCell ref="B79"/>
     <mergeCell ref="B315"/>
     <mergeCell ref="B302"/>
     <mergeCell ref="B81"/>
     <mergeCell ref="B252"/>
-    <mergeCell ref="B208"/>
     <mergeCell ref="B210"/>
     <mergeCell ref="B318"/>
+    <mergeCell ref="B189:B190"/>
     <mergeCell ref="B170"/>
     <mergeCell ref="B157"/>
     <mergeCell ref="B328"/>
     <mergeCell ref="B333"/>
-    <mergeCell ref="B234"/>
-    <mergeCell ref="A322:A331"/>
+    <mergeCell ref="B66:B67"/>
     <mergeCell ref="B172"/>
     <mergeCell ref="B28"/>
     <mergeCell ref="B99"/>
-    <mergeCell ref="B186"/>
     <mergeCell ref="B137:B139"/>
     <mergeCell ref="B257"/>
     <mergeCell ref="B30"/>
@@ -5826,18 +6040,18 @@
     <mergeCell ref="B265"/>
     <mergeCell ref="B54"/>
     <mergeCell ref="B125"/>
-    <mergeCell ref="B56"/>
+    <mergeCell ref="B323"/>
     <mergeCell ref="B176"/>
     <mergeCell ref="B120"/>
-    <mergeCell ref="B219:B221"/>
     <mergeCell ref="B147"/>
     <mergeCell ref="B245"/>
     <mergeCell ref="B9"/>
+    <mergeCell ref="B359"/>
     <mergeCell ref="B207"/>
     <mergeCell ref="B334"/>
-    <mergeCell ref="B67:B68"/>
     <mergeCell ref="B113"/>
     <mergeCell ref="B173"/>
+    <mergeCell ref="B33:B37"/>
     <mergeCell ref="B100"/>
     <mergeCell ref="B271"/>
     <mergeCell ref="B336"/>
@@ -5845,115 +6059,112 @@
     <mergeCell ref="B202"/>
     <mergeCell ref="B102"/>
     <mergeCell ref="B273"/>
+    <mergeCell ref="B232:B234"/>
     <mergeCell ref="B39"/>
-    <mergeCell ref="A67:A77"/>
     <mergeCell ref="B191"/>
     <mergeCell ref="B349"/>
     <mergeCell ref="B255"/>
     <mergeCell ref="B226"/>
     <mergeCell ref="B49"/>
     <mergeCell ref="B192"/>
+    <mergeCell ref="A280:A289"/>
     <mergeCell ref="B284"/>
     <mergeCell ref="B222"/>
     <mergeCell ref="A313:A321"/>
     <mergeCell ref="B63"/>
     <mergeCell ref="B197"/>
     <mergeCell ref="B50"/>
-    <mergeCell ref="A78:A92"/>
+    <mergeCell ref="A57:A65"/>
     <mergeCell ref="B286"/>
+    <mergeCell ref="B261"/>
     <mergeCell ref="B27"/>
     <mergeCell ref="B337"/>
+    <mergeCell ref="B352"/>
     <mergeCell ref="B103"/>
     <mergeCell ref="B174"/>
-    <mergeCell ref="B230"/>
     <mergeCell ref="B205"/>
     <mergeCell ref="B339"/>
     <mergeCell ref="B118"/>
+    <mergeCell ref="A66:A76"/>
     <mergeCell ref="B55"/>
-    <mergeCell ref="A288:A295"/>
     <mergeCell ref="B169"/>
-    <mergeCell ref="B322:B323"/>
+    <mergeCell ref="B355"/>
     <mergeCell ref="B7"/>
     <mergeCell ref="B129"/>
-    <mergeCell ref="B200"/>
     <mergeCell ref="B134"/>
     <mergeCell ref="B194"/>
     <mergeCell ref="B121"/>
     <mergeCell ref="B292"/>
+    <mergeCell ref="B357"/>
     <mergeCell ref="B71"/>
     <mergeCell ref="B131"/>
     <mergeCell ref="B236"/>
     <mergeCell ref="B307"/>
     <mergeCell ref="B58"/>
     <mergeCell ref="B52"/>
+    <mergeCell ref="B223"/>
     <mergeCell ref="B294"/>
-    <mergeCell ref="B350"/>
     <mergeCell ref="B2"/>
     <mergeCell ref="B195"/>
     <mergeCell ref="B60"/>
-    <mergeCell ref="A58:A66"/>
     <mergeCell ref="B231"/>
+    <mergeCell ref="B287"/>
+    <mergeCell ref="B358"/>
     <mergeCell ref="A24:A32"/>
     <mergeCell ref="B53"/>
+    <mergeCell ref="A341:A350"/>
     <mergeCell ref="A152:A166"/>
-    <mergeCell ref="B289"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="B241"/>
     <mergeCell ref="B124"/>
+    <mergeCell ref="B178:B184"/>
     <mergeCell ref="B142"/>
     <mergeCell ref="B80"/>
     <mergeCell ref="B213"/>
     <mergeCell ref="B305"/>
-    <mergeCell ref="B188"/>
     <mergeCell ref="B126"/>
+    <mergeCell ref="B218"/>
     <mergeCell ref="B242"/>
-    <mergeCell ref="B190"/>
     <mergeCell ref="B46"/>
     <mergeCell ref="B282"/>
-    <mergeCell ref="A271:A280"/>
     <mergeCell ref="B48"/>
+    <mergeCell ref="B219"/>
     <mergeCell ref="B346"/>
+    <mergeCell ref="A297:A304"/>
     <mergeCell ref="B8"/>
     <mergeCell ref="B73"/>
     <mergeCell ref="B10"/>
     <mergeCell ref="B308"/>
     <mergeCell ref="B74"/>
+    <mergeCell ref="B68"/>
     <mergeCell ref="B201"/>
     <mergeCell ref="B239"/>
     <mergeCell ref="B310"/>
     <mergeCell ref="B5"/>
-    <mergeCell ref="B76"/>
     <mergeCell ref="B203"/>
-    <mergeCell ref="B232"/>
     <mergeCell ref="B150"/>
     <mergeCell ref="B326"/>
     <mergeCell ref="B215"/>
     <mergeCell ref="B21"/>
     <mergeCell ref="B263"/>
     <mergeCell ref="B244"/>
-    <mergeCell ref="B229"/>
-    <mergeCell ref="B93:B97"/>
     <mergeCell ref="A167:A177"/>
     <mergeCell ref="B283"/>
     <mergeCell ref="B87"/>
-    <mergeCell ref="B258"/>
-    <mergeCell ref="A238:A249"/>
     <mergeCell ref="B298"/>
     <mergeCell ref="B285"/>
-    <mergeCell ref="B260"/>
     <mergeCell ref="B64"/>
     <mergeCell ref="B51"/>
     <mergeCell ref="B163"/>
     <mergeCell ref="B309"/>
-    <mergeCell ref="B209"/>
-    <mergeCell ref="B41:B43"/>
     <mergeCell ref="B165"/>
     <mergeCell ref="B140"/>
     <mergeCell ref="B311"/>
     <mergeCell ref="B238"/>
+    <mergeCell ref="B105:B107"/>
+    <mergeCell ref="B77"/>
     <mergeCell ref="B253"/>
     <mergeCell ref="B240"/>
-    <mergeCell ref="B33:B38"/>
     <mergeCell ref="A2:A11"/>
     <mergeCell ref="B29"/>
     <mergeCell ref="B158"/>
@@ -5962,16 +6173,17 @@
     <mergeCell ref="B24"/>
     <mergeCell ref="B266"/>
     <mergeCell ref="B89"/>
+    <mergeCell ref="B198:B200"/>
+    <mergeCell ref="B92:B96"/>
     <mergeCell ref="B26"/>
-    <mergeCell ref="B330"/>
+    <mergeCell ref="B97"/>
     <mergeCell ref="B268"/>
     <mergeCell ref="B324"/>
+    <mergeCell ref="B224"/>
     <mergeCell ref="B90"/>
-    <mergeCell ref="B184"/>
     <mergeCell ref="B148"/>
+    <mergeCell ref="B250"/>
     <mergeCell ref="B44"/>
-    <mergeCell ref="B304"/>
-    <mergeCell ref="B279"/>
     <mergeCell ref="B115:B116"/>
     <mergeCell ref="B254"/>
     <mergeCell ref="B143"/>
@@ -5983,47 +6195,49 @@
     <mergeCell ref="B160:B162"/>
     <mergeCell ref="B159"/>
     <mergeCell ref="B272"/>
-    <mergeCell ref="B332"/>
-    <mergeCell ref="B259"/>
     <mergeCell ref="B111"/>
     <mergeCell ref="B98"/>
+    <mergeCell ref="B225"/>
     <mergeCell ref="B274"/>
     <mergeCell ref="B175"/>
+    <mergeCell ref="B228:B230"/>
     <mergeCell ref="A129:A136"/>
     <mergeCell ref="B267"/>
     <mergeCell ref="B269"/>
-    <mergeCell ref="B187"/>
-    <mergeCell ref="B178:B182"/>
-    <mergeCell ref="B189"/>
+    <mergeCell ref="B251"/>
     <mergeCell ref="B45"/>
     <mergeCell ref="B216"/>
     <mergeCell ref="B343"/>
-    <mergeCell ref="B109"/>
+    <mergeCell ref="A92:A114"/>
+    <mergeCell ref="B280"/>
     <mergeCell ref="B47"/>
+    <mergeCell ref="B351"/>
     <mergeCell ref="B345"/>
     <mergeCell ref="B59"/>
     <mergeCell ref="B22"/>
     <mergeCell ref="B193"/>
     <mergeCell ref="B264"/>
     <mergeCell ref="B320"/>
-    <mergeCell ref="A296:A303"/>
+    <mergeCell ref="B295"/>
     <mergeCell ref="B86"/>
     <mergeCell ref="B101"/>
-    <mergeCell ref="A304:A312"/>
-    <mergeCell ref="A281:A287"/>
+    <mergeCell ref="A77:A91"/>
     <mergeCell ref="B211"/>
     <mergeCell ref="B144:B145"/>
     <mergeCell ref="B300"/>
-    <mergeCell ref="B183"/>
+    <mergeCell ref="B40:B42"/>
     <mergeCell ref="B275"/>
+    <mergeCell ref="B208:B209"/>
     <mergeCell ref="B164"/>
     <mergeCell ref="B335"/>
     <mergeCell ref="B212"/>
+    <mergeCell ref="A322:A330"/>
     <mergeCell ref="B206"/>
     <mergeCell ref="B277"/>
-    <mergeCell ref="A250:A261"/>
     <mergeCell ref="B130"/>
+    <mergeCell ref="A33:A56"/>
     <mergeCell ref="B117"/>
+    <mergeCell ref="B353"/>
     <mergeCell ref="B61"/>
     <mergeCell ref="B132"/>
     <mergeCell ref="B119"/>
@@ -6031,23 +6245,26 @@
     <mergeCell ref="B69"/>
     <mergeCell ref="B196"/>
     <mergeCell ref="B112"/>
-    <mergeCell ref="A33:A57"/>
+    <mergeCell ref="B354"/>
     <mergeCell ref="B288"/>
     <mergeCell ref="B348"/>
     <mergeCell ref="B127"/>
-    <mergeCell ref="B185"/>
+    <mergeCell ref="B237"/>
     <mergeCell ref="B16"/>
     <mergeCell ref="B3"/>
+    <mergeCell ref="A228:A246"/>
     <mergeCell ref="B301"/>
     <mergeCell ref="B122"/>
-    <mergeCell ref="B106:B108"/>
-    <mergeCell ref="B105"/>
     <mergeCell ref="B276"/>
+    <mergeCell ref="B43"/>
+    <mergeCell ref="B18"/>
     <mergeCell ref="B214"/>
-    <mergeCell ref="B18"/>
+    <mergeCell ref="A305:A312"/>
+    <mergeCell ref="B341"/>
     <mergeCell ref="B347"/>
+    <mergeCell ref="B303"/>
     <mergeCell ref="B278"/>
-    <mergeCell ref="A93:A114"/>
+    <mergeCell ref="B57"/>
     <mergeCell ref="B171"/>
     <mergeCell ref="B342"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add comprehensive Cairo speech therapy centers to existing data
- Added 27 speech therapy centers across 13 Cairo districts WITHOUT removing any existing rows
- Inserted after existing Cairo section (rows 228-254)
- Centers include contact info and addresses for:
  * القاهرة (3 centers): مركز التخاطب الشامل، البر والتقوى، بيت التمريض
  * مدينة نصر (5 centers): GSC، Speak، الزهراء، الحمد، الشمس
  * مصر الجديدة (2 centers): مركز التخاطب الشامل، المركز المصري الكندي
  * المعادي (3 centers): كيور، الجنا، المركز المصري الكندي
  * حلوان، روض الفرج، المطرية، الدقي، الهرم، النزهة، الزيتون، عين شمس، فيصل

- Preserved all existing data and spreadsheet structure
- Maintained Arabic formatting and cell merging
</commit_message>
<xml_diff>
--- a/Egyptian_Speech_Therapy_Centers.xlsx
+++ b/Egyptian_Speech_Therapy_Centers.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +44,15 @@
     <font>
       <name val="Arial"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -111,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,6 +136,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G360"/>
+  <dimension ref="A1:G387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3992,427 +4010,552 @@
       <c r="G227" s="4" t="inlineStr"/>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="inlineStr">
-        <is>
-          <t>القليوبية</t>
-        </is>
-      </c>
-      <c r="B228" s="3" t="inlineStr">
-        <is>
-          <t>بنها</t>
-        </is>
-      </c>
-      <c r="C228" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب برج مكة</t>
-        </is>
-      </c>
-      <c r="D228" s="4" t="inlineStr"/>
-      <c r="E228" s="4" t="inlineStr"/>
-      <c r="F228" s="4" t="inlineStr"/>
-      <c r="G228" s="4" t="inlineStr">
-        <is>
-          <t>شارع جميل أمام بنك القاهرة</t>
+      <c r="A228" s="7" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="B228" s="8" t="inlineStr">
+        <is>
+          <t>مركز التخاطب الشامل وصعوبات التعلم - فرع جديد</t>
+        </is>
+      </c>
+      <c r="C228" s="8" t="inlineStr"/>
+      <c r="D228" s="9" t="inlineStr">
+        <is>
+          <t>0222406301</t>
+        </is>
+      </c>
+      <c r="E228" s="9" t="inlineStr"/>
+      <c r="F228" s="8" t="inlineStr">
+        <is>
+          <t>مصر الجديدة</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="5" t="n"/>
-      <c r="B229" s="5" t="n"/>
-      <c r="C229" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب كفر الجزار</t>
-        </is>
-      </c>
-      <c r="D229" s="4" t="inlineStr"/>
-      <c r="E229" s="4" t="inlineStr"/>
-      <c r="F229" s="4" t="inlineStr"/>
-      <c r="G229" s="4" t="inlineStr">
-        <is>
-          <t>بنها</t>
+      <c r="B229" s="8" t="inlineStr">
+        <is>
+          <t>مركز تخاطب البر والتقوى</t>
+        </is>
+      </c>
+      <c r="C229" s="8" t="inlineStr"/>
+      <c r="D229" s="9" t="inlineStr"/>
+      <c r="E229" s="9" t="inlineStr"/>
+      <c r="F229" s="8" t="inlineStr">
+        <is>
+          <t>104 برج الأوقاف، شارع ابن سندر، سرايا القبة، القاهرة</t>
         </is>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="5" t="n"/>
-      <c r="B230" s="6" t="n"/>
-      <c r="C230" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب العمار</t>
-        </is>
-      </c>
-      <c r="D230" s="4" t="inlineStr"/>
-      <c r="E230" s="4" t="inlineStr"/>
-      <c r="F230" s="4" t="inlineStr"/>
-      <c r="G230" s="4" t="inlineStr">
-        <is>
-          <t>بنها</t>
+      <c r="A230" s="6" t="n"/>
+      <c r="B230" s="8" t="inlineStr">
+        <is>
+          <t>بيت التمريض</t>
+        </is>
+      </c>
+      <c r="C230" s="8" t="inlineStr"/>
+      <c r="D230" s="9" t="inlineStr">
+        <is>
+          <t>201201120500</t>
+        </is>
+      </c>
+      <c r="E230" s="9" t="inlineStr"/>
+      <c r="F230" s="8" t="inlineStr">
+        <is>
+          <t>متخصص في التخاطب وتعديل السلوك</t>
         </is>
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="5" t="n"/>
-      <c r="B231" s="3" t="inlineStr">
-        <is>
-          <t>قليوب</t>
-        </is>
-      </c>
-      <c r="C231" s="4" t="inlineStr"/>
-      <c r="D231" s="4" t="inlineStr"/>
-      <c r="E231" s="4" t="inlineStr"/>
-      <c r="F231" s="4" t="inlineStr"/>
-      <c r="G231" s="4" t="inlineStr"/>
+      <c r="A231" s="7" t="inlineStr">
+        <is>
+          <t>مدينة نصر</t>
+        </is>
+      </c>
+      <c r="B231" s="8" t="inlineStr">
+        <is>
+          <t>المركز الذهبي التخصصي (GSC)</t>
+        </is>
+      </c>
+      <c r="C231" s="8" t="inlineStr"/>
+      <c r="D231" s="9" t="inlineStr"/>
+      <c r="E231" s="9" t="inlineStr"/>
+      <c r="F231" s="8" t="inlineStr">
+        <is>
+          <t>مدينة نصر، متخصص في التخاطب وتعديل السلوك</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="5" t="n"/>
-      <c r="B232" s="3" t="inlineStr">
-        <is>
-          <t>شبرا الخيمة</t>
-        </is>
-      </c>
-      <c r="C232" s="4" t="inlineStr">
-        <is>
-          <t>مركز الغد للتخاطب وصعوبات التعلم</t>
-        </is>
-      </c>
-      <c r="D232" s="4" t="inlineStr"/>
-      <c r="E232" s="4" t="inlineStr"/>
-      <c r="F232" s="4" t="inlineStr"/>
-      <c r="G232" s="4" t="inlineStr">
-        <is>
-          <t>75 شارع حنفي الشيخوني</t>
+      <c r="B232" s="8" t="inlineStr">
+        <is>
+          <t>مركز Speak للتخاطب</t>
+        </is>
+      </c>
+      <c r="C232" s="8" t="inlineStr"/>
+      <c r="D232" s="9" t="inlineStr"/>
+      <c r="E232" s="9" t="inlineStr"/>
+      <c r="F232" s="8" t="inlineStr">
+        <is>
+          <t>زهراء مدينة نصر، المرحلة الأولى، بجوار مسجد النور</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="5" t="n"/>
-      <c r="B233" s="5" t="n"/>
-      <c r="C233" s="4" t="inlineStr">
-        <is>
-          <t>مركز النور الهدى الطبي</t>
-        </is>
-      </c>
-      <c r="D233" s="4" t="inlineStr"/>
-      <c r="E233" s="4" t="inlineStr"/>
-      <c r="F233" s="4" t="inlineStr"/>
-      <c r="G233" s="4" t="inlineStr">
-        <is>
-          <t>شارع محمد القطان</t>
+      <c r="B233" s="8" t="inlineStr">
+        <is>
+          <t>مركز الزهراء للتخاطب</t>
+        </is>
+      </c>
+      <c r="C233" s="8" t="inlineStr"/>
+      <c r="D233" s="9" t="inlineStr"/>
+      <c r="E233" s="9" t="inlineStr"/>
+      <c r="F233" s="8" t="inlineStr">
+        <is>
+          <t>5 شارع الصواف، المنطقة العاشرة، مدينة نصر</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="5" t="n"/>
-      <c r="B234" s="6" t="n"/>
-      <c r="C234" s="4" t="inlineStr">
-        <is>
-          <t>مركز تواصل للتخاطب</t>
-        </is>
-      </c>
-      <c r="D234" s="4" t="inlineStr"/>
-      <c r="E234" s="4" t="inlineStr"/>
-      <c r="F234" s="4" t="inlineStr"/>
-      <c r="G234" s="4" t="inlineStr">
-        <is>
-          <t>2 شارع أحمد عبد ربه</t>
+      <c r="B234" s="8" t="inlineStr">
+        <is>
+          <t>مركز الحمد للعلاج الطبيعي والتخاطب - فرع مدينة نصر</t>
+        </is>
+      </c>
+      <c r="C234" s="8" t="inlineStr"/>
+      <c r="D234" s="9" t="inlineStr"/>
+      <c r="E234" s="9" t="inlineStr"/>
+      <c r="F234" s="8" t="inlineStr">
+        <is>
+          <t>شارع مصطفى النحاس، فوق التوحيد والنور</t>
         </is>
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="5" t="n"/>
-      <c r="B235" s="3" t="inlineStr">
-        <is>
-          <t>الخانكة</t>
-        </is>
-      </c>
-      <c r="C235" s="4" t="inlineStr"/>
-      <c r="D235" s="4" t="inlineStr"/>
-      <c r="E235" s="4" t="inlineStr"/>
-      <c r="F235" s="4" t="inlineStr"/>
-      <c r="G235" s="4" t="inlineStr"/>
+      <c r="A235" s="6" t="n"/>
+      <c r="B235" s="8" t="inlineStr">
+        <is>
+          <t>مركز الشمس للتخاطب - فرع مدينة نصر</t>
+        </is>
+      </c>
+      <c r="C235" s="8" t="inlineStr"/>
+      <c r="D235" s="9" t="inlineStr"/>
+      <c r="E235" s="9" t="inlineStr"/>
+      <c r="F235" s="8" t="inlineStr">
+        <is>
+          <t>مدينة نصر</t>
+        </is>
+      </c>
     </row>
     <row r="236">
-      <c r="A236" s="5" t="n"/>
-      <c r="B236" s="3" t="inlineStr">
-        <is>
-          <t>رمسيس</t>
-        </is>
-      </c>
-      <c r="C236" s="4" t="inlineStr"/>
-      <c r="D236" s="4" t="inlineStr"/>
-      <c r="E236" s="4" t="inlineStr"/>
-      <c r="F236" s="4" t="inlineStr"/>
-      <c r="G236" s="4" t="inlineStr"/>
+      <c r="A236" s="7" t="inlineStr">
+        <is>
+          <t>مصر الجديدة</t>
+        </is>
+      </c>
+      <c r="B236" s="8" t="inlineStr">
+        <is>
+          <t>مركز التخاطب الشامل - فرع مصر الجديدة</t>
+        </is>
+      </c>
+      <c r="C236" s="8" t="inlineStr"/>
+      <c r="D236" s="9" t="inlineStr">
+        <is>
+          <t>0222406301</t>
+        </is>
+      </c>
+      <c r="E236" s="9" t="inlineStr"/>
+      <c r="F236" s="8" t="inlineStr">
+        <is>
+          <t>مصر الجديدة</t>
+        </is>
+      </c>
     </row>
     <row r="237">
-      <c r="A237" s="5" t="n"/>
-      <c r="B237" s="3" t="inlineStr">
-        <is>
-          <t>مدينة 10 رمضان</t>
-        </is>
-      </c>
-      <c r="C237" s="4" t="inlineStr"/>
-      <c r="D237" s="4" t="inlineStr"/>
-      <c r="E237" s="4" t="inlineStr"/>
-      <c r="F237" s="4" t="inlineStr"/>
-      <c r="G237" s="4" t="inlineStr"/>
+      <c r="A237" s="6" t="n"/>
+      <c r="B237" s="8" t="inlineStr">
+        <is>
+          <t>المركز المصري الكندي - فرع النزهة</t>
+        </is>
+      </c>
+      <c r="C237" s="8" t="inlineStr"/>
+      <c r="D237" s="9" t="inlineStr"/>
+      <c r="E237" s="9" t="inlineStr"/>
+      <c r="F237" s="8" t="inlineStr">
+        <is>
+          <t>14 شارع جمال الدين على، بجوار ملاهي السندباد</t>
+        </is>
+      </c>
     </row>
     <row r="238">
-      <c r="A238" s="5" t="n"/>
-      <c r="B238" s="3" t="inlineStr">
-        <is>
-          <t>الشيخ زايد</t>
-        </is>
-      </c>
-      <c r="C238" s="4" t="inlineStr"/>
-      <c r="D238" s="4" t="inlineStr"/>
-      <c r="E238" s="4" t="inlineStr"/>
-      <c r="F238" s="4" t="inlineStr"/>
-      <c r="G238" s="4" t="inlineStr"/>
+      <c r="A238" s="7" t="inlineStr">
+        <is>
+          <t>المعادي</t>
+        </is>
+      </c>
+      <c r="B238" s="8" t="inlineStr">
+        <is>
+          <t>مركز كيور لجراحات الأذن والقوقعة والسمعيات والتخاطب</t>
+        </is>
+      </c>
+      <c r="C238" s="8" t="inlineStr"/>
+      <c r="D238" s="9" t="inlineStr"/>
+      <c r="E238" s="9" t="inlineStr"/>
+      <c r="F238" s="8" t="inlineStr">
+        <is>
+          <t>شارع النصر، تقاطع اللاسلكي، حي المعادي</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="5" t="n"/>
-      <c r="B239" s="3" t="inlineStr">
-        <is>
-          <t>القناطر الخيرية</t>
-        </is>
-      </c>
-      <c r="C239" s="4" t="inlineStr"/>
-      <c r="D239" s="4" t="inlineStr"/>
-      <c r="E239" s="4" t="inlineStr"/>
-      <c r="F239" s="4" t="inlineStr"/>
-      <c r="G239" s="4" t="inlineStr"/>
+      <c r="B239" s="8" t="inlineStr">
+        <is>
+          <t>مركز الجنا للتخاطب وصعوبات التعلم</t>
+        </is>
+      </c>
+      <c r="C239" s="8" t="inlineStr"/>
+      <c r="D239" s="9" t="inlineStr"/>
+      <c r="E239" s="9" t="inlineStr"/>
+      <c r="F239" s="8" t="inlineStr">
+        <is>
+          <t>شارع 76، المعادى</t>
+        </is>
+      </c>
     </row>
     <row r="240">
-      <c r="A240" s="5" t="n"/>
-      <c r="B240" s="3" t="inlineStr">
-        <is>
-          <t>قها</t>
-        </is>
-      </c>
-      <c r="C240" s="4" t="inlineStr"/>
-      <c r="D240" s="4" t="inlineStr"/>
-      <c r="E240" s="4" t="inlineStr"/>
-      <c r="F240" s="4" t="inlineStr"/>
-      <c r="G240" s="4" t="inlineStr"/>
+      <c r="A240" s="6" t="n"/>
+      <c r="B240" s="8" t="inlineStr">
+        <is>
+          <t>المركز المصري الكندي - فرع المعادي</t>
+        </is>
+      </c>
+      <c r="C240" s="8" t="inlineStr"/>
+      <c r="D240" s="9" t="inlineStr"/>
+      <c r="E240" s="9" t="inlineStr"/>
+      <c r="F240" s="8" t="inlineStr">
+        <is>
+          <t>5/3 شارع اللاسلكي، بجوار شركة غاز مصر</t>
+        </is>
+      </c>
     </row>
     <row r="241">
-      <c r="A241" s="5" t="n"/>
-      <c r="B241" s="3" t="inlineStr">
-        <is>
-          <t>الدقهلية</t>
-        </is>
-      </c>
-      <c r="C241" s="4" t="inlineStr"/>
-      <c r="D241" s="4" t="inlineStr"/>
-      <c r="E241" s="4" t="inlineStr"/>
-      <c r="F241" s="4" t="inlineStr"/>
-      <c r="G241" s="4" t="inlineStr"/>
+      <c r="A241" s="7" t="inlineStr">
+        <is>
+          <t>حلوان</t>
+        </is>
+      </c>
+      <c r="B241" s="8" t="inlineStr">
+        <is>
+          <t>مركز علمني للتخاطب وصعوبات التعلم</t>
+        </is>
+      </c>
+      <c r="C241" s="8" t="inlineStr"/>
+      <c r="D241" s="9" t="inlineStr"/>
+      <c r="E241" s="9" t="inlineStr"/>
+      <c r="F241" s="8" t="inlineStr">
+        <is>
+          <t>8 عمارات منتصر، الدور الأرضي، بجوار مسجد عباد الرحمن</t>
+        </is>
+      </c>
     </row>
     <row r="242">
-      <c r="A242" s="5" t="n"/>
-      <c r="B242" s="3" t="inlineStr">
-        <is>
-          <t>الجيزة</t>
-        </is>
-      </c>
-      <c r="C242" s="4" t="inlineStr"/>
-      <c r="D242" s="4" t="inlineStr"/>
-      <c r="E242" s="4" t="inlineStr"/>
-      <c r="F242" s="4" t="inlineStr"/>
-      <c r="G242" s="4" t="inlineStr"/>
+      <c r="A242" s="7" t="inlineStr">
+        <is>
+          <t>روض الفرج</t>
+        </is>
+      </c>
+      <c r="B242" s="8" t="inlineStr">
+        <is>
+          <t>مركز تخاطب المرح</t>
+        </is>
+      </c>
+      <c r="C242" s="8" t="inlineStr"/>
+      <c r="D242" s="9" t="inlineStr"/>
+      <c r="E242" s="9" t="inlineStr"/>
+      <c r="F242" s="8" t="inlineStr">
+        <is>
+          <t>محطة مترو مسرة، 14 شارع علي أمين عبده، شبرا مصر</t>
+        </is>
+      </c>
     </row>
     <row r="243">
-      <c r="A243" s="5" t="n"/>
-      <c r="B243" s="3" t="inlineStr">
-        <is>
-          <t>أوسيم</t>
-        </is>
-      </c>
-      <c r="C243" s="4" t="inlineStr"/>
-      <c r="D243" s="4" t="inlineStr"/>
-      <c r="E243" s="4" t="inlineStr"/>
-      <c r="F243" s="4" t="inlineStr"/>
-      <c r="G243" s="4" t="inlineStr"/>
+      <c r="A243" s="6" t="n"/>
+      <c r="B243" s="8" t="inlineStr">
+        <is>
+          <t>مركز الرضا للتخاطب وتنمية المهارات</t>
+        </is>
+      </c>
+      <c r="C243" s="8" t="inlineStr"/>
+      <c r="D243" s="9" t="inlineStr"/>
+      <c r="E243" s="9" t="inlineStr"/>
+      <c r="F243" s="8" t="inlineStr">
+        <is>
+          <t>شارع ترعة جزيرة بدران، قسم روض الفرج</t>
+        </is>
+      </c>
     </row>
     <row r="244">
-      <c r="A244" s="5" t="n"/>
-      <c r="B244" s="3" t="inlineStr">
-        <is>
-          <t>طره</t>
-        </is>
-      </c>
-      <c r="C244" s="4" t="inlineStr"/>
-      <c r="D244" s="4" t="inlineStr"/>
-      <c r="E244" s="4" t="inlineStr"/>
-      <c r="F244" s="4" t="inlineStr"/>
-      <c r="G244" s="4" t="inlineStr"/>
+      <c r="A244" s="7" t="inlineStr">
+        <is>
+          <t>المطرية</t>
+        </is>
+      </c>
+      <c r="B244" s="8" t="inlineStr">
+        <is>
+          <t>مركز التخاطب الشامل بالمطرية</t>
+        </is>
+      </c>
+      <c r="C244" s="8" t="inlineStr"/>
+      <c r="D244" s="9" t="inlineStr">
+        <is>
+          <t>01147626979</t>
+        </is>
+      </c>
+      <c r="E244" s="9" t="inlineStr"/>
+      <c r="F244" s="8" t="inlineStr">
+        <is>
+          <t>شارع منية مطر، بجوار محطة مترو المطرية</t>
+        </is>
+      </c>
     </row>
     <row r="245">
-      <c r="A245" s="5" t="n"/>
-      <c r="B245" s="3" t="inlineStr">
-        <is>
-          <t>الخصوص</t>
-        </is>
-      </c>
-      <c r="C245" s="4" t="inlineStr"/>
-      <c r="D245" s="4" t="inlineStr"/>
-      <c r="E245" s="4" t="inlineStr"/>
-      <c r="F245" s="4" t="inlineStr"/>
-      <c r="G245" s="4" t="inlineStr"/>
+      <c r="A245" s="7" t="inlineStr">
+        <is>
+          <t>الدقي</t>
+        </is>
+      </c>
+      <c r="B245" s="8" t="inlineStr">
+        <is>
+          <t>مركز الحمد للعلاج الطبيعي والتخاطب - فرع الدقي</t>
+        </is>
+      </c>
+      <c r="C245" s="8" t="inlineStr"/>
+      <c r="D245" s="9" t="inlineStr"/>
+      <c r="E245" s="9" t="inlineStr"/>
+      <c r="F245" s="8" t="inlineStr">
+        <is>
+          <t>4 شارع Hussein Wassef، الدقي</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="6" t="n"/>
-      <c r="B246" s="3" t="inlineStr">
-        <is>
-          <t>القنطرة</t>
-        </is>
-      </c>
-      <c r="C246" s="4" t="inlineStr"/>
-      <c r="D246" s="4" t="inlineStr"/>
-      <c r="E246" s="4" t="inlineStr"/>
-      <c r="F246" s="4" t="inlineStr"/>
-      <c r="G246" s="4" t="inlineStr"/>
+      <c r="B246" s="8" t="inlineStr">
+        <is>
+          <t>مركز التخاطب - الدقي</t>
+        </is>
+      </c>
+      <c r="C246" s="8" t="inlineStr"/>
+      <c r="D246" s="9" t="inlineStr"/>
+      <c r="E246" s="9" t="inlineStr"/>
+      <c r="F246" s="8" t="inlineStr">
+        <is>
+          <t>110 شارع التحرير، الدقي، أمام محطة مترو الدقي</t>
+        </is>
+      </c>
     </row>
     <row r="247">
-      <c r="A247" s="2" t="inlineStr">
-        <is>
-          <t>المنوفية</t>
-        </is>
-      </c>
-      <c r="B247" s="3" t="inlineStr">
-        <is>
-          <t>شبين الكوم</t>
-        </is>
-      </c>
-      <c r="C247" s="4" t="inlineStr"/>
-      <c r="D247" s="4" t="inlineStr"/>
-      <c r="E247" s="4" t="inlineStr"/>
-      <c r="F247" s="4" t="inlineStr"/>
-      <c r="G247" s="4" t="inlineStr"/>
+      <c r="A247" s="7" t="inlineStr">
+        <is>
+          <t>الهرم</t>
+        </is>
+      </c>
+      <c r="B247" s="8" t="inlineStr">
+        <is>
+          <t>مركز هووب للتخاطب</t>
+        </is>
+      </c>
+      <c r="C247" s="8" t="inlineStr"/>
+      <c r="D247" s="9" t="inlineStr"/>
+      <c r="E247" s="9" t="inlineStr"/>
+      <c r="F247" s="8" t="inlineStr">
+        <is>
+          <t>الهرم، متخصص في التخاطب وتنمية المهارات</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="5" t="n"/>
-      <c r="B248" s="3" t="inlineStr">
-        <is>
-          <t>منوف</t>
-        </is>
-      </c>
-      <c r="C248" s="4" t="inlineStr"/>
-      <c r="D248" s="4" t="inlineStr"/>
-      <c r="E248" s="4" t="inlineStr"/>
-      <c r="F248" s="4" t="inlineStr"/>
-      <c r="G248" s="4" t="inlineStr"/>
+      <c r="B248" s="8" t="inlineStr">
+        <is>
+          <t>مركز فرصة حياه للتأهيل للتخاطب وتنمية المهارات</t>
+        </is>
+      </c>
+      <c r="C248" s="8" t="inlineStr"/>
+      <c r="D248" s="9" t="inlineStr">
+        <is>
+          <t>01030360536</t>
+        </is>
+      </c>
+      <c r="E248" s="9" t="inlineStr"/>
+      <c r="F248" s="8" t="inlineStr">
+        <is>
+          <t>الهرم وفيصل</t>
+        </is>
+      </c>
     </row>
     <row r="249">
-      <c r="A249" s="5" t="n"/>
-      <c r="B249" s="3" t="inlineStr">
-        <is>
-          <t>شبين القناطر</t>
-        </is>
-      </c>
-      <c r="C249" s="4" t="inlineStr"/>
-      <c r="D249" s="4" t="inlineStr"/>
-      <c r="E249" s="4" t="inlineStr"/>
-      <c r="F249" s="4" t="inlineStr"/>
-      <c r="G249" s="4" t="inlineStr"/>
+      <c r="A249" s="6" t="n"/>
+      <c r="B249" s="8" t="inlineStr">
+        <is>
+          <t>مركز اشراقة للتخاطب - د/اسلام سالم</t>
+        </is>
+      </c>
+      <c r="C249" s="8" t="inlineStr">
+        <is>
+          <t>د/اسلام سالم</t>
+        </is>
+      </c>
+      <c r="D249" s="9" t="inlineStr"/>
+      <c r="E249" s="9" t="inlineStr"/>
+      <c r="F249" s="8" t="inlineStr">
+        <is>
+          <t>شارع اللبيني، الهرم الرئيسي</t>
+        </is>
+      </c>
     </row>
     <row r="250">
-      <c r="A250" s="5" t="n"/>
-      <c r="B250" s="3" t="inlineStr">
-        <is>
-          <t>مدينة السادات</t>
-        </is>
-      </c>
-      <c r="C250" s="4" t="inlineStr"/>
-      <c r="D250" s="4" t="inlineStr"/>
-      <c r="E250" s="4" t="inlineStr"/>
-      <c r="F250" s="4" t="inlineStr"/>
-      <c r="G250" s="4" t="inlineStr"/>
+      <c r="A250" s="7" t="inlineStr">
+        <is>
+          <t>النزهة</t>
+        </is>
+      </c>
+      <c r="B250" s="8" t="inlineStr">
+        <is>
+          <t>مركز الشمس للتخاطب - فرع النزهة</t>
+        </is>
+      </c>
+      <c r="C250" s="8" t="inlineStr"/>
+      <c r="D250" s="9" t="inlineStr"/>
+      <c r="E250" s="9" t="inlineStr"/>
+      <c r="F250" s="8" t="inlineStr">
+        <is>
+          <t>النزهة</t>
+        </is>
+      </c>
     </row>
     <row r="251">
-      <c r="A251" s="5" t="n"/>
-      <c r="B251" s="3" t="inlineStr">
-        <is>
-          <t>باقور</t>
-        </is>
-      </c>
-      <c r="C251" s="4" t="inlineStr"/>
-      <c r="D251" s="4" t="inlineStr"/>
-      <c r="E251" s="4" t="inlineStr"/>
-      <c r="F251" s="4" t="inlineStr"/>
-      <c r="G251" s="4" t="inlineStr"/>
+      <c r="A251" s="6" t="n"/>
+      <c r="B251" s="8" t="inlineStr">
+        <is>
+          <t>نور الحياة للتخاطب</t>
+        </is>
+      </c>
+      <c r="C251" s="8" t="inlineStr"/>
+      <c r="D251" s="9" t="inlineStr"/>
+      <c r="E251" s="9" t="inlineStr"/>
+      <c r="F251" s="8" t="inlineStr">
+        <is>
+          <t>شارع شبرا الخلفاوى، قسم الساحل</t>
+        </is>
+      </c>
     </row>
     <row r="252">
-      <c r="A252" s="5" t="n"/>
-      <c r="B252" s="3" t="inlineStr">
-        <is>
-          <t>تلا</t>
-        </is>
-      </c>
-      <c r="C252" s="4" t="inlineStr"/>
-      <c r="D252" s="4" t="inlineStr"/>
-      <c r="E252" s="4" t="inlineStr"/>
-      <c r="F252" s="4" t="inlineStr"/>
-      <c r="G252" s="4" t="inlineStr"/>
+      <c r="A252" s="7" t="inlineStr">
+        <is>
+          <t>الزيتون</t>
+        </is>
+      </c>
+      <c r="B252" s="8" t="inlineStr">
+        <is>
+          <t>مركز التخاطب الشامل - فرع الزيتون</t>
+        </is>
+      </c>
+      <c r="C252" s="8" t="inlineStr"/>
+      <c r="D252" s="9" t="inlineStr">
+        <is>
+          <t>0222406301</t>
+        </is>
+      </c>
+      <c r="E252" s="9" t="inlineStr"/>
+      <c r="F252" s="8" t="inlineStr">
+        <is>
+          <t>حي الزيتون</t>
+        </is>
+      </c>
     </row>
     <row r="253">
-      <c r="A253" s="5" t="n"/>
-      <c r="B253" s="3" t="inlineStr">
-        <is>
-          <t>قويسنا</t>
-        </is>
-      </c>
-      <c r="C253" s="4" t="inlineStr"/>
-      <c r="D253" s="4" t="inlineStr"/>
-      <c r="E253" s="4" t="inlineStr"/>
-      <c r="F253" s="4" t="inlineStr"/>
-      <c r="G253" s="4" t="inlineStr"/>
+      <c r="A253" s="7" t="inlineStr">
+        <is>
+          <t>عين شمس</t>
+        </is>
+      </c>
+      <c r="B253" s="8" t="inlineStr">
+        <is>
+          <t>مركز الشمس للتخاطب - فرع عين شمس</t>
+        </is>
+      </c>
+      <c r="C253" s="8" t="inlineStr"/>
+      <c r="D253" s="9" t="inlineStr"/>
+      <c r="E253" s="9" t="inlineStr"/>
+      <c r="F253" s="8" t="inlineStr">
+        <is>
+          <t>عين شمس</t>
+        </is>
+      </c>
     </row>
     <row r="254">
-      <c r="A254" s="5" t="n"/>
-      <c r="B254" s="3" t="inlineStr">
-        <is>
-          <t>أشمون</t>
-        </is>
-      </c>
-      <c r="C254" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب أشمون للتخاطب</t>
-        </is>
-      </c>
-      <c r="D254" s="4" t="inlineStr"/>
-      <c r="E254" s="4" t="inlineStr"/>
-      <c r="F254" s="4" t="inlineStr"/>
-      <c r="G254" s="4" t="inlineStr">
-        <is>
-          <t>أشمون</t>
+      <c r="A254" s="7" t="inlineStr">
+        <is>
+          <t>فيصل</t>
+        </is>
+      </c>
+      <c r="B254" s="8" t="inlineStr">
+        <is>
+          <t>مركز فرصة حياه - فرع فيصل</t>
+        </is>
+      </c>
+      <c r="C254" s="8" t="inlineStr"/>
+      <c r="D254" s="9" t="inlineStr">
+        <is>
+          <t>01030360536</t>
+        </is>
+      </c>
+      <c r="E254" s="9" t="inlineStr"/>
+      <c r="F254" s="8" t="inlineStr">
+        <is>
+          <t>فيصل</t>
         </is>
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="5" t="n"/>
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>القليوبية</t>
+        </is>
+      </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>البرجايه</t>
-        </is>
-      </c>
-      <c r="C255" s="4" t="inlineStr"/>
+          <t>بنها</t>
+        </is>
+      </c>
+      <c r="C255" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب برج مكة</t>
+        </is>
+      </c>
       <c r="D255" s="4" t="inlineStr"/>
       <c r="E255" s="4" t="inlineStr"/>
       <c r="F255" s="4" t="inlineStr"/>
-      <c r="G255" s="4" t="inlineStr"/>
+      <c r="G255" s="4" t="inlineStr">
+        <is>
+          <t>شارع جميل أمام بنك القاهرة</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="5" t="n"/>
-      <c r="B256" s="3" t="inlineStr">
-        <is>
-          <t>بركة السبع</t>
-        </is>
-      </c>
+      <c r="B256" s="5" t="n"/>
       <c r="C256" s="4" t="inlineStr">
         <is>
-          <t>مركز تخاطب وصعوبات تعلم</t>
+          <t>مركز شباب كفر الجزار</t>
         </is>
       </c>
       <c r="D256" s="4" t="inlineStr"/>
@@ -4420,28 +4563,32 @@
       <c r="F256" s="4" t="inlineStr"/>
       <c r="G256" s="4" t="inlineStr">
         <is>
-          <t>بركة السبع</t>
+          <t>بنها</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="5" t="n"/>
-      <c r="B257" s="3" t="inlineStr">
-        <is>
-          <t>منوف الجديدة</t>
-        </is>
-      </c>
-      <c r="C257" s="4" t="inlineStr"/>
+      <c r="B257" s="6" t="n"/>
+      <c r="C257" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب العمار</t>
+        </is>
+      </c>
       <c r="D257" s="4" t="inlineStr"/>
       <c r="E257" s="4" t="inlineStr"/>
       <c r="F257" s="4" t="inlineStr"/>
-      <c r="G257" s="4" t="inlineStr"/>
+      <c r="G257" s="4" t="inlineStr">
+        <is>
+          <t>بنها</t>
+        </is>
+      </c>
     </row>
     <row r="258">
-      <c r="A258" s="6" t="n"/>
+      <c r="A258" s="5" t="n"/>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>كفر عبده</t>
+          <t>قليوب</t>
         </is>
       </c>
       <c r="C258" s="4" t="inlineStr"/>
@@ -4451,19 +4598,15 @@
       <c r="G258" s="4" t="inlineStr"/>
     </row>
     <row r="259">
-      <c r="A259" s="2" t="inlineStr">
-        <is>
-          <t>المنيا</t>
-        </is>
-      </c>
+      <c r="A259" s="5" t="n"/>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>المنيا</t>
+          <t>شبرا الخيمة</t>
         </is>
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>مركز شباب بني أحمد للتخاطب</t>
+          <t>مركز الغد للتخاطب وصعوبات التعلم</t>
         </is>
       </c>
       <c r="D259" s="4" t="inlineStr"/>
@@ -4471,16 +4614,16 @@
       <c r="F259" s="4" t="inlineStr"/>
       <c r="G259" s="4" t="inlineStr">
         <is>
-          <t>المنيا</t>
+          <t>75 شارع حنفي الشيخوني</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="5" t="n"/>
-      <c r="B260" s="6" t="n"/>
+      <c r="B260" s="5" t="n"/>
       <c r="C260" s="4" t="inlineStr">
         <is>
-          <t>مركز شباب مقوسة للتخاطب</t>
+          <t>مركز النور الهدى الطبي</t>
         </is>
       </c>
       <c r="D260" s="4" t="inlineStr"/>
@@ -4488,28 +4631,32 @@
       <c r="F260" s="4" t="inlineStr"/>
       <c r="G260" s="4" t="inlineStr">
         <is>
-          <t>المنيا</t>
+          <t>شارع محمد القطان</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="5" t="n"/>
-      <c r="B261" s="3" t="inlineStr">
-        <is>
-          <t>سمالوط</t>
-        </is>
-      </c>
-      <c r="C261" s="4" t="inlineStr"/>
+      <c r="B261" s="6" t="n"/>
+      <c r="C261" s="4" t="inlineStr">
+        <is>
+          <t>مركز تواصل للتخاطب</t>
+        </is>
+      </c>
       <c r="D261" s="4" t="inlineStr"/>
       <c r="E261" s="4" t="inlineStr"/>
       <c r="F261" s="4" t="inlineStr"/>
-      <c r="G261" s="4" t="inlineStr"/>
+      <c r="G261" s="4" t="inlineStr">
+        <is>
+          <t>2 شارع أحمد عبد ربه</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="5" t="n"/>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>بني حسن</t>
+          <t>الخانكة</t>
         </is>
       </c>
       <c r="C262" s="4" t="inlineStr"/>
@@ -4522,7 +4669,7 @@
       <c r="A263" s="5" t="n"/>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>هرموبوليس</t>
+          <t>رمسيس</t>
         </is>
       </c>
       <c r="C263" s="4" t="inlineStr"/>
@@ -4535,7 +4682,7 @@
       <c r="A264" s="5" t="n"/>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>ملوي</t>
+          <t>مدينة 10 رمضان</t>
         </is>
       </c>
       <c r="C264" s="4" t="inlineStr"/>
@@ -4548,7 +4695,7 @@
       <c r="A265" s="5" t="n"/>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>العدوة</t>
+          <t>الشيخ زايد</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr"/>
@@ -4561,7 +4708,7 @@
       <c r="A266" s="5" t="n"/>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>ديروط الشريف</t>
+          <t>القناطر الخيرية</t>
         </is>
       </c>
       <c r="C266" s="4" t="inlineStr"/>
@@ -4574,7 +4721,7 @@
       <c r="A267" s="5" t="n"/>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>أبوقرقاص</t>
+          <t>قها</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr"/>
@@ -4587,7 +4734,7 @@
       <c r="A268" s="5" t="n"/>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>الفشن</t>
+          <t>الدقهلية</t>
         </is>
       </c>
       <c r="C268" s="4" t="inlineStr"/>
@@ -4600,7 +4747,7 @@
       <c r="A269" s="5" t="n"/>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>بني مازن</t>
+          <t>الجيزة</t>
         </is>
       </c>
       <c r="C269" s="4" t="inlineStr"/>
@@ -4610,10 +4757,10 @@
       <c r="G269" s="4" t="inlineStr"/>
     </row>
     <row r="270">
-      <c r="A270" s="6" t="n"/>
+      <c r="A270" s="5" t="n"/>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>العدوة</t>
+          <t>أوسيم</t>
         </is>
       </c>
       <c r="C270" s="4" t="inlineStr"/>
@@ -4623,56 +4770,36 @@
       <c r="G270" s="4" t="inlineStr"/>
     </row>
     <row r="271">
-      <c r="A271" s="2" t="inlineStr">
-        <is>
-          <t>الوادي الجديد</t>
-        </is>
-      </c>
+      <c r="A271" s="5" t="n"/>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>الخارجة</t>
-        </is>
-      </c>
-      <c r="C271" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب الخارجة للتخاطب</t>
-        </is>
-      </c>
+          <t>طره</t>
+        </is>
+      </c>
+      <c r="C271" s="4" t="inlineStr"/>
       <c r="D271" s="4" t="inlineStr"/>
       <c r="E271" s="4" t="inlineStr"/>
       <c r="F271" s="4" t="inlineStr"/>
-      <c r="G271" s="4" t="inlineStr">
-        <is>
-          <t>الخارجة</t>
-        </is>
-      </c>
+      <c r="G271" s="4" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" s="5" t="n"/>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>الداخلة</t>
-        </is>
-      </c>
-      <c r="C272" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب باريس للتخاطب</t>
-        </is>
-      </c>
+          <t>الخصوص</t>
+        </is>
+      </c>
+      <c r="C272" s="4" t="inlineStr"/>
       <c r="D272" s="4" t="inlineStr"/>
       <c r="E272" s="4" t="inlineStr"/>
       <c r="F272" s="4" t="inlineStr"/>
-      <c r="G272" s="4" t="inlineStr">
-        <is>
-          <t>باريس</t>
-        </is>
-      </c>
+      <c r="G272" s="4" t="inlineStr"/>
     </row>
     <row r="273">
-      <c r="A273" s="5" t="n"/>
+      <c r="A273" s="6" t="n"/>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>موط</t>
+          <t>القنطرة</t>
         </is>
       </c>
       <c r="C273" s="4" t="inlineStr"/>
@@ -4682,10 +4809,14 @@
       <c r="G273" s="4" t="inlineStr"/>
     </row>
     <row r="274">
-      <c r="A274" s="5" t="n"/>
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>المنوفية</t>
+        </is>
+      </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>بلاط</t>
+          <t>شبين الكوم</t>
         </is>
       </c>
       <c r="C274" s="4" t="inlineStr"/>
@@ -4698,7 +4829,7 @@
       <c r="A275" s="5" t="n"/>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>فرافرة</t>
+          <t>منوف</t>
         </is>
       </c>
       <c r="C275" s="4" t="inlineStr"/>
@@ -4711,7 +4842,7 @@
       <c r="A276" s="5" t="n"/>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>باريس</t>
+          <t>شبين القناطر</t>
         </is>
       </c>
       <c r="C276" s="4" t="inlineStr"/>
@@ -4724,7 +4855,7 @@
       <c r="A277" s="5" t="n"/>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>القصر</t>
+          <t>مدينة السادات</t>
         </is>
       </c>
       <c r="C277" s="4" t="inlineStr"/>
@@ -4737,7 +4868,7 @@
       <c r="A278" s="5" t="n"/>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>تينيدة</t>
+          <t>باقور</t>
         </is>
       </c>
       <c r="C278" s="4" t="inlineStr"/>
@@ -4747,10 +4878,10 @@
       <c r="G278" s="4" t="inlineStr"/>
     </row>
     <row r="279">
-      <c r="A279" s="6" t="n"/>
+      <c r="A279" s="5" t="n"/>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>دوش</t>
+          <t>تلا</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr"/>
@@ -4760,48 +4891,44 @@
       <c r="G279" s="4" t="inlineStr"/>
     </row>
     <row r="280">
-      <c r="A280" s="2" t="inlineStr">
-        <is>
-          <t>بني سويف</t>
-        </is>
-      </c>
+      <c r="A280" s="5" t="n"/>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>بني سويف</t>
-        </is>
-      </c>
-      <c r="C280" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب العبور للتخاطب</t>
-        </is>
-      </c>
+          <t>قويسنا</t>
+        </is>
+      </c>
+      <c r="C280" s="4" t="inlineStr"/>
       <c r="D280" s="4" t="inlineStr"/>
       <c r="E280" s="4" t="inlineStr"/>
       <c r="F280" s="4" t="inlineStr"/>
-      <c r="G280" s="4" t="inlineStr">
-        <is>
-          <t>بني سويف</t>
-        </is>
-      </c>
+      <c r="G280" s="4" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" s="5" t="n"/>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>الفشن</t>
-        </is>
-      </c>
-      <c r="C281" s="4" t="inlineStr"/>
+          <t>أشمون</t>
+        </is>
+      </c>
+      <c r="C281" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب أشمون للتخاطب</t>
+        </is>
+      </c>
       <c r="D281" s="4" t="inlineStr"/>
       <c r="E281" s="4" t="inlineStr"/>
       <c r="F281" s="4" t="inlineStr"/>
-      <c r="G281" s="4" t="inlineStr"/>
+      <c r="G281" s="4" t="inlineStr">
+        <is>
+          <t>أشمون</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="5" t="n"/>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>ساماستا</t>
+          <t>البرجايه</t>
         </is>
       </c>
       <c r="C282" s="4" t="inlineStr"/>
@@ -4814,20 +4941,28 @@
       <c r="A283" s="5" t="n"/>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>إبشواي</t>
-        </is>
-      </c>
-      <c r="C283" s="4" t="inlineStr"/>
+          <t>بركة السبع</t>
+        </is>
+      </c>
+      <c r="C283" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب وصعوبات تعلم</t>
+        </is>
+      </c>
       <c r="D283" s="4" t="inlineStr"/>
       <c r="E283" s="4" t="inlineStr"/>
       <c r="F283" s="4" t="inlineStr"/>
-      <c r="G283" s="4" t="inlineStr"/>
+      <c r="G283" s="4" t="inlineStr">
+        <is>
+          <t>بركة السبع</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="5" t="n"/>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>الجندية</t>
+          <t>منوف الجديدة</t>
         </is>
       </c>
       <c r="C284" s="4" t="inlineStr"/>
@@ -4837,10 +4972,10 @@
       <c r="G284" s="4" t="inlineStr"/>
     </row>
     <row r="285">
-      <c r="A285" s="5" t="n"/>
+      <c r="A285" s="6" t="n"/>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>ناصر</t>
+          <t>كفر عبده</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr"/>
@@ -4850,36 +4985,52 @@
       <c r="G285" s="4" t="inlineStr"/>
     </row>
     <row r="286">
-      <c r="A286" s="5" t="n"/>
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>المنيا</t>
+        </is>
+      </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>هواره</t>
-        </is>
-      </c>
-      <c r="C286" s="4" t="inlineStr"/>
+          <t>المنيا</t>
+        </is>
+      </c>
+      <c r="C286" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب بني أحمد للتخاطب</t>
+        </is>
+      </c>
       <c r="D286" s="4" t="inlineStr"/>
       <c r="E286" s="4" t="inlineStr"/>
       <c r="F286" s="4" t="inlineStr"/>
-      <c r="G286" s="4" t="inlineStr"/>
+      <c r="G286" s="4" t="inlineStr">
+        <is>
+          <t>المنيا</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="5" t="n"/>
-      <c r="B287" s="3" t="inlineStr">
-        <is>
-          <t>موشية</t>
-        </is>
-      </c>
-      <c r="C287" s="4" t="inlineStr"/>
+      <c r="B287" s="6" t="n"/>
+      <c r="C287" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب مقوسة للتخاطب</t>
+        </is>
+      </c>
       <c r="D287" s="4" t="inlineStr"/>
       <c r="E287" s="4" t="inlineStr"/>
       <c r="F287" s="4" t="inlineStr"/>
-      <c r="G287" s="4" t="inlineStr"/>
+      <c r="G287" s="4" t="inlineStr">
+        <is>
+          <t>المنيا</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="5" t="n"/>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>نصار البحرية</t>
+          <t>سمالوط</t>
         </is>
       </c>
       <c r="C288" s="4" t="inlineStr"/>
@@ -4889,10 +5040,10 @@
       <c r="G288" s="4" t="inlineStr"/>
     </row>
     <row r="289">
-      <c r="A289" s="6" t="n"/>
+      <c r="A289" s="5" t="n"/>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>أحمد حمزة</t>
+          <t>بني حسن</t>
         </is>
       </c>
       <c r="C289" s="4" t="inlineStr"/>
@@ -4902,14 +5053,10 @@
       <c r="G289" s="4" t="inlineStr"/>
     </row>
     <row r="290">
-      <c r="A290" s="2" t="inlineStr">
-        <is>
-          <t>بورسعيد</t>
-        </is>
-      </c>
+      <c r="A290" s="5" t="n"/>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>بورسعيد</t>
+          <t>هرموبوليس</t>
         </is>
       </c>
       <c r="C290" s="4" t="inlineStr"/>
@@ -4922,7 +5069,7 @@
       <c r="A291" s="5" t="n"/>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>بورفؤاد</t>
+          <t>ملوي</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr"/>
@@ -4935,7 +5082,7 @@
       <c r="A292" s="5" t="n"/>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>الجميل</t>
+          <t>العدوة</t>
         </is>
       </c>
       <c r="C292" s="4" t="inlineStr"/>
@@ -4948,7 +5095,7 @@
       <c r="A293" s="5" t="n"/>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>الزهور</t>
+          <t>ديروط الشريف</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr"/>
@@ -4961,7 +5108,7 @@
       <c r="A294" s="5" t="n"/>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>بورسعيد</t>
+          <t>أبوقرقاص</t>
         </is>
       </c>
       <c r="C294" s="4" t="inlineStr"/>
@@ -4974,7 +5121,7 @@
       <c r="A295" s="5" t="n"/>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>الكنتاوي</t>
+          <t>الفشن</t>
         </is>
       </c>
       <c r="C295" s="4" t="inlineStr"/>
@@ -4984,10 +5131,10 @@
       <c r="G295" s="4" t="inlineStr"/>
     </row>
     <row r="296">
-      <c r="A296" s="6" t="n"/>
+      <c r="A296" s="5" t="n"/>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>الضواحي</t>
+          <t>بني مازن</t>
         </is>
       </c>
       <c r="C296" s="4" t="inlineStr"/>
@@ -4997,14 +5144,10 @@
       <c r="G296" s="4" t="inlineStr"/>
     </row>
     <row r="297">
-      <c r="A297" s="2" t="inlineStr">
-        <is>
-          <t>جنوب سيناء</t>
-        </is>
-      </c>
+      <c r="A297" s="6" t="n"/>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>شرم الشيخ</t>
+          <t>العدوة</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr"/>
@@ -5014,36 +5157,56 @@
       <c r="G297" s="4" t="inlineStr"/>
     </row>
     <row r="298">
-      <c r="A298" s="5" t="n"/>
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>الوادي الجديد</t>
+        </is>
+      </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>داهب</t>
-        </is>
-      </c>
-      <c r="C298" s="4" t="inlineStr"/>
+          <t>الخارجة</t>
+        </is>
+      </c>
+      <c r="C298" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب الخارجة للتخاطب</t>
+        </is>
+      </c>
       <c r="D298" s="4" t="inlineStr"/>
       <c r="E298" s="4" t="inlineStr"/>
       <c r="F298" s="4" t="inlineStr"/>
-      <c r="G298" s="4" t="inlineStr"/>
+      <c r="G298" s="4" t="inlineStr">
+        <is>
+          <t>الخارجة</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="5" t="n"/>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>نويبع</t>
-        </is>
-      </c>
-      <c r="C299" s="4" t="inlineStr"/>
+          <t>الداخلة</t>
+        </is>
+      </c>
+      <c r="C299" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب باريس للتخاطب</t>
+        </is>
+      </c>
       <c r="D299" s="4" t="inlineStr"/>
       <c r="E299" s="4" t="inlineStr"/>
       <c r="F299" s="4" t="inlineStr"/>
-      <c r="G299" s="4" t="inlineStr"/>
+      <c r="G299" s="4" t="inlineStr">
+        <is>
+          <t>باريس</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="5" t="n"/>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>سانت كاترين</t>
+          <t>موط</t>
         </is>
       </c>
       <c r="C300" s="4" t="inlineStr"/>
@@ -5056,7 +5219,7 @@
       <c r="A301" s="5" t="n"/>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>طابا</t>
+          <t>بلاط</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr"/>
@@ -5069,7 +5232,7 @@
       <c r="A302" s="5" t="n"/>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>رأس محمد</t>
+          <t>فرافرة</t>
         </is>
       </c>
       <c r="C302" s="4" t="inlineStr"/>
@@ -5082,7 +5245,7 @@
       <c r="A303" s="5" t="n"/>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>أم سيد</t>
+          <t>باريس</t>
         </is>
       </c>
       <c r="C303" s="4" t="inlineStr"/>
@@ -5092,10 +5255,10 @@
       <c r="G303" s="4" t="inlineStr"/>
     </row>
     <row r="304">
-      <c r="A304" s="6" t="n"/>
+      <c r="A304" s="5" t="n"/>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>مدينة شرم الشيخ</t>
+          <t>القصر</t>
         </is>
       </c>
       <c r="C304" s="4" t="inlineStr"/>
@@ -5105,14 +5268,10 @@
       <c r="G304" s="4" t="inlineStr"/>
     </row>
     <row r="305">
-      <c r="A305" s="2" t="inlineStr">
-        <is>
-          <t>حلوان</t>
-        </is>
-      </c>
+      <c r="A305" s="5" t="n"/>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>حلوان</t>
+          <t>تينيدة</t>
         </is>
       </c>
       <c r="C305" s="4" t="inlineStr"/>
@@ -5122,10 +5281,10 @@
       <c r="G305" s="4" t="inlineStr"/>
     </row>
     <row r="306">
-      <c r="A306" s="5" t="n"/>
+      <c r="A306" s="6" t="n"/>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>المعادي</t>
+          <t>دوش</t>
         </is>
       </c>
       <c r="C306" s="4" t="inlineStr"/>
@@ -5135,23 +5294,35 @@
       <c r="G306" s="4" t="inlineStr"/>
     </row>
     <row r="307">
-      <c r="A307" s="5" t="n"/>
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>بني سويف</t>
+        </is>
+      </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>واحة الفيوم</t>
-        </is>
-      </c>
-      <c r="C307" s="4" t="inlineStr"/>
+          <t>بني سويف</t>
+        </is>
+      </c>
+      <c r="C307" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب العبور للتخاطب</t>
+        </is>
+      </c>
       <c r="D307" s="4" t="inlineStr"/>
       <c r="E307" s="4" t="inlineStr"/>
       <c r="F307" s="4" t="inlineStr"/>
-      <c r="G307" s="4" t="inlineStr"/>
+      <c r="G307" s="4" t="inlineStr">
+        <is>
+          <t>بني سويف</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="5" t="n"/>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>وادي حوف</t>
+          <t>الفشن</t>
         </is>
       </c>
       <c r="C308" s="4" t="inlineStr"/>
@@ -5164,7 +5335,7 @@
       <c r="A309" s="5" t="n"/>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>عين سخنة</t>
+          <t>ساماستا</t>
         </is>
       </c>
       <c r="C309" s="4" t="inlineStr"/>
@@ -5177,7 +5348,7 @@
       <c r="A310" s="5" t="n"/>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>الطور</t>
+          <t>إبشواي</t>
         </is>
       </c>
       <c r="C310" s="4" t="inlineStr"/>
@@ -5190,7 +5361,7 @@
       <c r="A311" s="5" t="n"/>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>الزيتون</t>
+          <t>الجندية</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr"/>
@@ -5200,10 +5371,10 @@
       <c r="G311" s="4" t="inlineStr"/>
     </row>
     <row r="312">
-      <c r="A312" s="6" t="n"/>
+      <c r="A312" s="5" t="n"/>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>المقطم</t>
+          <t>ناصر</t>
         </is>
       </c>
       <c r="C312" s="4" t="inlineStr"/>
@@ -5213,35 +5384,23 @@
       <c r="G312" s="4" t="inlineStr"/>
     </row>
     <row r="313">
-      <c r="A313" s="2" t="inlineStr">
-        <is>
-          <t>دمياط</t>
-        </is>
-      </c>
+      <c r="A313" s="5" t="n"/>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>دمياط</t>
-        </is>
-      </c>
-      <c r="C313" s="4" t="inlineStr">
-        <is>
-          <t>مركز حلم ابني للتخاطب</t>
-        </is>
-      </c>
+          <t>هواره</t>
+        </is>
+      </c>
+      <c r="C313" s="4" t="inlineStr"/>
       <c r="D313" s="4" t="inlineStr"/>
       <c r="E313" s="4" t="inlineStr"/>
       <c r="F313" s="4" t="inlineStr"/>
-      <c r="G313" s="4" t="inlineStr">
-        <is>
-          <t>دمياط ودمياط الجديدة</t>
-        </is>
-      </c>
+      <c r="G313" s="4" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" s="5" t="n"/>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>دمياط الجديدة</t>
+          <t>موشية</t>
         </is>
       </c>
       <c r="C314" s="4" t="inlineStr"/>
@@ -5254,7 +5413,7 @@
       <c r="A315" s="5" t="n"/>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>بورت فؤاد</t>
+          <t>نصار البحرية</t>
         </is>
       </c>
       <c r="C315" s="4" t="inlineStr"/>
@@ -5264,10 +5423,10 @@
       <c r="G315" s="4" t="inlineStr"/>
     </row>
     <row r="316">
-      <c r="A316" s="5" t="n"/>
+      <c r="A316" s="6" t="n"/>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>كفر البطة</t>
+          <t>أحمد حمزة</t>
         </is>
       </c>
       <c r="C316" s="4" t="inlineStr"/>
@@ -5277,10 +5436,14 @@
       <c r="G316" s="4" t="inlineStr"/>
     </row>
     <row r="317">
-      <c r="A317" s="5" t="n"/>
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>بورسعيد</t>
+        </is>
+      </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>كفر سعيد</t>
+          <t>بورسعيد</t>
         </is>
       </c>
       <c r="C317" s="4" t="inlineStr"/>
@@ -5293,7 +5456,7 @@
       <c r="A318" s="5" t="n"/>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>الروضة</t>
+          <t>بورفؤاد</t>
         </is>
       </c>
       <c r="C318" s="4" t="inlineStr"/>
@@ -5306,7 +5469,7 @@
       <c r="A319" s="5" t="n"/>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>الزرقا</t>
+          <t>الجميل</t>
         </is>
       </c>
       <c r="C319" s="4" t="inlineStr"/>
@@ -5319,7 +5482,7 @@
       <c r="A320" s="5" t="n"/>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>فارسكور</t>
+          <t>الزهور</t>
         </is>
       </c>
       <c r="C320" s="4" t="inlineStr"/>
@@ -5329,10 +5492,10 @@
       <c r="G320" s="4" t="inlineStr"/>
     </row>
     <row r="321">
-      <c r="A321" s="6" t="n"/>
+      <c r="A321" s="5" t="n"/>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>رومانية</t>
+          <t>بورسعيد</t>
         </is>
       </c>
       <c r="C321" s="4" t="inlineStr"/>
@@ -5342,77 +5505,53 @@
       <c r="G321" s="4" t="inlineStr"/>
     </row>
     <row r="322">
-      <c r="A322" s="2" t="inlineStr">
-        <is>
-          <t>شمال سيناء</t>
-        </is>
-      </c>
+      <c r="A322" s="5" t="n"/>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>العريش</t>
-        </is>
-      </c>
-      <c r="C322" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب العريش للتخاطب</t>
-        </is>
-      </c>
+          <t>الكنتاوي</t>
+        </is>
+      </c>
+      <c r="C322" s="4" t="inlineStr"/>
       <c r="D322" s="4" t="inlineStr"/>
       <c r="E322" s="4" t="inlineStr"/>
       <c r="F322" s="4" t="inlineStr"/>
-      <c r="G322" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب العريش</t>
-        </is>
-      </c>
+      <c r="G322" s="4" t="inlineStr"/>
     </row>
     <row r="323">
-      <c r="A323" s="5" t="n"/>
+      <c r="A323" s="6" t="n"/>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>رفح</t>
-        </is>
-      </c>
-      <c r="C323" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب رفح</t>
-        </is>
-      </c>
+          <t>الضواحي</t>
+        </is>
+      </c>
+      <c r="C323" s="4" t="inlineStr"/>
       <c r="D323" s="4" t="inlineStr"/>
       <c r="E323" s="4" t="inlineStr"/>
       <c r="F323" s="4" t="inlineStr"/>
-      <c r="G323" s="4" t="inlineStr">
-        <is>
-          <t>رفح</t>
-        </is>
-      </c>
+      <c r="G323" s="4" t="inlineStr"/>
     </row>
     <row r="324">
-      <c r="A324" s="5" t="n"/>
+      <c r="A324" s="2" t="inlineStr">
+        <is>
+          <t>جنوب سيناء</t>
+        </is>
+      </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>الشيخ زويد</t>
-        </is>
-      </c>
-      <c r="C324" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب الشيخ زويد (قيد الإنشاء)</t>
-        </is>
-      </c>
+          <t>شرم الشيخ</t>
+        </is>
+      </c>
+      <c r="C324" s="4" t="inlineStr"/>
       <c r="D324" s="4" t="inlineStr"/>
       <c r="E324" s="4" t="inlineStr"/>
       <c r="F324" s="4" t="inlineStr"/>
-      <c r="G324" s="4" t="inlineStr">
-        <is>
-          <t>الشيخ زويد</t>
-        </is>
-      </c>
+      <c r="G324" s="4" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" s="5" t="n"/>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>بئر العبد</t>
+          <t>داهب</t>
         </is>
       </c>
       <c r="C325" s="4" t="inlineStr"/>
@@ -5425,7 +5564,7 @@
       <c r="A326" s="5" t="n"/>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>القنطرة، سيناء</t>
+          <t>نويبع</t>
         </is>
       </c>
       <c r="C326" s="4" t="inlineStr"/>
@@ -5438,7 +5577,7 @@
       <c r="A327" s="5" t="n"/>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>نخل</t>
+          <t>سانت كاترين</t>
         </is>
       </c>
       <c r="C327" s="4" t="inlineStr"/>
@@ -5451,7 +5590,7 @@
       <c r="A328" s="5" t="n"/>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>جديدة، حسنة</t>
+          <t>طابا</t>
         </is>
       </c>
       <c r="C328" s="4" t="inlineStr"/>
@@ -5464,7 +5603,7 @@
       <c r="A329" s="5" t="n"/>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>دهب الشرقية</t>
+          <t>رأس محمد</t>
         </is>
       </c>
       <c r="C329" s="4" t="inlineStr"/>
@@ -5474,10 +5613,10 @@
       <c r="G329" s="4" t="inlineStr"/>
     </row>
     <row r="330">
-      <c r="A330" s="6" t="n"/>
+      <c r="A330" s="5" t="n"/>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>طابا</t>
+          <t>أم سيد</t>
         </is>
       </c>
       <c r="C330" s="4" t="inlineStr"/>
@@ -5487,52 +5626,40 @@
       <c r="G330" s="4" t="inlineStr"/>
     </row>
     <row r="331">
-      <c r="A331" s="2" t="inlineStr">
-        <is>
-          <t>قنا</t>
-        </is>
-      </c>
+      <c r="A331" s="6" t="n"/>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>قنا</t>
-        </is>
-      </c>
-      <c r="C331" s="4" t="inlineStr">
-        <is>
-          <t>مركز التخاطب بمدينة العمال</t>
-        </is>
-      </c>
+          <t>مدينة شرم الشيخ</t>
+        </is>
+      </c>
+      <c r="C331" s="4" t="inlineStr"/>
       <c r="D331" s="4" t="inlineStr"/>
       <c r="E331" s="4" t="inlineStr"/>
       <c r="F331" s="4" t="inlineStr"/>
-      <c r="G331" s="4" t="inlineStr">
-        <is>
-          <t>مدينة العمال، قنا</t>
-        </is>
-      </c>
+      <c r="G331" s="4" t="inlineStr"/>
     </row>
     <row r="332">
-      <c r="A332" s="5" t="n"/>
-      <c r="B332" s="6" t="n"/>
-      <c r="C332" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب حجير خزام</t>
-        </is>
-      </c>
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>حلوان</t>
+        </is>
+      </c>
+      <c r="B332" s="3" t="inlineStr">
+        <is>
+          <t>حلوان</t>
+        </is>
+      </c>
+      <c r="C332" s="4" t="inlineStr"/>
       <c r="D332" s="4" t="inlineStr"/>
       <c r="E332" s="4" t="inlineStr"/>
       <c r="F332" s="4" t="inlineStr"/>
-      <c r="G332" s="4" t="inlineStr">
-        <is>
-          <t>قنا</t>
-        </is>
-      </c>
+      <c r="G332" s="4" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" s="5" t="n"/>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>نجع حمادي</t>
+          <t>المعادي</t>
         </is>
       </c>
       <c r="C333" s="4" t="inlineStr"/>
@@ -5545,7 +5672,7 @@
       <c r="A334" s="5" t="n"/>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>دندرة</t>
+          <t>واحة الفيوم</t>
         </is>
       </c>
       <c r="C334" s="4" t="inlineStr"/>
@@ -5558,7 +5685,7 @@
       <c r="A335" s="5" t="n"/>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>أبيدوس</t>
+          <t>وادي حوف</t>
         </is>
       </c>
       <c r="C335" s="4" t="inlineStr"/>
@@ -5571,7 +5698,7 @@
       <c r="A336" s="5" t="n"/>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>قفطي</t>
+          <t>عين سخنة</t>
         </is>
       </c>
       <c r="C336" s="4" t="inlineStr"/>
@@ -5584,7 +5711,7 @@
       <c r="A337" s="5" t="n"/>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>أخميم</t>
+          <t>الطور</t>
         </is>
       </c>
       <c r="C337" s="4" t="inlineStr"/>
@@ -5597,7 +5724,7 @@
       <c r="A338" s="5" t="n"/>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>سوهاج القديمة</t>
+          <t>الزيتون</t>
         </is>
       </c>
       <c r="C338" s="4" t="inlineStr"/>
@@ -5607,10 +5734,10 @@
       <c r="G338" s="4" t="inlineStr"/>
     </row>
     <row r="339">
-      <c r="A339" s="5" t="n"/>
+      <c r="A339" s="6" t="n"/>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>النجع البحري</t>
+          <t>المقطم</t>
         </is>
       </c>
       <c r="C339" s="4" t="inlineStr"/>
@@ -5620,69 +5747,61 @@
       <c r="G339" s="4" t="inlineStr"/>
     </row>
     <row r="340">
-      <c r="A340" s="6" t="n"/>
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>دمياط</t>
+        </is>
+      </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>الشنقي</t>
-        </is>
-      </c>
-      <c r="C340" s="4" t="inlineStr"/>
+          <t>دمياط</t>
+        </is>
+      </c>
+      <c r="C340" s="4" t="inlineStr">
+        <is>
+          <t>مركز حلم ابني للتخاطب</t>
+        </is>
+      </c>
       <c r="D340" s="4" t="inlineStr"/>
       <c r="E340" s="4" t="inlineStr"/>
       <c r="F340" s="4" t="inlineStr"/>
-      <c r="G340" s="4" t="inlineStr"/>
+      <c r="G340" s="4" t="inlineStr">
+        <is>
+          <t>دمياط ودمياط الجديدة</t>
+        </is>
+      </c>
     </row>
     <row r="341">
-      <c r="A341" s="2" t="inlineStr">
-        <is>
-          <t>كفر الشيخ</t>
-        </is>
-      </c>
+      <c r="A341" s="5" t="n"/>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>كفر الشيخ</t>
-        </is>
-      </c>
-      <c r="C341" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب كفر الشيخ للتخاطب</t>
-        </is>
-      </c>
+          <t>دمياط الجديدة</t>
+        </is>
+      </c>
+      <c r="C341" s="4" t="inlineStr"/>
       <c r="D341" s="4" t="inlineStr"/>
       <c r="E341" s="4" t="inlineStr"/>
       <c r="F341" s="4" t="inlineStr"/>
-      <c r="G341" s="4" t="inlineStr">
-        <is>
-          <t>كفر الشيخ</t>
-        </is>
-      </c>
+      <c r="G341" s="4" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" s="5" t="n"/>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>دسوق</t>
-        </is>
-      </c>
-      <c r="C342" s="4" t="inlineStr">
-        <is>
-          <t>مركز رعايه للتخاطب والتدخل المبكر</t>
-        </is>
-      </c>
+          <t>بورت فؤاد</t>
+        </is>
+      </c>
+      <c r="C342" s="4" t="inlineStr"/>
       <c r="D342" s="4" t="inlineStr"/>
       <c r="E342" s="4" t="inlineStr"/>
       <c r="F342" s="4" t="inlineStr"/>
-      <c r="G342" s="4" t="inlineStr">
-        <is>
-          <t>شارع شهداء المغربي، خلف جمعية الشروق</t>
-        </is>
-      </c>
+      <c r="G342" s="4" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" s="5" t="n"/>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>بلامون</t>
+          <t>كفر البطة</t>
         </is>
       </c>
       <c r="C343" s="4" t="inlineStr"/>
@@ -5695,7 +5814,7 @@
       <c r="A344" s="5" t="n"/>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>الرياض</t>
+          <t>كفر سعيد</t>
         </is>
       </c>
       <c r="C344" s="4" t="inlineStr"/>
@@ -5708,7 +5827,7 @@
       <c r="A345" s="5" t="n"/>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>سيدي سالم</t>
+          <t>الروضة</t>
         </is>
       </c>
       <c r="C345" s="4" t="inlineStr"/>
@@ -5721,7 +5840,7 @@
       <c r="A346" s="5" t="n"/>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>الحامول</t>
+          <t>الزرقا</t>
         </is>
       </c>
       <c r="C346" s="4" t="inlineStr"/>
@@ -5734,7 +5853,7 @@
       <c r="A347" s="5" t="n"/>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>برج البرلس</t>
+          <t>فارسكور</t>
         </is>
       </c>
       <c r="C347" s="4" t="inlineStr"/>
@@ -5744,10 +5863,10 @@
       <c r="G347" s="4" t="inlineStr"/>
     </row>
     <row r="348">
-      <c r="A348" s="5" t="n"/>
+      <c r="A348" s="6" t="n"/>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>مطوبس</t>
+          <t>رومانية</t>
         </is>
       </c>
       <c r="C348" s="4" t="inlineStr"/>
@@ -5757,57 +5876,77 @@
       <c r="G348" s="4" t="inlineStr"/>
     </row>
     <row r="349">
-      <c r="A349" s="5" t="n"/>
+      <c r="A349" s="2" t="inlineStr">
+        <is>
+          <t>شمال سيناء</t>
+        </is>
+      </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>المحمودية</t>
-        </is>
-      </c>
-      <c r="C349" s="4" t="inlineStr"/>
+          <t>العريش</t>
+        </is>
+      </c>
+      <c r="C349" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب العريش للتخاطب</t>
+        </is>
+      </c>
       <c r="D349" s="4" t="inlineStr"/>
       <c r="E349" s="4" t="inlineStr"/>
       <c r="F349" s="4" t="inlineStr"/>
-      <c r="G349" s="4" t="inlineStr"/>
+      <c r="G349" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب العريش</t>
+        </is>
+      </c>
     </row>
     <row r="350">
-      <c r="A350" s="6" t="n"/>
+      <c r="A350" s="5" t="n"/>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>بيلا</t>
-        </is>
-      </c>
-      <c r="C350" s="4" t="inlineStr"/>
+          <t>رفح</t>
+        </is>
+      </c>
+      <c r="C350" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب رفح</t>
+        </is>
+      </c>
       <c r="D350" s="4" t="inlineStr"/>
       <c r="E350" s="4" t="inlineStr"/>
       <c r="F350" s="4" t="inlineStr"/>
-      <c r="G350" s="4" t="inlineStr"/>
+      <c r="G350" s="4" t="inlineStr">
+        <is>
+          <t>رفح</t>
+        </is>
+      </c>
     </row>
     <row r="351">
-      <c r="A351" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A351" s="5" t="n"/>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="C351" s="4" t="inlineStr"/>
+          <t>الشيخ زويد</t>
+        </is>
+      </c>
+      <c r="C351" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب الشيخ زويد (قيد الإنشاء)</t>
+        </is>
+      </c>
       <c r="D351" s="4" t="inlineStr"/>
       <c r="E351" s="4" t="inlineStr"/>
       <c r="F351" s="4" t="inlineStr"/>
-      <c r="G351" s="4" t="inlineStr"/>
+      <c r="G351" s="4" t="inlineStr">
+        <is>
+          <t>الشيخ زويد</t>
+        </is>
+      </c>
     </row>
     <row r="352">
-      <c r="A352" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A352" s="5" t="n"/>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>سيوه</t>
+          <t>بئر العبد</t>
         </is>
       </c>
       <c r="C352" s="4" t="inlineStr"/>
@@ -5817,14 +5956,10 @@
       <c r="G352" s="4" t="inlineStr"/>
     </row>
     <row r="353">
-      <c r="A353" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A353" s="5" t="n"/>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>السلوم</t>
+          <t>القنطرة، سيناء</t>
         </is>
       </c>
       <c r="C353" s="4" t="inlineStr"/>
@@ -5834,14 +5969,10 @@
       <c r="G353" s="4" t="inlineStr"/>
     </row>
     <row r="354">
-      <c r="A354" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A354" s="5" t="n"/>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>سيدي براني</t>
+          <t>نخل</t>
         </is>
       </c>
       <c r="C354" s="4" t="inlineStr"/>
@@ -5851,14 +5982,10 @@
       <c r="G354" s="4" t="inlineStr"/>
     </row>
     <row r="355">
-      <c r="A355" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A355" s="5" t="n"/>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>العلمين</t>
+          <t>جديدة، حسنة</t>
         </is>
       </c>
       <c r="C355" s="4" t="inlineStr"/>
@@ -5868,14 +5995,10 @@
       <c r="G355" s="4" t="inlineStr"/>
     </row>
     <row r="356">
-      <c r="A356" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A356" s="5" t="n"/>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>مارينا</t>
+          <t>دهب الشرقية</t>
         </is>
       </c>
       <c r="C356" s="4" t="inlineStr"/>
@@ -5885,14 +6008,10 @@
       <c r="G356" s="4" t="inlineStr"/>
     </row>
     <row r="357">
-      <c r="A357" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A357" s="6" t="n"/>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>توريدو</t>
+          <t>طابا</t>
         </is>
       </c>
       <c r="C357" s="4" t="inlineStr"/>
@@ -5904,46 +6023,50 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>مطروح</t>
+          <t>قنا</t>
         </is>
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>جنوب سيوه</t>
-        </is>
-      </c>
-      <c r="C358" s="4" t="inlineStr"/>
+          <t>قنا</t>
+        </is>
+      </c>
+      <c r="C358" s="4" t="inlineStr">
+        <is>
+          <t>مركز التخاطب بمدينة العمال</t>
+        </is>
+      </c>
       <c r="D358" s="4" t="inlineStr"/>
       <c r="E358" s="4" t="inlineStr"/>
       <c r="F358" s="4" t="inlineStr"/>
-      <c r="G358" s="4" t="inlineStr"/>
+      <c r="G358" s="4" t="inlineStr">
+        <is>
+          <t>مدينة العمال، قنا</t>
+        </is>
+      </c>
     </row>
     <row r="359">
-      <c r="A359" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B359" s="3" t="inlineStr">
-        <is>
-          <t>شمال سيوه</t>
-        </is>
-      </c>
-      <c r="C359" s="4" t="inlineStr"/>
+      <c r="A359" s="5" t="n"/>
+      <c r="B359" s="6" t="n"/>
+      <c r="C359" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب حجير خزام</t>
+        </is>
+      </c>
       <c r="D359" s="4" t="inlineStr"/>
       <c r="E359" s="4" t="inlineStr"/>
       <c r="F359" s="4" t="inlineStr"/>
-      <c r="G359" s="4" t="inlineStr"/>
+      <c r="G359" s="4" t="inlineStr">
+        <is>
+          <t>قنا</t>
+        </is>
+      </c>
     </row>
     <row r="360">
-      <c r="A360" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
+      <c r="A360" s="5" t="n"/>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>كشته</t>
+          <t>نجع حمادي</t>
         </is>
       </c>
       <c r="C360" s="4" t="inlineStr"/>
@@ -5951,6 +6074,417 @@
       <c r="E360" s="4" t="inlineStr"/>
       <c r="F360" s="4" t="inlineStr"/>
       <c r="G360" s="4" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="5" t="n"/>
+      <c r="B361" s="3" t="inlineStr">
+        <is>
+          <t>دندرة</t>
+        </is>
+      </c>
+      <c r="C361" s="4" t="inlineStr"/>
+      <c r="D361" s="4" t="inlineStr"/>
+      <c r="E361" s="4" t="inlineStr"/>
+      <c r="F361" s="4" t="inlineStr"/>
+      <c r="G361" s="4" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="5" t="n"/>
+      <c r="B362" s="3" t="inlineStr">
+        <is>
+          <t>أبيدوس</t>
+        </is>
+      </c>
+      <c r="C362" s="4" t="inlineStr"/>
+      <c r="D362" s="4" t="inlineStr"/>
+      <c r="E362" s="4" t="inlineStr"/>
+      <c r="F362" s="4" t="inlineStr"/>
+      <c r="G362" s="4" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="5" t="n"/>
+      <c r="B363" s="3" t="inlineStr">
+        <is>
+          <t>قفطي</t>
+        </is>
+      </c>
+      <c r="C363" s="4" t="inlineStr"/>
+      <c r="D363" s="4" t="inlineStr"/>
+      <c r="E363" s="4" t="inlineStr"/>
+      <c r="F363" s="4" t="inlineStr"/>
+      <c r="G363" s="4" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="5" t="n"/>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>أخميم</t>
+        </is>
+      </c>
+      <c r="C364" s="4" t="inlineStr"/>
+      <c r="D364" s="4" t="inlineStr"/>
+      <c r="E364" s="4" t="inlineStr"/>
+      <c r="F364" s="4" t="inlineStr"/>
+      <c r="G364" s="4" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="5" t="n"/>
+      <c r="B365" s="3" t="inlineStr">
+        <is>
+          <t>سوهاج القديمة</t>
+        </is>
+      </c>
+      <c r="C365" s="4" t="inlineStr"/>
+      <c r="D365" s="4" t="inlineStr"/>
+      <c r="E365" s="4" t="inlineStr"/>
+      <c r="F365" s="4" t="inlineStr"/>
+      <c r="G365" s="4" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="5" t="n"/>
+      <c r="B366" s="3" t="inlineStr">
+        <is>
+          <t>النجع البحري</t>
+        </is>
+      </c>
+      <c r="C366" s="4" t="inlineStr"/>
+      <c r="D366" s="4" t="inlineStr"/>
+      <c r="E366" s="4" t="inlineStr"/>
+      <c r="F366" s="4" t="inlineStr"/>
+      <c r="G366" s="4" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="6" t="n"/>
+      <c r="B367" s="3" t="inlineStr">
+        <is>
+          <t>الشنقي</t>
+        </is>
+      </c>
+      <c r="C367" s="4" t="inlineStr"/>
+      <c r="D367" s="4" t="inlineStr"/>
+      <c r="E367" s="4" t="inlineStr"/>
+      <c r="F367" s="4" t="inlineStr"/>
+      <c r="G367" s="4" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
+      <c r="B368" s="3" t="inlineStr">
+        <is>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
+      <c r="C368" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب كفر الشيخ للتخاطب</t>
+        </is>
+      </c>
+      <c r="D368" s="4" t="inlineStr"/>
+      <c r="E368" s="4" t="inlineStr"/>
+      <c r="F368" s="4" t="inlineStr"/>
+      <c r="G368" s="4" t="inlineStr">
+        <is>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="5" t="n"/>
+      <c r="B369" s="3" t="inlineStr">
+        <is>
+          <t>دسوق</t>
+        </is>
+      </c>
+      <c r="C369" s="4" t="inlineStr">
+        <is>
+          <t>مركز رعايه للتخاطب والتدخل المبكر</t>
+        </is>
+      </c>
+      <c r="D369" s="4" t="inlineStr"/>
+      <c r="E369" s="4" t="inlineStr"/>
+      <c r="F369" s="4" t="inlineStr"/>
+      <c r="G369" s="4" t="inlineStr">
+        <is>
+          <t>شارع شهداء المغربي، خلف جمعية الشروق</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="5" t="n"/>
+      <c r="B370" s="3" t="inlineStr">
+        <is>
+          <t>بلامون</t>
+        </is>
+      </c>
+      <c r="C370" s="4" t="inlineStr"/>
+      <c r="D370" s="4" t="inlineStr"/>
+      <c r="E370" s="4" t="inlineStr"/>
+      <c r="F370" s="4" t="inlineStr"/>
+      <c r="G370" s="4" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="5" t="n"/>
+      <c r="B371" s="3" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="C371" s="4" t="inlineStr"/>
+      <c r="D371" s="4" t="inlineStr"/>
+      <c r="E371" s="4" t="inlineStr"/>
+      <c r="F371" s="4" t="inlineStr"/>
+      <c r="G371" s="4" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="5" t="n"/>
+      <c r="B372" s="3" t="inlineStr">
+        <is>
+          <t>سيدي سالم</t>
+        </is>
+      </c>
+      <c r="C372" s="4" t="inlineStr"/>
+      <c r="D372" s="4" t="inlineStr"/>
+      <c r="E372" s="4" t="inlineStr"/>
+      <c r="F372" s="4" t="inlineStr"/>
+      <c r="G372" s="4" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="5" t="n"/>
+      <c r="B373" s="3" t="inlineStr">
+        <is>
+          <t>الحامول</t>
+        </is>
+      </c>
+      <c r="C373" s="4" t="inlineStr"/>
+      <c r="D373" s="4" t="inlineStr"/>
+      <c r="E373" s="4" t="inlineStr"/>
+      <c r="F373" s="4" t="inlineStr"/>
+      <c r="G373" s="4" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="5" t="n"/>
+      <c r="B374" s="3" t="inlineStr">
+        <is>
+          <t>برج البرلس</t>
+        </is>
+      </c>
+      <c r="C374" s="4" t="inlineStr"/>
+      <c r="D374" s="4" t="inlineStr"/>
+      <c r="E374" s="4" t="inlineStr"/>
+      <c r="F374" s="4" t="inlineStr"/>
+      <c r="G374" s="4" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="5" t="n"/>
+      <c r="B375" s="3" t="inlineStr">
+        <is>
+          <t>مطوبس</t>
+        </is>
+      </c>
+      <c r="C375" s="4" t="inlineStr"/>
+      <c r="D375" s="4" t="inlineStr"/>
+      <c r="E375" s="4" t="inlineStr"/>
+      <c r="F375" s="4" t="inlineStr"/>
+      <c r="G375" s="4" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="5" t="n"/>
+      <c r="B376" s="3" t="inlineStr">
+        <is>
+          <t>المحمودية</t>
+        </is>
+      </c>
+      <c r="C376" s="4" t="inlineStr"/>
+      <c r="D376" s="4" t="inlineStr"/>
+      <c r="E376" s="4" t="inlineStr"/>
+      <c r="F376" s="4" t="inlineStr"/>
+      <c r="G376" s="4" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="6" t="n"/>
+      <c r="B377" s="3" t="inlineStr">
+        <is>
+          <t>بيلا</t>
+        </is>
+      </c>
+      <c r="C377" s="4" t="inlineStr"/>
+      <c r="D377" s="4" t="inlineStr"/>
+      <c r="E377" s="4" t="inlineStr"/>
+      <c r="F377" s="4" t="inlineStr"/>
+      <c r="G377" s="4" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B378" s="3" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="C378" s="4" t="inlineStr"/>
+      <c r="D378" s="4" t="inlineStr"/>
+      <c r="E378" s="4" t="inlineStr"/>
+      <c r="F378" s="4" t="inlineStr"/>
+      <c r="G378" s="4" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B379" s="3" t="inlineStr">
+        <is>
+          <t>سيوه</t>
+        </is>
+      </c>
+      <c r="C379" s="4" t="inlineStr"/>
+      <c r="D379" s="4" t="inlineStr"/>
+      <c r="E379" s="4" t="inlineStr"/>
+      <c r="F379" s="4" t="inlineStr"/>
+      <c r="G379" s="4" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B380" s="3" t="inlineStr">
+        <is>
+          <t>السلوم</t>
+        </is>
+      </c>
+      <c r="C380" s="4" t="inlineStr"/>
+      <c r="D380" s="4" t="inlineStr"/>
+      <c r="E380" s="4" t="inlineStr"/>
+      <c r="F380" s="4" t="inlineStr"/>
+      <c r="G380" s="4" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B381" s="3" t="inlineStr">
+        <is>
+          <t>سيدي براني</t>
+        </is>
+      </c>
+      <c r="C381" s="4" t="inlineStr"/>
+      <c r="D381" s="4" t="inlineStr"/>
+      <c r="E381" s="4" t="inlineStr"/>
+      <c r="F381" s="4" t="inlineStr"/>
+      <c r="G381" s="4" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B382" s="3" t="inlineStr">
+        <is>
+          <t>العلمين</t>
+        </is>
+      </c>
+      <c r="C382" s="4" t="inlineStr"/>
+      <c r="D382" s="4" t="inlineStr"/>
+      <c r="E382" s="4" t="inlineStr"/>
+      <c r="F382" s="4" t="inlineStr"/>
+      <c r="G382" s="4" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>مارينا</t>
+        </is>
+      </c>
+      <c r="C383" s="4" t="inlineStr"/>
+      <c r="D383" s="4" t="inlineStr"/>
+      <c r="E383" s="4" t="inlineStr"/>
+      <c r="F383" s="4" t="inlineStr"/>
+      <c r="G383" s="4" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B384" s="3" t="inlineStr">
+        <is>
+          <t>توريدو</t>
+        </is>
+      </c>
+      <c r="C384" s="4" t="inlineStr"/>
+      <c r="D384" s="4" t="inlineStr"/>
+      <c r="E384" s="4" t="inlineStr"/>
+      <c r="F384" s="4" t="inlineStr"/>
+      <c r="G384" s="4" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B385" s="3" t="inlineStr">
+        <is>
+          <t>جنوب سيوه</t>
+        </is>
+      </c>
+      <c r="C385" s="4" t="inlineStr"/>
+      <c r="D385" s="4" t="inlineStr"/>
+      <c r="E385" s="4" t="inlineStr"/>
+      <c r="F385" s="4" t="inlineStr"/>
+      <c r="G385" s="4" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B386" s="3" t="inlineStr">
+        <is>
+          <t>شمال سيوه</t>
+        </is>
+      </c>
+      <c r="C386" s="4" t="inlineStr"/>
+      <c r="D386" s="4" t="inlineStr"/>
+      <c r="E386" s="4" t="inlineStr"/>
+      <c r="F386" s="4" t="inlineStr"/>
+      <c r="G386" s="4" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B387" s="3" t="inlineStr">
+        <is>
+          <t>كشته</t>
+        </is>
+      </c>
+      <c r="C387" s="4" t="inlineStr"/>
+      <c r="D387" s="4" t="inlineStr"/>
+      <c r="E387" s="4" t="inlineStr"/>
+      <c r="F387" s="4" t="inlineStr"/>
+      <c r="G387" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="313">

</xml_diff>

<commit_message>
Revert "Add comprehensive Cairo speech therapy centers to existing data"
This reverts commit a4f69dca1db3d9d58d9afa0eb633e3e086d4c722.
</commit_message>
<xml_diff>
--- a/Egyptian_Speech_Therapy_Centers.xlsx
+++ b/Egyptian_Speech_Therapy_Centers.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,15 +44,6 @@
     <font>
       <name val="Arial"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="00000000"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -120,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -136,15 +127,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -510,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G387"/>
+  <dimension ref="A1:G360"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4010,552 +3992,427 @@
       <c r="G227" s="4" t="inlineStr"/>
     </row>
     <row r="228">
-      <c r="A228" s="7" t="inlineStr">
-        <is>
-          <t>القاهرة</t>
-        </is>
-      </c>
-      <c r="B228" s="8" t="inlineStr">
-        <is>
-          <t>مركز التخاطب الشامل وصعوبات التعلم - فرع جديد</t>
-        </is>
-      </c>
-      <c r="C228" s="8" t="inlineStr"/>
-      <c r="D228" s="9" t="inlineStr">
-        <is>
-          <t>0222406301</t>
-        </is>
-      </c>
-      <c r="E228" s="9" t="inlineStr"/>
-      <c r="F228" s="8" t="inlineStr">
-        <is>
-          <t>مصر الجديدة</t>
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>القليوبية</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>بنها</t>
+        </is>
+      </c>
+      <c r="C228" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب برج مكة</t>
+        </is>
+      </c>
+      <c r="D228" s="4" t="inlineStr"/>
+      <c r="E228" s="4" t="inlineStr"/>
+      <c r="F228" s="4" t="inlineStr"/>
+      <c r="G228" s="4" t="inlineStr">
+        <is>
+          <t>شارع جميل أمام بنك القاهرة</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="5" t="n"/>
-      <c r="B229" s="8" t="inlineStr">
-        <is>
-          <t>مركز تخاطب البر والتقوى</t>
-        </is>
-      </c>
-      <c r="C229" s="8" t="inlineStr"/>
-      <c r="D229" s="9" t="inlineStr"/>
-      <c r="E229" s="9" t="inlineStr"/>
-      <c r="F229" s="8" t="inlineStr">
-        <is>
-          <t>104 برج الأوقاف، شارع ابن سندر، سرايا القبة، القاهرة</t>
+      <c r="B229" s="5" t="n"/>
+      <c r="C229" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب كفر الجزار</t>
+        </is>
+      </c>
+      <c r="D229" s="4" t="inlineStr"/>
+      <c r="E229" s="4" t="inlineStr"/>
+      <c r="F229" s="4" t="inlineStr"/>
+      <c r="G229" s="4" t="inlineStr">
+        <is>
+          <t>بنها</t>
         </is>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="6" t="n"/>
-      <c r="B230" s="8" t="inlineStr">
-        <is>
-          <t>بيت التمريض</t>
-        </is>
-      </c>
-      <c r="C230" s="8" t="inlineStr"/>
-      <c r="D230" s="9" t="inlineStr">
-        <is>
-          <t>201201120500</t>
-        </is>
-      </c>
-      <c r="E230" s="9" t="inlineStr"/>
-      <c r="F230" s="8" t="inlineStr">
-        <is>
-          <t>متخصص في التخاطب وتعديل السلوك</t>
+      <c r="A230" s="5" t="n"/>
+      <c r="B230" s="6" t="n"/>
+      <c r="C230" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب العمار</t>
+        </is>
+      </c>
+      <c r="D230" s="4" t="inlineStr"/>
+      <c r="E230" s="4" t="inlineStr"/>
+      <c r="F230" s="4" t="inlineStr"/>
+      <c r="G230" s="4" t="inlineStr">
+        <is>
+          <t>بنها</t>
         </is>
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="7" t="inlineStr">
-        <is>
-          <t>مدينة نصر</t>
-        </is>
-      </c>
-      <c r="B231" s="8" t="inlineStr">
-        <is>
-          <t>المركز الذهبي التخصصي (GSC)</t>
-        </is>
-      </c>
-      <c r="C231" s="8" t="inlineStr"/>
-      <c r="D231" s="9" t="inlineStr"/>
-      <c r="E231" s="9" t="inlineStr"/>
-      <c r="F231" s="8" t="inlineStr">
-        <is>
-          <t>مدينة نصر، متخصص في التخاطب وتعديل السلوك</t>
-        </is>
-      </c>
+      <c r="A231" s="5" t="n"/>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>قليوب</t>
+        </is>
+      </c>
+      <c r="C231" s="4" t="inlineStr"/>
+      <c r="D231" s="4" t="inlineStr"/>
+      <c r="E231" s="4" t="inlineStr"/>
+      <c r="F231" s="4" t="inlineStr"/>
+      <c r="G231" s="4" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="5" t="n"/>
-      <c r="B232" s="8" t="inlineStr">
-        <is>
-          <t>مركز Speak للتخاطب</t>
-        </is>
-      </c>
-      <c r="C232" s="8" t="inlineStr"/>
-      <c r="D232" s="9" t="inlineStr"/>
-      <c r="E232" s="9" t="inlineStr"/>
-      <c r="F232" s="8" t="inlineStr">
-        <is>
-          <t>زهراء مدينة نصر، المرحلة الأولى، بجوار مسجد النور</t>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>شبرا الخيمة</t>
+        </is>
+      </c>
+      <c r="C232" s="4" t="inlineStr">
+        <is>
+          <t>مركز الغد للتخاطب وصعوبات التعلم</t>
+        </is>
+      </c>
+      <c r="D232" s="4" t="inlineStr"/>
+      <c r="E232" s="4" t="inlineStr"/>
+      <c r="F232" s="4" t="inlineStr"/>
+      <c r="G232" s="4" t="inlineStr">
+        <is>
+          <t>75 شارع حنفي الشيخوني</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="5" t="n"/>
-      <c r="B233" s="8" t="inlineStr">
-        <is>
-          <t>مركز الزهراء للتخاطب</t>
-        </is>
-      </c>
-      <c r="C233" s="8" t="inlineStr"/>
-      <c r="D233" s="9" t="inlineStr"/>
-      <c r="E233" s="9" t="inlineStr"/>
-      <c r="F233" s="8" t="inlineStr">
-        <is>
-          <t>5 شارع الصواف، المنطقة العاشرة، مدينة نصر</t>
+      <c r="B233" s="5" t="n"/>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>مركز النور الهدى الطبي</t>
+        </is>
+      </c>
+      <c r="D233" s="4" t="inlineStr"/>
+      <c r="E233" s="4" t="inlineStr"/>
+      <c r="F233" s="4" t="inlineStr"/>
+      <c r="G233" s="4" t="inlineStr">
+        <is>
+          <t>شارع محمد القطان</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="5" t="n"/>
-      <c r="B234" s="8" t="inlineStr">
-        <is>
-          <t>مركز الحمد للعلاج الطبيعي والتخاطب - فرع مدينة نصر</t>
-        </is>
-      </c>
-      <c r="C234" s="8" t="inlineStr"/>
-      <c r="D234" s="9" t="inlineStr"/>
-      <c r="E234" s="9" t="inlineStr"/>
-      <c r="F234" s="8" t="inlineStr">
-        <is>
-          <t>شارع مصطفى النحاس، فوق التوحيد والنور</t>
+      <c r="B234" s="6" t="n"/>
+      <c r="C234" s="4" t="inlineStr">
+        <is>
+          <t>مركز تواصل للتخاطب</t>
+        </is>
+      </c>
+      <c r="D234" s="4" t="inlineStr"/>
+      <c r="E234" s="4" t="inlineStr"/>
+      <c r="F234" s="4" t="inlineStr"/>
+      <c r="G234" s="4" t="inlineStr">
+        <is>
+          <t>2 شارع أحمد عبد ربه</t>
         </is>
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="6" t="n"/>
-      <c r="B235" s="8" t="inlineStr">
-        <is>
-          <t>مركز الشمس للتخاطب - فرع مدينة نصر</t>
-        </is>
-      </c>
-      <c r="C235" s="8" t="inlineStr"/>
-      <c r="D235" s="9" t="inlineStr"/>
-      <c r="E235" s="9" t="inlineStr"/>
-      <c r="F235" s="8" t="inlineStr">
-        <is>
-          <t>مدينة نصر</t>
-        </is>
-      </c>
+      <c r="A235" s="5" t="n"/>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>الخانكة</t>
+        </is>
+      </c>
+      <c r="C235" s="4" t="inlineStr"/>
+      <c r="D235" s="4" t="inlineStr"/>
+      <c r="E235" s="4" t="inlineStr"/>
+      <c r="F235" s="4" t="inlineStr"/>
+      <c r="G235" s="4" t="inlineStr"/>
     </row>
     <row r="236">
-      <c r="A236" s="7" t="inlineStr">
-        <is>
-          <t>مصر الجديدة</t>
-        </is>
-      </c>
-      <c r="B236" s="8" t="inlineStr">
-        <is>
-          <t>مركز التخاطب الشامل - فرع مصر الجديدة</t>
-        </is>
-      </c>
-      <c r="C236" s="8" t="inlineStr"/>
-      <c r="D236" s="9" t="inlineStr">
-        <is>
-          <t>0222406301</t>
-        </is>
-      </c>
-      <c r="E236" s="9" t="inlineStr"/>
-      <c r="F236" s="8" t="inlineStr">
-        <is>
-          <t>مصر الجديدة</t>
-        </is>
-      </c>
+      <c r="A236" s="5" t="n"/>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>رمسيس</t>
+        </is>
+      </c>
+      <c r="C236" s="4" t="inlineStr"/>
+      <c r="D236" s="4" t="inlineStr"/>
+      <c r="E236" s="4" t="inlineStr"/>
+      <c r="F236" s="4" t="inlineStr"/>
+      <c r="G236" s="4" t="inlineStr"/>
     </row>
     <row r="237">
-      <c r="A237" s="6" t="n"/>
-      <c r="B237" s="8" t="inlineStr">
-        <is>
-          <t>المركز المصري الكندي - فرع النزهة</t>
-        </is>
-      </c>
-      <c r="C237" s="8" t="inlineStr"/>
-      <c r="D237" s="9" t="inlineStr"/>
-      <c r="E237" s="9" t="inlineStr"/>
-      <c r="F237" s="8" t="inlineStr">
-        <is>
-          <t>14 شارع جمال الدين على، بجوار ملاهي السندباد</t>
-        </is>
-      </c>
+      <c r="A237" s="5" t="n"/>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>مدينة 10 رمضان</t>
+        </is>
+      </c>
+      <c r="C237" s="4" t="inlineStr"/>
+      <c r="D237" s="4" t="inlineStr"/>
+      <c r="E237" s="4" t="inlineStr"/>
+      <c r="F237" s="4" t="inlineStr"/>
+      <c r="G237" s="4" t="inlineStr"/>
     </row>
     <row r="238">
-      <c r="A238" s="7" t="inlineStr">
-        <is>
-          <t>المعادي</t>
-        </is>
-      </c>
-      <c r="B238" s="8" t="inlineStr">
-        <is>
-          <t>مركز كيور لجراحات الأذن والقوقعة والسمعيات والتخاطب</t>
-        </is>
-      </c>
-      <c r="C238" s="8" t="inlineStr"/>
-      <c r="D238" s="9" t="inlineStr"/>
-      <c r="E238" s="9" t="inlineStr"/>
-      <c r="F238" s="8" t="inlineStr">
-        <is>
-          <t>شارع النصر، تقاطع اللاسلكي، حي المعادي</t>
-        </is>
-      </c>
+      <c r="A238" s="5" t="n"/>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>الشيخ زايد</t>
+        </is>
+      </c>
+      <c r="C238" s="4" t="inlineStr"/>
+      <c r="D238" s="4" t="inlineStr"/>
+      <c r="E238" s="4" t="inlineStr"/>
+      <c r="F238" s="4" t="inlineStr"/>
+      <c r="G238" s="4" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="5" t="n"/>
-      <c r="B239" s="8" t="inlineStr">
-        <is>
-          <t>مركز الجنا للتخاطب وصعوبات التعلم</t>
-        </is>
-      </c>
-      <c r="C239" s="8" t="inlineStr"/>
-      <c r="D239" s="9" t="inlineStr"/>
-      <c r="E239" s="9" t="inlineStr"/>
-      <c r="F239" s="8" t="inlineStr">
-        <is>
-          <t>شارع 76، المعادى</t>
-        </is>
-      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>القناطر الخيرية</t>
+        </is>
+      </c>
+      <c r="C239" s="4" t="inlineStr"/>
+      <c r="D239" s="4" t="inlineStr"/>
+      <c r="E239" s="4" t="inlineStr"/>
+      <c r="F239" s="4" t="inlineStr"/>
+      <c r="G239" s="4" t="inlineStr"/>
     </row>
     <row r="240">
-      <c r="A240" s="6" t="n"/>
-      <c r="B240" s="8" t="inlineStr">
-        <is>
-          <t>المركز المصري الكندي - فرع المعادي</t>
-        </is>
-      </c>
-      <c r="C240" s="8" t="inlineStr"/>
-      <c r="D240" s="9" t="inlineStr"/>
-      <c r="E240" s="9" t="inlineStr"/>
-      <c r="F240" s="8" t="inlineStr">
-        <is>
-          <t>5/3 شارع اللاسلكي، بجوار شركة غاز مصر</t>
-        </is>
-      </c>
+      <c r="A240" s="5" t="n"/>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
+          <t>قها</t>
+        </is>
+      </c>
+      <c r="C240" s="4" t="inlineStr"/>
+      <c r="D240" s="4" t="inlineStr"/>
+      <c r="E240" s="4" t="inlineStr"/>
+      <c r="F240" s="4" t="inlineStr"/>
+      <c r="G240" s="4" t="inlineStr"/>
     </row>
     <row r="241">
-      <c r="A241" s="7" t="inlineStr">
-        <is>
-          <t>حلوان</t>
-        </is>
-      </c>
-      <c r="B241" s="8" t="inlineStr">
-        <is>
-          <t>مركز علمني للتخاطب وصعوبات التعلم</t>
-        </is>
-      </c>
-      <c r="C241" s="8" t="inlineStr"/>
-      <c r="D241" s="9" t="inlineStr"/>
-      <c r="E241" s="9" t="inlineStr"/>
-      <c r="F241" s="8" t="inlineStr">
-        <is>
-          <t>8 عمارات منتصر، الدور الأرضي، بجوار مسجد عباد الرحمن</t>
-        </is>
-      </c>
+      <c r="A241" s="5" t="n"/>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>الدقهلية</t>
+        </is>
+      </c>
+      <c r="C241" s="4" t="inlineStr"/>
+      <c r="D241" s="4" t="inlineStr"/>
+      <c r="E241" s="4" t="inlineStr"/>
+      <c r="F241" s="4" t="inlineStr"/>
+      <c r="G241" s="4" t="inlineStr"/>
     </row>
     <row r="242">
-      <c r="A242" s="7" t="inlineStr">
-        <is>
-          <t>روض الفرج</t>
-        </is>
-      </c>
-      <c r="B242" s="8" t="inlineStr">
-        <is>
-          <t>مركز تخاطب المرح</t>
-        </is>
-      </c>
-      <c r="C242" s="8" t="inlineStr"/>
-      <c r="D242" s="9" t="inlineStr"/>
-      <c r="E242" s="9" t="inlineStr"/>
-      <c r="F242" s="8" t="inlineStr">
-        <is>
-          <t>محطة مترو مسرة، 14 شارع علي أمين عبده، شبرا مصر</t>
-        </is>
-      </c>
+      <c r="A242" s="5" t="n"/>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="C242" s="4" t="inlineStr"/>
+      <c r="D242" s="4" t="inlineStr"/>
+      <c r="E242" s="4" t="inlineStr"/>
+      <c r="F242" s="4" t="inlineStr"/>
+      <c r="G242" s="4" t="inlineStr"/>
     </row>
     <row r="243">
-      <c r="A243" s="6" t="n"/>
-      <c r="B243" s="8" t="inlineStr">
-        <is>
-          <t>مركز الرضا للتخاطب وتنمية المهارات</t>
-        </is>
-      </c>
-      <c r="C243" s="8" t="inlineStr"/>
-      <c r="D243" s="9" t="inlineStr"/>
-      <c r="E243" s="9" t="inlineStr"/>
-      <c r="F243" s="8" t="inlineStr">
-        <is>
-          <t>شارع ترعة جزيرة بدران، قسم روض الفرج</t>
-        </is>
-      </c>
+      <c r="A243" s="5" t="n"/>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t>أوسيم</t>
+        </is>
+      </c>
+      <c r="C243" s="4" t="inlineStr"/>
+      <c r="D243" s="4" t="inlineStr"/>
+      <c r="E243" s="4" t="inlineStr"/>
+      <c r="F243" s="4" t="inlineStr"/>
+      <c r="G243" s="4" t="inlineStr"/>
     </row>
     <row r="244">
-      <c r="A244" s="7" t="inlineStr">
-        <is>
-          <t>المطرية</t>
-        </is>
-      </c>
-      <c r="B244" s="8" t="inlineStr">
-        <is>
-          <t>مركز التخاطب الشامل بالمطرية</t>
-        </is>
-      </c>
-      <c r="C244" s="8" t="inlineStr"/>
-      <c r="D244" s="9" t="inlineStr">
-        <is>
-          <t>01147626979</t>
-        </is>
-      </c>
-      <c r="E244" s="9" t="inlineStr"/>
-      <c r="F244" s="8" t="inlineStr">
-        <is>
-          <t>شارع منية مطر، بجوار محطة مترو المطرية</t>
-        </is>
-      </c>
+      <c r="A244" s="5" t="n"/>
+      <c r="B244" s="3" t="inlineStr">
+        <is>
+          <t>طره</t>
+        </is>
+      </c>
+      <c r="C244" s="4" t="inlineStr"/>
+      <c r="D244" s="4" t="inlineStr"/>
+      <c r="E244" s="4" t="inlineStr"/>
+      <c r="F244" s="4" t="inlineStr"/>
+      <c r="G244" s="4" t="inlineStr"/>
     </row>
     <row r="245">
-      <c r="A245" s="7" t="inlineStr">
-        <is>
-          <t>الدقي</t>
-        </is>
-      </c>
-      <c r="B245" s="8" t="inlineStr">
-        <is>
-          <t>مركز الحمد للعلاج الطبيعي والتخاطب - فرع الدقي</t>
-        </is>
-      </c>
-      <c r="C245" s="8" t="inlineStr"/>
-      <c r="D245" s="9" t="inlineStr"/>
-      <c r="E245" s="9" t="inlineStr"/>
-      <c r="F245" s="8" t="inlineStr">
-        <is>
-          <t>4 شارع Hussein Wassef، الدقي</t>
-        </is>
-      </c>
+      <c r="A245" s="5" t="n"/>
+      <c r="B245" s="3" t="inlineStr">
+        <is>
+          <t>الخصوص</t>
+        </is>
+      </c>
+      <c r="C245" s="4" t="inlineStr"/>
+      <c r="D245" s="4" t="inlineStr"/>
+      <c r="E245" s="4" t="inlineStr"/>
+      <c r="F245" s="4" t="inlineStr"/>
+      <c r="G245" s="4" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="6" t="n"/>
-      <c r="B246" s="8" t="inlineStr">
-        <is>
-          <t>مركز التخاطب - الدقي</t>
-        </is>
-      </c>
-      <c r="C246" s="8" t="inlineStr"/>
-      <c r="D246" s="9" t="inlineStr"/>
-      <c r="E246" s="9" t="inlineStr"/>
-      <c r="F246" s="8" t="inlineStr">
-        <is>
-          <t>110 شارع التحرير، الدقي، أمام محطة مترو الدقي</t>
-        </is>
-      </c>
+      <c r="B246" s="3" t="inlineStr">
+        <is>
+          <t>القنطرة</t>
+        </is>
+      </c>
+      <c r="C246" s="4" t="inlineStr"/>
+      <c r="D246" s="4" t="inlineStr"/>
+      <c r="E246" s="4" t="inlineStr"/>
+      <c r="F246" s="4" t="inlineStr"/>
+      <c r="G246" s="4" t="inlineStr"/>
     </row>
     <row r="247">
-      <c r="A247" s="7" t="inlineStr">
-        <is>
-          <t>الهرم</t>
-        </is>
-      </c>
-      <c r="B247" s="8" t="inlineStr">
-        <is>
-          <t>مركز هووب للتخاطب</t>
-        </is>
-      </c>
-      <c r="C247" s="8" t="inlineStr"/>
-      <c r="D247" s="9" t="inlineStr"/>
-      <c r="E247" s="9" t="inlineStr"/>
-      <c r="F247" s="8" t="inlineStr">
-        <is>
-          <t>الهرم، متخصص في التخاطب وتنمية المهارات</t>
-        </is>
-      </c>
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>المنوفية</t>
+        </is>
+      </c>
+      <c r="B247" s="3" t="inlineStr">
+        <is>
+          <t>شبين الكوم</t>
+        </is>
+      </c>
+      <c r="C247" s="4" t="inlineStr"/>
+      <c r="D247" s="4" t="inlineStr"/>
+      <c r="E247" s="4" t="inlineStr"/>
+      <c r="F247" s="4" t="inlineStr"/>
+      <c r="G247" s="4" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="5" t="n"/>
-      <c r="B248" s="8" t="inlineStr">
-        <is>
-          <t>مركز فرصة حياه للتأهيل للتخاطب وتنمية المهارات</t>
-        </is>
-      </c>
-      <c r="C248" s="8" t="inlineStr"/>
-      <c r="D248" s="9" t="inlineStr">
-        <is>
-          <t>01030360536</t>
-        </is>
-      </c>
-      <c r="E248" s="9" t="inlineStr"/>
-      <c r="F248" s="8" t="inlineStr">
-        <is>
-          <t>الهرم وفيصل</t>
-        </is>
-      </c>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t>منوف</t>
+        </is>
+      </c>
+      <c r="C248" s="4" t="inlineStr"/>
+      <c r="D248" s="4" t="inlineStr"/>
+      <c r="E248" s="4" t="inlineStr"/>
+      <c r="F248" s="4" t="inlineStr"/>
+      <c r="G248" s="4" t="inlineStr"/>
     </row>
     <row r="249">
-      <c r="A249" s="6" t="n"/>
-      <c r="B249" s="8" t="inlineStr">
-        <is>
-          <t>مركز اشراقة للتخاطب - د/اسلام سالم</t>
-        </is>
-      </c>
-      <c r="C249" s="8" t="inlineStr">
-        <is>
-          <t>د/اسلام سالم</t>
-        </is>
-      </c>
-      <c r="D249" s="9" t="inlineStr"/>
-      <c r="E249" s="9" t="inlineStr"/>
-      <c r="F249" s="8" t="inlineStr">
-        <is>
-          <t>شارع اللبيني، الهرم الرئيسي</t>
-        </is>
-      </c>
+      <c r="A249" s="5" t="n"/>
+      <c r="B249" s="3" t="inlineStr">
+        <is>
+          <t>شبين القناطر</t>
+        </is>
+      </c>
+      <c r="C249" s="4" t="inlineStr"/>
+      <c r="D249" s="4" t="inlineStr"/>
+      <c r="E249" s="4" t="inlineStr"/>
+      <c r="F249" s="4" t="inlineStr"/>
+      <c r="G249" s="4" t="inlineStr"/>
     </row>
     <row r="250">
-      <c r="A250" s="7" t="inlineStr">
-        <is>
-          <t>النزهة</t>
-        </is>
-      </c>
-      <c r="B250" s="8" t="inlineStr">
-        <is>
-          <t>مركز الشمس للتخاطب - فرع النزهة</t>
-        </is>
-      </c>
-      <c r="C250" s="8" t="inlineStr"/>
-      <c r="D250" s="9" t="inlineStr"/>
-      <c r="E250" s="9" t="inlineStr"/>
-      <c r="F250" s="8" t="inlineStr">
-        <is>
-          <t>النزهة</t>
-        </is>
-      </c>
+      <c r="A250" s="5" t="n"/>
+      <c r="B250" s="3" t="inlineStr">
+        <is>
+          <t>مدينة السادات</t>
+        </is>
+      </c>
+      <c r="C250" s="4" t="inlineStr"/>
+      <c r="D250" s="4" t="inlineStr"/>
+      <c r="E250" s="4" t="inlineStr"/>
+      <c r="F250" s="4" t="inlineStr"/>
+      <c r="G250" s="4" t="inlineStr"/>
     </row>
     <row r="251">
-      <c r="A251" s="6" t="n"/>
-      <c r="B251" s="8" t="inlineStr">
-        <is>
-          <t>نور الحياة للتخاطب</t>
-        </is>
-      </c>
-      <c r="C251" s="8" t="inlineStr"/>
-      <c r="D251" s="9" t="inlineStr"/>
-      <c r="E251" s="9" t="inlineStr"/>
-      <c r="F251" s="8" t="inlineStr">
-        <is>
-          <t>شارع شبرا الخلفاوى، قسم الساحل</t>
-        </is>
-      </c>
+      <c r="A251" s="5" t="n"/>
+      <c r="B251" s="3" t="inlineStr">
+        <is>
+          <t>باقور</t>
+        </is>
+      </c>
+      <c r="C251" s="4" t="inlineStr"/>
+      <c r="D251" s="4" t="inlineStr"/>
+      <c r="E251" s="4" t="inlineStr"/>
+      <c r="F251" s="4" t="inlineStr"/>
+      <c r="G251" s="4" t="inlineStr"/>
     </row>
     <row r="252">
-      <c r="A252" s="7" t="inlineStr">
-        <is>
-          <t>الزيتون</t>
-        </is>
-      </c>
-      <c r="B252" s="8" t="inlineStr">
-        <is>
-          <t>مركز التخاطب الشامل - فرع الزيتون</t>
-        </is>
-      </c>
-      <c r="C252" s="8" t="inlineStr"/>
-      <c r="D252" s="9" t="inlineStr">
-        <is>
-          <t>0222406301</t>
-        </is>
-      </c>
-      <c r="E252" s="9" t="inlineStr"/>
-      <c r="F252" s="8" t="inlineStr">
-        <is>
-          <t>حي الزيتون</t>
-        </is>
-      </c>
+      <c r="A252" s="5" t="n"/>
+      <c r="B252" s="3" t="inlineStr">
+        <is>
+          <t>تلا</t>
+        </is>
+      </c>
+      <c r="C252" s="4" t="inlineStr"/>
+      <c r="D252" s="4" t="inlineStr"/>
+      <c r="E252" s="4" t="inlineStr"/>
+      <c r="F252" s="4" t="inlineStr"/>
+      <c r="G252" s="4" t="inlineStr"/>
     </row>
     <row r="253">
-      <c r="A253" s="7" t="inlineStr">
-        <is>
-          <t>عين شمس</t>
-        </is>
-      </c>
-      <c r="B253" s="8" t="inlineStr">
-        <is>
-          <t>مركز الشمس للتخاطب - فرع عين شمس</t>
-        </is>
-      </c>
-      <c r="C253" s="8" t="inlineStr"/>
-      <c r="D253" s="9" t="inlineStr"/>
-      <c r="E253" s="9" t="inlineStr"/>
-      <c r="F253" s="8" t="inlineStr">
-        <is>
-          <t>عين شمس</t>
-        </is>
-      </c>
+      <c r="A253" s="5" t="n"/>
+      <c r="B253" s="3" t="inlineStr">
+        <is>
+          <t>قويسنا</t>
+        </is>
+      </c>
+      <c r="C253" s="4" t="inlineStr"/>
+      <c r="D253" s="4" t="inlineStr"/>
+      <c r="E253" s="4" t="inlineStr"/>
+      <c r="F253" s="4" t="inlineStr"/>
+      <c r="G253" s="4" t="inlineStr"/>
     </row>
     <row r="254">
-      <c r="A254" s="7" t="inlineStr">
-        <is>
-          <t>فيصل</t>
-        </is>
-      </c>
-      <c r="B254" s="8" t="inlineStr">
-        <is>
-          <t>مركز فرصة حياه - فرع فيصل</t>
-        </is>
-      </c>
-      <c r="C254" s="8" t="inlineStr"/>
-      <c r="D254" s="9" t="inlineStr">
-        <is>
-          <t>01030360536</t>
-        </is>
-      </c>
-      <c r="E254" s="9" t="inlineStr"/>
-      <c r="F254" s="8" t="inlineStr">
-        <is>
-          <t>فيصل</t>
+      <c r="A254" s="5" t="n"/>
+      <c r="B254" s="3" t="inlineStr">
+        <is>
+          <t>أشمون</t>
+        </is>
+      </c>
+      <c r="C254" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب أشمون للتخاطب</t>
+        </is>
+      </c>
+      <c r="D254" s="4" t="inlineStr"/>
+      <c r="E254" s="4" t="inlineStr"/>
+      <c r="F254" s="4" t="inlineStr"/>
+      <c r="G254" s="4" t="inlineStr">
+        <is>
+          <t>أشمون</t>
         </is>
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="2" t="inlineStr">
-        <is>
-          <t>القليوبية</t>
-        </is>
-      </c>
+      <c r="A255" s="5" t="n"/>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>بنها</t>
-        </is>
-      </c>
-      <c r="C255" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب برج مكة</t>
-        </is>
-      </c>
+          <t>البرجايه</t>
+        </is>
+      </c>
+      <c r="C255" s="4" t="inlineStr"/>
       <c r="D255" s="4" t="inlineStr"/>
       <c r="E255" s="4" t="inlineStr"/>
       <c r="F255" s="4" t="inlineStr"/>
-      <c r="G255" s="4" t="inlineStr">
-        <is>
-          <t>شارع جميل أمام بنك القاهرة</t>
-        </is>
-      </c>
+      <c r="G255" s="4" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="5" t="n"/>
-      <c r="B256" s="5" t="n"/>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t>بركة السبع</t>
+        </is>
+      </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
-          <t>مركز شباب كفر الجزار</t>
+          <t>مركز تخاطب وصعوبات تعلم</t>
         </is>
       </c>
       <c r="D256" s="4" t="inlineStr"/>
@@ -4563,32 +4420,28 @@
       <c r="F256" s="4" t="inlineStr"/>
       <c r="G256" s="4" t="inlineStr">
         <is>
-          <t>بنها</t>
+          <t>بركة السبع</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="5" t="n"/>
-      <c r="B257" s="6" t="n"/>
-      <c r="C257" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب العمار</t>
-        </is>
-      </c>
+      <c r="B257" s="3" t="inlineStr">
+        <is>
+          <t>منوف الجديدة</t>
+        </is>
+      </c>
+      <c r="C257" s="4" t="inlineStr"/>
       <c r="D257" s="4" t="inlineStr"/>
       <c r="E257" s="4" t="inlineStr"/>
       <c r="F257" s="4" t="inlineStr"/>
-      <c r="G257" s="4" t="inlineStr">
-        <is>
-          <t>بنها</t>
-        </is>
-      </c>
+      <c r="G257" s="4" t="inlineStr"/>
     </row>
     <row r="258">
-      <c r="A258" s="5" t="n"/>
+      <c r="A258" s="6" t="n"/>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>قليوب</t>
+          <t>كفر عبده</t>
         </is>
       </c>
       <c r="C258" s="4" t="inlineStr"/>
@@ -4598,15 +4451,19 @@
       <c r="G258" s="4" t="inlineStr"/>
     </row>
     <row r="259">
-      <c r="A259" s="5" t="n"/>
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>المنيا</t>
+        </is>
+      </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>شبرا الخيمة</t>
+          <t>المنيا</t>
         </is>
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>مركز الغد للتخاطب وصعوبات التعلم</t>
+          <t>مركز شباب بني أحمد للتخاطب</t>
         </is>
       </c>
       <c r="D259" s="4" t="inlineStr"/>
@@ -4614,16 +4471,16 @@
       <c r="F259" s="4" t="inlineStr"/>
       <c r="G259" s="4" t="inlineStr">
         <is>
-          <t>75 شارع حنفي الشيخوني</t>
+          <t>المنيا</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="5" t="n"/>
-      <c r="B260" s="5" t="n"/>
+      <c r="B260" s="6" t="n"/>
       <c r="C260" s="4" t="inlineStr">
         <is>
-          <t>مركز النور الهدى الطبي</t>
+          <t>مركز شباب مقوسة للتخاطب</t>
         </is>
       </c>
       <c r="D260" s="4" t="inlineStr"/>
@@ -4631,32 +4488,28 @@
       <c r="F260" s="4" t="inlineStr"/>
       <c r="G260" s="4" t="inlineStr">
         <is>
-          <t>شارع محمد القطان</t>
+          <t>المنيا</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="5" t="n"/>
-      <c r="B261" s="6" t="n"/>
-      <c r="C261" s="4" t="inlineStr">
-        <is>
-          <t>مركز تواصل للتخاطب</t>
-        </is>
-      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
+          <t>سمالوط</t>
+        </is>
+      </c>
+      <c r="C261" s="4" t="inlineStr"/>
       <c r="D261" s="4" t="inlineStr"/>
       <c r="E261" s="4" t="inlineStr"/>
       <c r="F261" s="4" t="inlineStr"/>
-      <c r="G261" s="4" t="inlineStr">
-        <is>
-          <t>2 شارع أحمد عبد ربه</t>
-        </is>
-      </c>
+      <c r="G261" s="4" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="5" t="n"/>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>الخانكة</t>
+          <t>بني حسن</t>
         </is>
       </c>
       <c r="C262" s="4" t="inlineStr"/>
@@ -4669,7 +4522,7 @@
       <c r="A263" s="5" t="n"/>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>رمسيس</t>
+          <t>هرموبوليس</t>
         </is>
       </c>
       <c r="C263" s="4" t="inlineStr"/>
@@ -4682,7 +4535,7 @@
       <c r="A264" s="5" t="n"/>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>مدينة 10 رمضان</t>
+          <t>ملوي</t>
         </is>
       </c>
       <c r="C264" s="4" t="inlineStr"/>
@@ -4695,7 +4548,7 @@
       <c r="A265" s="5" t="n"/>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>الشيخ زايد</t>
+          <t>العدوة</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr"/>
@@ -4708,7 +4561,7 @@
       <c r="A266" s="5" t="n"/>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>القناطر الخيرية</t>
+          <t>ديروط الشريف</t>
         </is>
       </c>
       <c r="C266" s="4" t="inlineStr"/>
@@ -4721,7 +4574,7 @@
       <c r="A267" s="5" t="n"/>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>قها</t>
+          <t>أبوقرقاص</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr"/>
@@ -4734,7 +4587,7 @@
       <c r="A268" s="5" t="n"/>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>الدقهلية</t>
+          <t>الفشن</t>
         </is>
       </c>
       <c r="C268" s="4" t="inlineStr"/>
@@ -4747,7 +4600,7 @@
       <c r="A269" s="5" t="n"/>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>الجيزة</t>
+          <t>بني مازن</t>
         </is>
       </c>
       <c r="C269" s="4" t="inlineStr"/>
@@ -4757,10 +4610,10 @@
       <c r="G269" s="4" t="inlineStr"/>
     </row>
     <row r="270">
-      <c r="A270" s="5" t="n"/>
+      <c r="A270" s="6" t="n"/>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>أوسيم</t>
+          <t>العدوة</t>
         </is>
       </c>
       <c r="C270" s="4" t="inlineStr"/>
@@ -4770,36 +4623,56 @@
       <c r="G270" s="4" t="inlineStr"/>
     </row>
     <row r="271">
-      <c r="A271" s="5" t="n"/>
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>الوادي الجديد</t>
+        </is>
+      </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>طره</t>
-        </is>
-      </c>
-      <c r="C271" s="4" t="inlineStr"/>
+          <t>الخارجة</t>
+        </is>
+      </c>
+      <c r="C271" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب الخارجة للتخاطب</t>
+        </is>
+      </c>
       <c r="D271" s="4" t="inlineStr"/>
       <c r="E271" s="4" t="inlineStr"/>
       <c r="F271" s="4" t="inlineStr"/>
-      <c r="G271" s="4" t="inlineStr"/>
+      <c r="G271" s="4" t="inlineStr">
+        <is>
+          <t>الخارجة</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="5" t="n"/>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>الخصوص</t>
-        </is>
-      </c>
-      <c r="C272" s="4" t="inlineStr"/>
+          <t>الداخلة</t>
+        </is>
+      </c>
+      <c r="C272" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب باريس للتخاطب</t>
+        </is>
+      </c>
       <c r="D272" s="4" t="inlineStr"/>
       <c r="E272" s="4" t="inlineStr"/>
       <c r="F272" s="4" t="inlineStr"/>
-      <c r="G272" s="4" t="inlineStr"/>
+      <c r="G272" s="4" t="inlineStr">
+        <is>
+          <t>باريس</t>
+        </is>
+      </c>
     </row>
     <row r="273">
-      <c r="A273" s="6" t="n"/>
+      <c r="A273" s="5" t="n"/>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>القنطرة</t>
+          <t>موط</t>
         </is>
       </c>
       <c r="C273" s="4" t="inlineStr"/>
@@ -4809,14 +4682,10 @@
       <c r="G273" s="4" t="inlineStr"/>
     </row>
     <row r="274">
-      <c r="A274" s="2" t="inlineStr">
-        <is>
-          <t>المنوفية</t>
-        </is>
-      </c>
+      <c r="A274" s="5" t="n"/>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>شبين الكوم</t>
+          <t>بلاط</t>
         </is>
       </c>
       <c r="C274" s="4" t="inlineStr"/>
@@ -4829,7 +4698,7 @@
       <c r="A275" s="5" t="n"/>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>منوف</t>
+          <t>فرافرة</t>
         </is>
       </c>
       <c r="C275" s="4" t="inlineStr"/>
@@ -4842,7 +4711,7 @@
       <c r="A276" s="5" t="n"/>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>شبين القناطر</t>
+          <t>باريس</t>
         </is>
       </c>
       <c r="C276" s="4" t="inlineStr"/>
@@ -4855,7 +4724,7 @@
       <c r="A277" s="5" t="n"/>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>مدينة السادات</t>
+          <t>القصر</t>
         </is>
       </c>
       <c r="C277" s="4" t="inlineStr"/>
@@ -4868,7 +4737,7 @@
       <c r="A278" s="5" t="n"/>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>باقور</t>
+          <t>تينيدة</t>
         </is>
       </c>
       <c r="C278" s="4" t="inlineStr"/>
@@ -4878,10 +4747,10 @@
       <c r="G278" s="4" t="inlineStr"/>
     </row>
     <row r="279">
-      <c r="A279" s="5" t="n"/>
+      <c r="A279" s="6" t="n"/>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>تلا</t>
+          <t>دوش</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr"/>
@@ -4891,44 +4760,48 @@
       <c r="G279" s="4" t="inlineStr"/>
     </row>
     <row r="280">
-      <c r="A280" s="5" t="n"/>
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>بني سويف</t>
+        </is>
+      </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>قويسنا</t>
-        </is>
-      </c>
-      <c r="C280" s="4" t="inlineStr"/>
+          <t>بني سويف</t>
+        </is>
+      </c>
+      <c r="C280" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب العبور للتخاطب</t>
+        </is>
+      </c>
       <c r="D280" s="4" t="inlineStr"/>
       <c r="E280" s="4" t="inlineStr"/>
       <c r="F280" s="4" t="inlineStr"/>
-      <c r="G280" s="4" t="inlineStr"/>
+      <c r="G280" s="4" t="inlineStr">
+        <is>
+          <t>بني سويف</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="5" t="n"/>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>أشمون</t>
-        </is>
-      </c>
-      <c r="C281" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب أشمون للتخاطب</t>
-        </is>
-      </c>
+          <t>الفشن</t>
+        </is>
+      </c>
+      <c r="C281" s="4" t="inlineStr"/>
       <c r="D281" s="4" t="inlineStr"/>
       <c r="E281" s="4" t="inlineStr"/>
       <c r="F281" s="4" t="inlineStr"/>
-      <c r="G281" s="4" t="inlineStr">
-        <is>
-          <t>أشمون</t>
-        </is>
-      </c>
+      <c r="G281" s="4" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" s="5" t="n"/>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>البرجايه</t>
+          <t>ساماستا</t>
         </is>
       </c>
       <c r="C282" s="4" t="inlineStr"/>
@@ -4941,28 +4814,20 @@
       <c r="A283" s="5" t="n"/>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>بركة السبع</t>
-        </is>
-      </c>
-      <c r="C283" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب وصعوبات تعلم</t>
-        </is>
-      </c>
+          <t>إبشواي</t>
+        </is>
+      </c>
+      <c r="C283" s="4" t="inlineStr"/>
       <c r="D283" s="4" t="inlineStr"/>
       <c r="E283" s="4" t="inlineStr"/>
       <c r="F283" s="4" t="inlineStr"/>
-      <c r="G283" s="4" t="inlineStr">
-        <is>
-          <t>بركة السبع</t>
-        </is>
-      </c>
+      <c r="G283" s="4" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" s="5" t="n"/>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>منوف الجديدة</t>
+          <t>الجندية</t>
         </is>
       </c>
       <c r="C284" s="4" t="inlineStr"/>
@@ -4972,10 +4837,10 @@
       <c r="G284" s="4" t="inlineStr"/>
     </row>
     <row r="285">
-      <c r="A285" s="6" t="n"/>
+      <c r="A285" s="5" t="n"/>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>كفر عبده</t>
+          <t>ناصر</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr"/>
@@ -4985,52 +4850,36 @@
       <c r="G285" s="4" t="inlineStr"/>
     </row>
     <row r="286">
-      <c r="A286" s="2" t="inlineStr">
-        <is>
-          <t>المنيا</t>
-        </is>
-      </c>
+      <c r="A286" s="5" t="n"/>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>المنيا</t>
-        </is>
-      </c>
-      <c r="C286" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب بني أحمد للتخاطب</t>
-        </is>
-      </c>
+          <t>هواره</t>
+        </is>
+      </c>
+      <c r="C286" s="4" t="inlineStr"/>
       <c r="D286" s="4" t="inlineStr"/>
       <c r="E286" s="4" t="inlineStr"/>
       <c r="F286" s="4" t="inlineStr"/>
-      <c r="G286" s="4" t="inlineStr">
-        <is>
-          <t>المنيا</t>
-        </is>
-      </c>
+      <c r="G286" s="4" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" s="5" t="n"/>
-      <c r="B287" s="6" t="n"/>
-      <c r="C287" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب مقوسة للتخاطب</t>
-        </is>
-      </c>
+      <c r="B287" s="3" t="inlineStr">
+        <is>
+          <t>موشية</t>
+        </is>
+      </c>
+      <c r="C287" s="4" t="inlineStr"/>
       <c r="D287" s="4" t="inlineStr"/>
       <c r="E287" s="4" t="inlineStr"/>
       <c r="F287" s="4" t="inlineStr"/>
-      <c r="G287" s="4" t="inlineStr">
-        <is>
-          <t>المنيا</t>
-        </is>
-      </c>
+      <c r="G287" s="4" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" s="5" t="n"/>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>سمالوط</t>
+          <t>نصار البحرية</t>
         </is>
       </c>
       <c r="C288" s="4" t="inlineStr"/>
@@ -5040,10 +4889,10 @@
       <c r="G288" s="4" t="inlineStr"/>
     </row>
     <row r="289">
-      <c r="A289" s="5" t="n"/>
+      <c r="A289" s="6" t="n"/>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>بني حسن</t>
+          <t>أحمد حمزة</t>
         </is>
       </c>
       <c r="C289" s="4" t="inlineStr"/>
@@ -5053,10 +4902,14 @@
       <c r="G289" s="4" t="inlineStr"/>
     </row>
     <row r="290">
-      <c r="A290" s="5" t="n"/>
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>بورسعيد</t>
+        </is>
+      </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>هرموبوليس</t>
+          <t>بورسعيد</t>
         </is>
       </c>
       <c r="C290" s="4" t="inlineStr"/>
@@ -5069,7 +4922,7 @@
       <c r="A291" s="5" t="n"/>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>ملوي</t>
+          <t>بورفؤاد</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr"/>
@@ -5082,7 +4935,7 @@
       <c r="A292" s="5" t="n"/>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>العدوة</t>
+          <t>الجميل</t>
         </is>
       </c>
       <c r="C292" s="4" t="inlineStr"/>
@@ -5095,7 +4948,7 @@
       <c r="A293" s="5" t="n"/>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>ديروط الشريف</t>
+          <t>الزهور</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr"/>
@@ -5108,7 +4961,7 @@
       <c r="A294" s="5" t="n"/>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>أبوقرقاص</t>
+          <t>بورسعيد</t>
         </is>
       </c>
       <c r="C294" s="4" t="inlineStr"/>
@@ -5121,7 +4974,7 @@
       <c r="A295" s="5" t="n"/>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>الفشن</t>
+          <t>الكنتاوي</t>
         </is>
       </c>
       <c r="C295" s="4" t="inlineStr"/>
@@ -5131,10 +4984,10 @@
       <c r="G295" s="4" t="inlineStr"/>
     </row>
     <row r="296">
-      <c r="A296" s="5" t="n"/>
+      <c r="A296" s="6" t="n"/>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>بني مازن</t>
+          <t>الضواحي</t>
         </is>
       </c>
       <c r="C296" s="4" t="inlineStr"/>
@@ -5144,10 +4997,14 @@
       <c r="G296" s="4" t="inlineStr"/>
     </row>
     <row r="297">
-      <c r="A297" s="6" t="n"/>
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>جنوب سيناء</t>
+        </is>
+      </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>العدوة</t>
+          <t>شرم الشيخ</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr"/>
@@ -5157,56 +5014,36 @@
       <c r="G297" s="4" t="inlineStr"/>
     </row>
     <row r="298">
-      <c r="A298" s="2" t="inlineStr">
-        <is>
-          <t>الوادي الجديد</t>
-        </is>
-      </c>
+      <c r="A298" s="5" t="n"/>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>الخارجة</t>
-        </is>
-      </c>
-      <c r="C298" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب الخارجة للتخاطب</t>
-        </is>
-      </c>
+          <t>داهب</t>
+        </is>
+      </c>
+      <c r="C298" s="4" t="inlineStr"/>
       <c r="D298" s="4" t="inlineStr"/>
       <c r="E298" s="4" t="inlineStr"/>
       <c r="F298" s="4" t="inlineStr"/>
-      <c r="G298" s="4" t="inlineStr">
-        <is>
-          <t>الخارجة</t>
-        </is>
-      </c>
+      <c r="G298" s="4" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" s="5" t="n"/>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>الداخلة</t>
-        </is>
-      </c>
-      <c r="C299" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب باريس للتخاطب</t>
-        </is>
-      </c>
+          <t>نويبع</t>
+        </is>
+      </c>
+      <c r="C299" s="4" t="inlineStr"/>
       <c r="D299" s="4" t="inlineStr"/>
       <c r="E299" s="4" t="inlineStr"/>
       <c r="F299" s="4" t="inlineStr"/>
-      <c r="G299" s="4" t="inlineStr">
-        <is>
-          <t>باريس</t>
-        </is>
-      </c>
+      <c r="G299" s="4" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" s="5" t="n"/>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>موط</t>
+          <t>سانت كاترين</t>
         </is>
       </c>
       <c r="C300" s="4" t="inlineStr"/>
@@ -5219,7 +5056,7 @@
       <c r="A301" s="5" t="n"/>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>بلاط</t>
+          <t>طابا</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr"/>
@@ -5232,7 +5069,7 @@
       <c r="A302" s="5" t="n"/>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>فرافرة</t>
+          <t>رأس محمد</t>
         </is>
       </c>
       <c r="C302" s="4" t="inlineStr"/>
@@ -5245,7 +5082,7 @@
       <c r="A303" s="5" t="n"/>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>باريس</t>
+          <t>أم سيد</t>
         </is>
       </c>
       <c r="C303" s="4" t="inlineStr"/>
@@ -5255,10 +5092,10 @@
       <c r="G303" s="4" t="inlineStr"/>
     </row>
     <row r="304">
-      <c r="A304" s="5" t="n"/>
+      <c r="A304" s="6" t="n"/>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>القصر</t>
+          <t>مدينة شرم الشيخ</t>
         </is>
       </c>
       <c r="C304" s="4" t="inlineStr"/>
@@ -5268,10 +5105,14 @@
       <c r="G304" s="4" t="inlineStr"/>
     </row>
     <row r="305">
-      <c r="A305" s="5" t="n"/>
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>حلوان</t>
+        </is>
+      </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>تينيدة</t>
+          <t>حلوان</t>
         </is>
       </c>
       <c r="C305" s="4" t="inlineStr"/>
@@ -5281,10 +5122,10 @@
       <c r="G305" s="4" t="inlineStr"/>
     </row>
     <row r="306">
-      <c r="A306" s="6" t="n"/>
+      <c r="A306" s="5" t="n"/>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>دوش</t>
+          <t>المعادي</t>
         </is>
       </c>
       <c r="C306" s="4" t="inlineStr"/>
@@ -5294,35 +5135,23 @@
       <c r="G306" s="4" t="inlineStr"/>
     </row>
     <row r="307">
-      <c r="A307" s="2" t="inlineStr">
-        <is>
-          <t>بني سويف</t>
-        </is>
-      </c>
+      <c r="A307" s="5" t="n"/>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>بني سويف</t>
-        </is>
-      </c>
-      <c r="C307" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب العبور للتخاطب</t>
-        </is>
-      </c>
+          <t>واحة الفيوم</t>
+        </is>
+      </c>
+      <c r="C307" s="4" t="inlineStr"/>
       <c r="D307" s="4" t="inlineStr"/>
       <c r="E307" s="4" t="inlineStr"/>
       <c r="F307" s="4" t="inlineStr"/>
-      <c r="G307" s="4" t="inlineStr">
-        <is>
-          <t>بني سويف</t>
-        </is>
-      </c>
+      <c r="G307" s="4" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" s="5" t="n"/>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>الفشن</t>
+          <t>وادي حوف</t>
         </is>
       </c>
       <c r="C308" s="4" t="inlineStr"/>
@@ -5335,7 +5164,7 @@
       <c r="A309" s="5" t="n"/>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>ساماستا</t>
+          <t>عين سخنة</t>
         </is>
       </c>
       <c r="C309" s="4" t="inlineStr"/>
@@ -5348,7 +5177,7 @@
       <c r="A310" s="5" t="n"/>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>إبشواي</t>
+          <t>الطور</t>
         </is>
       </c>
       <c r="C310" s="4" t="inlineStr"/>
@@ -5361,7 +5190,7 @@
       <c r="A311" s="5" t="n"/>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>الجندية</t>
+          <t>الزيتون</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr"/>
@@ -5371,10 +5200,10 @@
       <c r="G311" s="4" t="inlineStr"/>
     </row>
     <row r="312">
-      <c r="A312" s="5" t="n"/>
+      <c r="A312" s="6" t="n"/>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>ناصر</t>
+          <t>المقطم</t>
         </is>
       </c>
       <c r="C312" s="4" t="inlineStr"/>
@@ -5384,23 +5213,35 @@
       <c r="G312" s="4" t="inlineStr"/>
     </row>
     <row r="313">
-      <c r="A313" s="5" t="n"/>
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>دمياط</t>
+        </is>
+      </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>هواره</t>
-        </is>
-      </c>
-      <c r="C313" s="4" t="inlineStr"/>
+          <t>دمياط</t>
+        </is>
+      </c>
+      <c r="C313" s="4" t="inlineStr">
+        <is>
+          <t>مركز حلم ابني للتخاطب</t>
+        </is>
+      </c>
       <c r="D313" s="4" t="inlineStr"/>
       <c r="E313" s="4" t="inlineStr"/>
       <c r="F313" s="4" t="inlineStr"/>
-      <c r="G313" s="4" t="inlineStr"/>
+      <c r="G313" s="4" t="inlineStr">
+        <is>
+          <t>دمياط ودمياط الجديدة</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="5" t="n"/>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>موشية</t>
+          <t>دمياط الجديدة</t>
         </is>
       </c>
       <c r="C314" s="4" t="inlineStr"/>
@@ -5413,7 +5254,7 @@
       <c r="A315" s="5" t="n"/>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>نصار البحرية</t>
+          <t>بورت فؤاد</t>
         </is>
       </c>
       <c r="C315" s="4" t="inlineStr"/>
@@ -5423,10 +5264,10 @@
       <c r="G315" s="4" t="inlineStr"/>
     </row>
     <row r="316">
-      <c r="A316" s="6" t="n"/>
+      <c r="A316" s="5" t="n"/>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>أحمد حمزة</t>
+          <t>كفر البطة</t>
         </is>
       </c>
       <c r="C316" s="4" t="inlineStr"/>
@@ -5436,14 +5277,10 @@
       <c r="G316" s="4" t="inlineStr"/>
     </row>
     <row r="317">
-      <c r="A317" s="2" t="inlineStr">
-        <is>
-          <t>بورسعيد</t>
-        </is>
-      </c>
+      <c r="A317" s="5" t="n"/>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>بورسعيد</t>
+          <t>كفر سعيد</t>
         </is>
       </c>
       <c r="C317" s="4" t="inlineStr"/>
@@ -5456,7 +5293,7 @@
       <c r="A318" s="5" t="n"/>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>بورفؤاد</t>
+          <t>الروضة</t>
         </is>
       </c>
       <c r="C318" s="4" t="inlineStr"/>
@@ -5469,7 +5306,7 @@
       <c r="A319" s="5" t="n"/>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>الجميل</t>
+          <t>الزرقا</t>
         </is>
       </c>
       <c r="C319" s="4" t="inlineStr"/>
@@ -5482,7 +5319,7 @@
       <c r="A320" s="5" t="n"/>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>الزهور</t>
+          <t>فارسكور</t>
         </is>
       </c>
       <c r="C320" s="4" t="inlineStr"/>
@@ -5492,10 +5329,10 @@
       <c r="G320" s="4" t="inlineStr"/>
     </row>
     <row r="321">
-      <c r="A321" s="5" t="n"/>
+      <c r="A321" s="6" t="n"/>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>بورسعيد</t>
+          <t>رومانية</t>
         </is>
       </c>
       <c r="C321" s="4" t="inlineStr"/>
@@ -5505,53 +5342,77 @@
       <c r="G321" s="4" t="inlineStr"/>
     </row>
     <row r="322">
-      <c r="A322" s="5" t="n"/>
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>شمال سيناء</t>
+        </is>
+      </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>الكنتاوي</t>
-        </is>
-      </c>
-      <c r="C322" s="4" t="inlineStr"/>
+          <t>العريش</t>
+        </is>
+      </c>
+      <c r="C322" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب العريش للتخاطب</t>
+        </is>
+      </c>
       <c r="D322" s="4" t="inlineStr"/>
       <c r="E322" s="4" t="inlineStr"/>
       <c r="F322" s="4" t="inlineStr"/>
-      <c r="G322" s="4" t="inlineStr"/>
+      <c r="G322" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب العريش</t>
+        </is>
+      </c>
     </row>
     <row r="323">
-      <c r="A323" s="6" t="n"/>
+      <c r="A323" s="5" t="n"/>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>الضواحي</t>
-        </is>
-      </c>
-      <c r="C323" s="4" t="inlineStr"/>
+          <t>رفح</t>
+        </is>
+      </c>
+      <c r="C323" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب رفح</t>
+        </is>
+      </c>
       <c r="D323" s="4" t="inlineStr"/>
       <c r="E323" s="4" t="inlineStr"/>
       <c r="F323" s="4" t="inlineStr"/>
-      <c r="G323" s="4" t="inlineStr"/>
+      <c r="G323" s="4" t="inlineStr">
+        <is>
+          <t>رفح</t>
+        </is>
+      </c>
     </row>
     <row r="324">
-      <c r="A324" s="2" t="inlineStr">
-        <is>
-          <t>جنوب سيناء</t>
-        </is>
-      </c>
+      <c r="A324" s="5" t="n"/>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>شرم الشيخ</t>
-        </is>
-      </c>
-      <c r="C324" s="4" t="inlineStr"/>
+          <t>الشيخ زويد</t>
+        </is>
+      </c>
+      <c r="C324" s="4" t="inlineStr">
+        <is>
+          <t>مركز تخاطب الشيخ زويد (قيد الإنشاء)</t>
+        </is>
+      </c>
       <c r="D324" s="4" t="inlineStr"/>
       <c r="E324" s="4" t="inlineStr"/>
       <c r="F324" s="4" t="inlineStr"/>
-      <c r="G324" s="4" t="inlineStr"/>
+      <c r="G324" s="4" t="inlineStr">
+        <is>
+          <t>الشيخ زويد</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="5" t="n"/>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>داهب</t>
+          <t>بئر العبد</t>
         </is>
       </c>
       <c r="C325" s="4" t="inlineStr"/>
@@ -5564,7 +5425,7 @@
       <c r="A326" s="5" t="n"/>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>نويبع</t>
+          <t>القنطرة، سيناء</t>
         </is>
       </c>
       <c r="C326" s="4" t="inlineStr"/>
@@ -5577,7 +5438,7 @@
       <c r="A327" s="5" t="n"/>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>سانت كاترين</t>
+          <t>نخل</t>
         </is>
       </c>
       <c r="C327" s="4" t="inlineStr"/>
@@ -5590,7 +5451,7 @@
       <c r="A328" s="5" t="n"/>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>طابا</t>
+          <t>جديدة، حسنة</t>
         </is>
       </c>
       <c r="C328" s="4" t="inlineStr"/>
@@ -5603,7 +5464,7 @@
       <c r="A329" s="5" t="n"/>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>رأس محمد</t>
+          <t>دهب الشرقية</t>
         </is>
       </c>
       <c r="C329" s="4" t="inlineStr"/>
@@ -5613,10 +5474,10 @@
       <c r="G329" s="4" t="inlineStr"/>
     </row>
     <row r="330">
-      <c r="A330" s="5" t="n"/>
+      <c r="A330" s="6" t="n"/>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>أم سيد</t>
+          <t>طابا</t>
         </is>
       </c>
       <c r="C330" s="4" t="inlineStr"/>
@@ -5626,40 +5487,52 @@
       <c r="G330" s="4" t="inlineStr"/>
     </row>
     <row r="331">
-      <c r="A331" s="6" t="n"/>
+      <c r="A331" s="2" t="inlineStr">
+        <is>
+          <t>قنا</t>
+        </is>
+      </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>مدينة شرم الشيخ</t>
-        </is>
-      </c>
-      <c r="C331" s="4" t="inlineStr"/>
+          <t>قنا</t>
+        </is>
+      </c>
+      <c r="C331" s="4" t="inlineStr">
+        <is>
+          <t>مركز التخاطب بمدينة العمال</t>
+        </is>
+      </c>
       <c r="D331" s="4" t="inlineStr"/>
       <c r="E331" s="4" t="inlineStr"/>
       <c r="F331" s="4" t="inlineStr"/>
-      <c r="G331" s="4" t="inlineStr"/>
+      <c r="G331" s="4" t="inlineStr">
+        <is>
+          <t>مدينة العمال، قنا</t>
+        </is>
+      </c>
     </row>
     <row r="332">
-      <c r="A332" s="2" t="inlineStr">
-        <is>
-          <t>حلوان</t>
-        </is>
-      </c>
-      <c r="B332" s="3" t="inlineStr">
-        <is>
-          <t>حلوان</t>
-        </is>
-      </c>
-      <c r="C332" s="4" t="inlineStr"/>
+      <c r="A332" s="5" t="n"/>
+      <c r="B332" s="6" t="n"/>
+      <c r="C332" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب حجير خزام</t>
+        </is>
+      </c>
       <c r="D332" s="4" t="inlineStr"/>
       <c r="E332" s="4" t="inlineStr"/>
       <c r="F332" s="4" t="inlineStr"/>
-      <c r="G332" s="4" t="inlineStr"/>
+      <c r="G332" s="4" t="inlineStr">
+        <is>
+          <t>قنا</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="5" t="n"/>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>المعادي</t>
+          <t>نجع حمادي</t>
         </is>
       </c>
       <c r="C333" s="4" t="inlineStr"/>
@@ -5672,7 +5545,7 @@
       <c r="A334" s="5" t="n"/>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>واحة الفيوم</t>
+          <t>دندرة</t>
         </is>
       </c>
       <c r="C334" s="4" t="inlineStr"/>
@@ -5685,7 +5558,7 @@
       <c r="A335" s="5" t="n"/>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>وادي حوف</t>
+          <t>أبيدوس</t>
         </is>
       </c>
       <c r="C335" s="4" t="inlineStr"/>
@@ -5698,7 +5571,7 @@
       <c r="A336" s="5" t="n"/>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>عين سخنة</t>
+          <t>قفطي</t>
         </is>
       </c>
       <c r="C336" s="4" t="inlineStr"/>
@@ -5711,7 +5584,7 @@
       <c r="A337" s="5" t="n"/>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>الطور</t>
+          <t>أخميم</t>
         </is>
       </c>
       <c r="C337" s="4" t="inlineStr"/>
@@ -5724,7 +5597,7 @@
       <c r="A338" s="5" t="n"/>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>الزيتون</t>
+          <t>سوهاج القديمة</t>
         </is>
       </c>
       <c r="C338" s="4" t="inlineStr"/>
@@ -5734,10 +5607,10 @@
       <c r="G338" s="4" t="inlineStr"/>
     </row>
     <row r="339">
-      <c r="A339" s="6" t="n"/>
+      <c r="A339" s="5" t="n"/>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>المقطم</t>
+          <t>النجع البحري</t>
         </is>
       </c>
       <c r="C339" s="4" t="inlineStr"/>
@@ -5747,61 +5620,69 @@
       <c r="G339" s="4" t="inlineStr"/>
     </row>
     <row r="340">
-      <c r="A340" s="2" t="inlineStr">
-        <is>
-          <t>دمياط</t>
-        </is>
-      </c>
+      <c r="A340" s="6" t="n"/>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>دمياط</t>
-        </is>
-      </c>
-      <c r="C340" s="4" t="inlineStr">
-        <is>
-          <t>مركز حلم ابني للتخاطب</t>
-        </is>
-      </c>
+          <t>الشنقي</t>
+        </is>
+      </c>
+      <c r="C340" s="4" t="inlineStr"/>
       <c r="D340" s="4" t="inlineStr"/>
       <c r="E340" s="4" t="inlineStr"/>
       <c r="F340" s="4" t="inlineStr"/>
-      <c r="G340" s="4" t="inlineStr">
-        <is>
-          <t>دمياط ودمياط الجديدة</t>
-        </is>
-      </c>
+      <c r="G340" s="4" t="inlineStr"/>
     </row>
     <row r="341">
-      <c r="A341" s="5" t="n"/>
+      <c r="A341" s="2" t="inlineStr">
+        <is>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>دمياط الجديدة</t>
-        </is>
-      </c>
-      <c r="C341" s="4" t="inlineStr"/>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
+      <c r="C341" s="4" t="inlineStr">
+        <is>
+          <t>مركز شباب كفر الشيخ للتخاطب</t>
+        </is>
+      </c>
       <c r="D341" s="4" t="inlineStr"/>
       <c r="E341" s="4" t="inlineStr"/>
       <c r="F341" s="4" t="inlineStr"/>
-      <c r="G341" s="4" t="inlineStr"/>
+      <c r="G341" s="4" t="inlineStr">
+        <is>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="5" t="n"/>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>بورت فؤاد</t>
-        </is>
-      </c>
-      <c r="C342" s="4" t="inlineStr"/>
+          <t>دسوق</t>
+        </is>
+      </c>
+      <c r="C342" s="4" t="inlineStr">
+        <is>
+          <t>مركز رعايه للتخاطب والتدخل المبكر</t>
+        </is>
+      </c>
       <c r="D342" s="4" t="inlineStr"/>
       <c r="E342" s="4" t="inlineStr"/>
       <c r="F342" s="4" t="inlineStr"/>
-      <c r="G342" s="4" t="inlineStr"/>
+      <c r="G342" s="4" t="inlineStr">
+        <is>
+          <t>شارع شهداء المغربي، خلف جمعية الشروق</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="5" t="n"/>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>كفر البطة</t>
+          <t>بلامون</t>
         </is>
       </c>
       <c r="C343" s="4" t="inlineStr"/>
@@ -5814,7 +5695,7 @@
       <c r="A344" s="5" t="n"/>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>كفر سعيد</t>
+          <t>الرياض</t>
         </is>
       </c>
       <c r="C344" s="4" t="inlineStr"/>
@@ -5827,7 +5708,7 @@
       <c r="A345" s="5" t="n"/>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>الروضة</t>
+          <t>سيدي سالم</t>
         </is>
       </c>
       <c r="C345" s="4" t="inlineStr"/>
@@ -5840,7 +5721,7 @@
       <c r="A346" s="5" t="n"/>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>الزرقا</t>
+          <t>الحامول</t>
         </is>
       </c>
       <c r="C346" s="4" t="inlineStr"/>
@@ -5853,7 +5734,7 @@
       <c r="A347" s="5" t="n"/>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>فارسكور</t>
+          <t>برج البرلس</t>
         </is>
       </c>
       <c r="C347" s="4" t="inlineStr"/>
@@ -5863,10 +5744,10 @@
       <c r="G347" s="4" t="inlineStr"/>
     </row>
     <row r="348">
-      <c r="A348" s="6" t="n"/>
+      <c r="A348" s="5" t="n"/>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>رومانية</t>
+          <t>مطوبس</t>
         </is>
       </c>
       <c r="C348" s="4" t="inlineStr"/>
@@ -5876,77 +5757,57 @@
       <c r="G348" s="4" t="inlineStr"/>
     </row>
     <row r="349">
-      <c r="A349" s="2" t="inlineStr">
-        <is>
-          <t>شمال سيناء</t>
-        </is>
-      </c>
+      <c r="A349" s="5" t="n"/>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>العريش</t>
-        </is>
-      </c>
-      <c r="C349" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب العريش للتخاطب</t>
-        </is>
-      </c>
+          <t>المحمودية</t>
+        </is>
+      </c>
+      <c r="C349" s="4" t="inlineStr"/>
       <c r="D349" s="4" t="inlineStr"/>
       <c r="E349" s="4" t="inlineStr"/>
       <c r="F349" s="4" t="inlineStr"/>
-      <c r="G349" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب العريش</t>
-        </is>
-      </c>
+      <c r="G349" s="4" t="inlineStr"/>
     </row>
     <row r="350">
-      <c r="A350" s="5" t="n"/>
+      <c r="A350" s="6" t="n"/>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>رفح</t>
-        </is>
-      </c>
-      <c r="C350" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب رفح</t>
-        </is>
-      </c>
+          <t>بيلا</t>
+        </is>
+      </c>
+      <c r="C350" s="4" t="inlineStr"/>
       <c r="D350" s="4" t="inlineStr"/>
       <c r="E350" s="4" t="inlineStr"/>
       <c r="F350" s="4" t="inlineStr"/>
-      <c r="G350" s="4" t="inlineStr">
-        <is>
-          <t>رفح</t>
-        </is>
-      </c>
+      <c r="G350" s="4" t="inlineStr"/>
     </row>
     <row r="351">
-      <c r="A351" s="5" t="n"/>
+      <c r="A351" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>الشيخ زويد</t>
-        </is>
-      </c>
-      <c r="C351" s="4" t="inlineStr">
-        <is>
-          <t>مركز تخاطب الشيخ زويد (قيد الإنشاء)</t>
-        </is>
-      </c>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="C351" s="4" t="inlineStr"/>
       <c r="D351" s="4" t="inlineStr"/>
       <c r="E351" s="4" t="inlineStr"/>
       <c r="F351" s="4" t="inlineStr"/>
-      <c r="G351" s="4" t="inlineStr">
-        <is>
-          <t>الشيخ زويد</t>
-        </is>
-      </c>
+      <c r="G351" s="4" t="inlineStr"/>
     </row>
     <row r="352">
-      <c r="A352" s="5" t="n"/>
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>بئر العبد</t>
+          <t>سيوه</t>
         </is>
       </c>
       <c r="C352" s="4" t="inlineStr"/>
@@ -5956,10 +5817,14 @@
       <c r="G352" s="4" t="inlineStr"/>
     </row>
     <row r="353">
-      <c r="A353" s="5" t="n"/>
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>القنطرة، سيناء</t>
+          <t>السلوم</t>
         </is>
       </c>
       <c r="C353" s="4" t="inlineStr"/>
@@ -5969,10 +5834,14 @@
       <c r="G353" s="4" t="inlineStr"/>
     </row>
     <row r="354">
-      <c r="A354" s="5" t="n"/>
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>نخل</t>
+          <t>سيدي براني</t>
         </is>
       </c>
       <c r="C354" s="4" t="inlineStr"/>
@@ -5982,10 +5851,14 @@
       <c r="G354" s="4" t="inlineStr"/>
     </row>
     <row r="355">
-      <c r="A355" s="5" t="n"/>
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>جديدة، حسنة</t>
+          <t>العلمين</t>
         </is>
       </c>
       <c r="C355" s="4" t="inlineStr"/>
@@ -5995,10 +5868,14 @@
       <c r="G355" s="4" t="inlineStr"/>
     </row>
     <row r="356">
-      <c r="A356" s="5" t="n"/>
+      <c r="A356" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>دهب الشرقية</t>
+          <t>مارينا</t>
         </is>
       </c>
       <c r="C356" s="4" t="inlineStr"/>
@@ -6008,10 +5885,14 @@
       <c r="G356" s="4" t="inlineStr"/>
     </row>
     <row r="357">
-      <c r="A357" s="6" t="n"/>
+      <c r="A357" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>طابا</t>
+          <t>توريدو</t>
         </is>
       </c>
       <c r="C357" s="4" t="inlineStr"/>
@@ -6023,50 +5904,46 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>قنا</t>
+          <t>مطروح</t>
         </is>
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>قنا</t>
-        </is>
-      </c>
-      <c r="C358" s="4" t="inlineStr">
-        <is>
-          <t>مركز التخاطب بمدينة العمال</t>
-        </is>
-      </c>
+          <t>جنوب سيوه</t>
+        </is>
+      </c>
+      <c r="C358" s="4" t="inlineStr"/>
       <c r="D358" s="4" t="inlineStr"/>
       <c r="E358" s="4" t="inlineStr"/>
       <c r="F358" s="4" t="inlineStr"/>
-      <c r="G358" s="4" t="inlineStr">
-        <is>
-          <t>مدينة العمال، قنا</t>
-        </is>
-      </c>
+      <c r="G358" s="4" t="inlineStr"/>
     </row>
     <row r="359">
-      <c r="A359" s="5" t="n"/>
-      <c r="B359" s="6" t="n"/>
-      <c r="C359" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب حجير خزام</t>
-        </is>
-      </c>
+      <c r="A359" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="B359" s="3" t="inlineStr">
+        <is>
+          <t>شمال سيوه</t>
+        </is>
+      </c>
+      <c r="C359" s="4" t="inlineStr"/>
       <c r="D359" s="4" t="inlineStr"/>
       <c r="E359" s="4" t="inlineStr"/>
       <c r="F359" s="4" t="inlineStr"/>
-      <c r="G359" s="4" t="inlineStr">
-        <is>
-          <t>قنا</t>
-        </is>
-      </c>
+      <c r="G359" s="4" t="inlineStr"/>
     </row>
     <row r="360">
-      <c r="A360" s="5" t="n"/>
+      <c r="A360" s="2" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>نجع حمادي</t>
+          <t>كشته</t>
         </is>
       </c>
       <c r="C360" s="4" t="inlineStr"/>
@@ -6074,417 +5951,6 @@
       <c r="E360" s="4" t="inlineStr"/>
       <c r="F360" s="4" t="inlineStr"/>
       <c r="G360" s="4" t="inlineStr"/>
-    </row>
-    <row r="361">
-      <c r="A361" s="5" t="n"/>
-      <c r="B361" s="3" t="inlineStr">
-        <is>
-          <t>دندرة</t>
-        </is>
-      </c>
-      <c r="C361" s="4" t="inlineStr"/>
-      <c r="D361" s="4" t="inlineStr"/>
-      <c r="E361" s="4" t="inlineStr"/>
-      <c r="F361" s="4" t="inlineStr"/>
-      <c r="G361" s="4" t="inlineStr"/>
-    </row>
-    <row r="362">
-      <c r="A362" s="5" t="n"/>
-      <c r="B362" s="3" t="inlineStr">
-        <is>
-          <t>أبيدوس</t>
-        </is>
-      </c>
-      <c r="C362" s="4" t="inlineStr"/>
-      <c r="D362" s="4" t="inlineStr"/>
-      <c r="E362" s="4" t="inlineStr"/>
-      <c r="F362" s="4" t="inlineStr"/>
-      <c r="G362" s="4" t="inlineStr"/>
-    </row>
-    <row r="363">
-      <c r="A363" s="5" t="n"/>
-      <c r="B363" s="3" t="inlineStr">
-        <is>
-          <t>قفطي</t>
-        </is>
-      </c>
-      <c r="C363" s="4" t="inlineStr"/>
-      <c r="D363" s="4" t="inlineStr"/>
-      <c r="E363" s="4" t="inlineStr"/>
-      <c r="F363" s="4" t="inlineStr"/>
-      <c r="G363" s="4" t="inlineStr"/>
-    </row>
-    <row r="364">
-      <c r="A364" s="5" t="n"/>
-      <c r="B364" s="3" t="inlineStr">
-        <is>
-          <t>أخميم</t>
-        </is>
-      </c>
-      <c r="C364" s="4" t="inlineStr"/>
-      <c r="D364" s="4" t="inlineStr"/>
-      <c r="E364" s="4" t="inlineStr"/>
-      <c r="F364" s="4" t="inlineStr"/>
-      <c r="G364" s="4" t="inlineStr"/>
-    </row>
-    <row r="365">
-      <c r="A365" s="5" t="n"/>
-      <c r="B365" s="3" t="inlineStr">
-        <is>
-          <t>سوهاج القديمة</t>
-        </is>
-      </c>
-      <c r="C365" s="4" t="inlineStr"/>
-      <c r="D365" s="4" t="inlineStr"/>
-      <c r="E365" s="4" t="inlineStr"/>
-      <c r="F365" s="4" t="inlineStr"/>
-      <c r="G365" s="4" t="inlineStr"/>
-    </row>
-    <row r="366">
-      <c r="A366" s="5" t="n"/>
-      <c r="B366" s="3" t="inlineStr">
-        <is>
-          <t>النجع البحري</t>
-        </is>
-      </c>
-      <c r="C366" s="4" t="inlineStr"/>
-      <c r="D366" s="4" t="inlineStr"/>
-      <c r="E366" s="4" t="inlineStr"/>
-      <c r="F366" s="4" t="inlineStr"/>
-      <c r="G366" s="4" t="inlineStr"/>
-    </row>
-    <row r="367">
-      <c r="A367" s="6" t="n"/>
-      <c r="B367" s="3" t="inlineStr">
-        <is>
-          <t>الشنقي</t>
-        </is>
-      </c>
-      <c r="C367" s="4" t="inlineStr"/>
-      <c r="D367" s="4" t="inlineStr"/>
-      <c r="E367" s="4" t="inlineStr"/>
-      <c r="F367" s="4" t="inlineStr"/>
-      <c r="G367" s="4" t="inlineStr"/>
-    </row>
-    <row r="368">
-      <c r="A368" s="2" t="inlineStr">
-        <is>
-          <t>كفر الشيخ</t>
-        </is>
-      </c>
-      <c r="B368" s="3" t="inlineStr">
-        <is>
-          <t>كفر الشيخ</t>
-        </is>
-      </c>
-      <c r="C368" s="4" t="inlineStr">
-        <is>
-          <t>مركز شباب كفر الشيخ للتخاطب</t>
-        </is>
-      </c>
-      <c r="D368" s="4" t="inlineStr"/>
-      <c r="E368" s="4" t="inlineStr"/>
-      <c r="F368" s="4" t="inlineStr"/>
-      <c r="G368" s="4" t="inlineStr">
-        <is>
-          <t>كفر الشيخ</t>
-        </is>
-      </c>
-    </row>
-    <row r="369">
-      <c r="A369" s="5" t="n"/>
-      <c r="B369" s="3" t="inlineStr">
-        <is>
-          <t>دسوق</t>
-        </is>
-      </c>
-      <c r="C369" s="4" t="inlineStr">
-        <is>
-          <t>مركز رعايه للتخاطب والتدخل المبكر</t>
-        </is>
-      </c>
-      <c r="D369" s="4" t="inlineStr"/>
-      <c r="E369" s="4" t="inlineStr"/>
-      <c r="F369" s="4" t="inlineStr"/>
-      <c r="G369" s="4" t="inlineStr">
-        <is>
-          <t>شارع شهداء المغربي، خلف جمعية الشروق</t>
-        </is>
-      </c>
-    </row>
-    <row r="370">
-      <c r="A370" s="5" t="n"/>
-      <c r="B370" s="3" t="inlineStr">
-        <is>
-          <t>بلامون</t>
-        </is>
-      </c>
-      <c r="C370" s="4" t="inlineStr"/>
-      <c r="D370" s="4" t="inlineStr"/>
-      <c r="E370" s="4" t="inlineStr"/>
-      <c r="F370" s="4" t="inlineStr"/>
-      <c r="G370" s="4" t="inlineStr"/>
-    </row>
-    <row r="371">
-      <c r="A371" s="5" t="n"/>
-      <c r="B371" s="3" t="inlineStr">
-        <is>
-          <t>الرياض</t>
-        </is>
-      </c>
-      <c r="C371" s="4" t="inlineStr"/>
-      <c r="D371" s="4" t="inlineStr"/>
-      <c r="E371" s="4" t="inlineStr"/>
-      <c r="F371" s="4" t="inlineStr"/>
-      <c r="G371" s="4" t="inlineStr"/>
-    </row>
-    <row r="372">
-      <c r="A372" s="5" t="n"/>
-      <c r="B372" s="3" t="inlineStr">
-        <is>
-          <t>سيدي سالم</t>
-        </is>
-      </c>
-      <c r="C372" s="4" t="inlineStr"/>
-      <c r="D372" s="4" t="inlineStr"/>
-      <c r="E372" s="4" t="inlineStr"/>
-      <c r="F372" s="4" t="inlineStr"/>
-      <c r="G372" s="4" t="inlineStr"/>
-    </row>
-    <row r="373">
-      <c r="A373" s="5" t="n"/>
-      <c r="B373" s="3" t="inlineStr">
-        <is>
-          <t>الحامول</t>
-        </is>
-      </c>
-      <c r="C373" s="4" t="inlineStr"/>
-      <c r="D373" s="4" t="inlineStr"/>
-      <c r="E373" s="4" t="inlineStr"/>
-      <c r="F373" s="4" t="inlineStr"/>
-      <c r="G373" s="4" t="inlineStr"/>
-    </row>
-    <row r="374">
-      <c r="A374" s="5" t="n"/>
-      <c r="B374" s="3" t="inlineStr">
-        <is>
-          <t>برج البرلس</t>
-        </is>
-      </c>
-      <c r="C374" s="4" t="inlineStr"/>
-      <c r="D374" s="4" t="inlineStr"/>
-      <c r="E374" s="4" t="inlineStr"/>
-      <c r="F374" s="4" t="inlineStr"/>
-      <c r="G374" s="4" t="inlineStr"/>
-    </row>
-    <row r="375">
-      <c r="A375" s="5" t="n"/>
-      <c r="B375" s="3" t="inlineStr">
-        <is>
-          <t>مطوبس</t>
-        </is>
-      </c>
-      <c r="C375" s="4" t="inlineStr"/>
-      <c r="D375" s="4" t="inlineStr"/>
-      <c r="E375" s="4" t="inlineStr"/>
-      <c r="F375" s="4" t="inlineStr"/>
-      <c r="G375" s="4" t="inlineStr"/>
-    </row>
-    <row r="376">
-      <c r="A376" s="5" t="n"/>
-      <c r="B376" s="3" t="inlineStr">
-        <is>
-          <t>المحمودية</t>
-        </is>
-      </c>
-      <c r="C376" s="4" t="inlineStr"/>
-      <c r="D376" s="4" t="inlineStr"/>
-      <c r="E376" s="4" t="inlineStr"/>
-      <c r="F376" s="4" t="inlineStr"/>
-      <c r="G376" s="4" t="inlineStr"/>
-    </row>
-    <row r="377">
-      <c r="A377" s="6" t="n"/>
-      <c r="B377" s="3" t="inlineStr">
-        <is>
-          <t>بيلا</t>
-        </is>
-      </c>
-      <c r="C377" s="4" t="inlineStr"/>
-      <c r="D377" s="4" t="inlineStr"/>
-      <c r="E377" s="4" t="inlineStr"/>
-      <c r="F377" s="4" t="inlineStr"/>
-      <c r="G377" s="4" t="inlineStr"/>
-    </row>
-    <row r="378">
-      <c r="A378" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B378" s="3" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="C378" s="4" t="inlineStr"/>
-      <c r="D378" s="4" t="inlineStr"/>
-      <c r="E378" s="4" t="inlineStr"/>
-      <c r="F378" s="4" t="inlineStr"/>
-      <c r="G378" s="4" t="inlineStr"/>
-    </row>
-    <row r="379">
-      <c r="A379" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B379" s="3" t="inlineStr">
-        <is>
-          <t>سيوه</t>
-        </is>
-      </c>
-      <c r="C379" s="4" t="inlineStr"/>
-      <c r="D379" s="4" t="inlineStr"/>
-      <c r="E379" s="4" t="inlineStr"/>
-      <c r="F379" s="4" t="inlineStr"/>
-      <c r="G379" s="4" t="inlineStr"/>
-    </row>
-    <row r="380">
-      <c r="A380" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B380" s="3" t="inlineStr">
-        <is>
-          <t>السلوم</t>
-        </is>
-      </c>
-      <c r="C380" s="4" t="inlineStr"/>
-      <c r="D380" s="4" t="inlineStr"/>
-      <c r="E380" s="4" t="inlineStr"/>
-      <c r="F380" s="4" t="inlineStr"/>
-      <c r="G380" s="4" t="inlineStr"/>
-    </row>
-    <row r="381">
-      <c r="A381" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B381" s="3" t="inlineStr">
-        <is>
-          <t>سيدي براني</t>
-        </is>
-      </c>
-      <c r="C381" s="4" t="inlineStr"/>
-      <c r="D381" s="4" t="inlineStr"/>
-      <c r="E381" s="4" t="inlineStr"/>
-      <c r="F381" s="4" t="inlineStr"/>
-      <c r="G381" s="4" t="inlineStr"/>
-    </row>
-    <row r="382">
-      <c r="A382" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B382" s="3" t="inlineStr">
-        <is>
-          <t>العلمين</t>
-        </is>
-      </c>
-      <c r="C382" s="4" t="inlineStr"/>
-      <c r="D382" s="4" t="inlineStr"/>
-      <c r="E382" s="4" t="inlineStr"/>
-      <c r="F382" s="4" t="inlineStr"/>
-      <c r="G382" s="4" t="inlineStr"/>
-    </row>
-    <row r="383">
-      <c r="A383" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B383" s="3" t="inlineStr">
-        <is>
-          <t>مارينا</t>
-        </is>
-      </c>
-      <c r="C383" s="4" t="inlineStr"/>
-      <c r="D383" s="4" t="inlineStr"/>
-      <c r="E383" s="4" t="inlineStr"/>
-      <c r="F383" s="4" t="inlineStr"/>
-      <c r="G383" s="4" t="inlineStr"/>
-    </row>
-    <row r="384">
-      <c r="A384" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B384" s="3" t="inlineStr">
-        <is>
-          <t>توريدو</t>
-        </is>
-      </c>
-      <c r="C384" s="4" t="inlineStr"/>
-      <c r="D384" s="4" t="inlineStr"/>
-      <c r="E384" s="4" t="inlineStr"/>
-      <c r="F384" s="4" t="inlineStr"/>
-      <c r="G384" s="4" t="inlineStr"/>
-    </row>
-    <row r="385">
-      <c r="A385" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B385" s="3" t="inlineStr">
-        <is>
-          <t>جنوب سيوه</t>
-        </is>
-      </c>
-      <c r="C385" s="4" t="inlineStr"/>
-      <c r="D385" s="4" t="inlineStr"/>
-      <c r="E385" s="4" t="inlineStr"/>
-      <c r="F385" s="4" t="inlineStr"/>
-      <c r="G385" s="4" t="inlineStr"/>
-    </row>
-    <row r="386">
-      <c r="A386" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B386" s="3" t="inlineStr">
-        <is>
-          <t>شمال سيوه</t>
-        </is>
-      </c>
-      <c r="C386" s="4" t="inlineStr"/>
-      <c r="D386" s="4" t="inlineStr"/>
-      <c r="E386" s="4" t="inlineStr"/>
-      <c r="F386" s="4" t="inlineStr"/>
-      <c r="G386" s="4" t="inlineStr"/>
-    </row>
-    <row r="387">
-      <c r="A387" s="2" t="inlineStr">
-        <is>
-          <t>مطروح</t>
-        </is>
-      </c>
-      <c r="B387" s="3" t="inlineStr">
-        <is>
-          <t>كشته</t>
-        </is>
-      </c>
-      <c r="C387" s="4" t="inlineStr"/>
-      <c r="D387" s="4" t="inlineStr"/>
-      <c r="E387" s="4" t="inlineStr"/>
-      <c r="F387" s="4" t="inlineStr"/>
-      <c r="G387" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="313">

</xml_diff>